<commit_message>
feat: complete inventory and agency reporting settings
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -2295,7 +2295,7 @@
         <v>MVP 1</v>
       </c>
       <c r="H6" t="str">
-        <v>Firme, IRMS, poslovne godine, aktivni kontekst firma/godina, banke, ugovori, kontni plan globalni + override, partneri i tabela odgovornih lica su implementirani. Unos i detalj firme podržavaju izvršnog direktora i JMBG. Dodato je kontrolisano trajno brisanje testne firme i svih njenih podataka uz tačan puni naziv, transakciju i audit; ostaju puni ekran za više uloga, fina podešavanja firme i default konta.</v>
+        <v>Firme, IRMS, poslovne godine, aktivni kontekst firma/godina, banke, ugovori, kontni plan globalni + override, partneri i tabela odgovornih lica su implementirani. Unos i detalj firme podržavaju izvršnog direktora i JMBG. Konta domaćih/ino kupaca i dobavljača podešavaju se odvojeno i služe centralnim izvještajima. Dodato je kontrolisano trajno brisanje testne firme i svih njenih podataka uz tačan puni naziv, transakciju i audit; ostaju puni ekran za više uloga i fina podešavanja firme.</v>
       </c>
     </row>
     <row r="7">
@@ -2477,7 +2477,7 @@
         <v>MVP 1/2</v>
       </c>
       <c r="H13" t="str">
-        <v>Početna centralnih Izvještaja prikazuje postojeći Bruto bilans sa filterima, nivoima zbira, štampom i drill-downom na centralnu karticu konta. Početni agencijski dashboard prikazuje tenant/permission-aware nacrte naloga, kalkulacije koje čekaju KUF i izlazne račune koji čekaju KIF. Centralni Izvještaji imaju i funkcionalne kartice konta i partnera, PDV pregled, pregled izvještaja plata, lager listu i karticu artikla preko postojećih zajedničkih prikaza; kupci, dobavljači i finansijski izvještaji ostaju za centralno povezivanje.</v>
+        <v>Početna centralnih Izvještaja prikazuje postojeći Bruto bilans sa filterima, nivoima zbira, štampom i drill-downom na centralnu karticu konta. Početni agencijski dashboard prikazuje tenant/permission-aware nacrte naloga, kalkulacije koje čekaju KUF i izlazne račune koji čekaju KIF. Centralni Izvještaji imaju funkcionalne kartice konta/partnera, Kupce i Dobavljače sa domaćim/ino kontima, PDV, plate, lager listu i karticu artikla; finansijski izvještaji ostaju za centralno povezivanje.</v>
       </c>
     </row>
     <row r="301">
@@ -2697,7 +2697,7 @@
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z375"/>
+  <dimension ref="A1:AA376"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3594,7 +3594,7 @@
         <v>Podrazumijevana konta</v>
       </c>
       <c r="D27" t="str">
-        <v>Firma podešava default konta za kupce, dobavljače, PDV, banku, blagajnu itd.</v>
+        <v>Firma podešava konta za domaće i ino kupce i dobavljače koja određuju prikaz zbirnih partnerskih izvještaja.</v>
       </c>
       <c r="E27" t="str">
         <v>Vrlo visok</v>
@@ -3618,7 +3618,7 @@
         <v>F-021,F-022</v>
       </c>
       <c r="L27" t="str">
-        <v>Podrazumijevana konta firme implementirana za kupce, dobavljace, PDV, banku, blagajnu, prihod, trosak, robu i plate.</v>
+        <v>Admin-only /agencija/podesavanja/podrazumijevana-konta čuva četiri konta samo za izvještaje Kupci i Dobavljači; ne koriste se u šemama automatskog knjiženja.</v>
       </c>
     </row>
     <row r="28">
@@ -3656,7 +3656,10 @@
         <v>F-014,F-021</v>
       </c>
       <c r="L28" t="str">
-        <v>Sistemske vrste naloga seedovane migracijom; ekran /agencija/nalozi/vrste prikazuje vrste i admin moze dodati agencijsku ili firmi specificnu vrstu.</v>
+        <v>Sistemske vrste naloga seedovane migracijom; zajednicki ekran je dostupan kroz /agencija/nalozi/vrste i /agencija/podesavanja/vrste-naloga</v>
+      </c>
+      <c r="M28" t="str">
+        <v xml:space="preserve"> a admin moze dodati agencijsku ili firmi specificnu vrstu.</v>
       </c>
     </row>
     <row r="29">
@@ -4138,7 +4141,7 @@
         <v>Da</v>
       </c>
       <c r="H41" t="str">
-        <v>Partner je obavezan za analiticka konta; implementirana analiticka kartica sa filterima konto/partner/period i zbirna stranica Kupci / dobavljaci sa otvorenim saldom po partneru.</v>
+        <v>Partner je obavezan za analiticka konta; kartice i centralni izvještaji Kupci/Dobavljači imaju tabove domaći/ino/svi te filtere partnera i perioda.</v>
       </c>
       <c r="I41" t="str">
         <v>Djelimicno</v>
@@ -4150,7 +4153,7 @@
         <v>F-036,F-027</v>
       </c>
       <c r="L41" t="str">
-        <v>Kartica partnera vodi na nalog; Kupci / dobavljaci vode na karticu partnera za klasu 2 ili 4.</v>
+        <v>Centralni izvještaji koriste četiri firm-specific konta iz Podešavanja i samo POSTED stavke; red vodi na karticu partnera. Ostaju štampa/export.</v>
       </c>
     </row>
     <row r="42">
@@ -5006,13 +5009,13 @@
         <v>Vrlo visok</v>
       </c>
       <c r="F322" t="str">
-        <v>Zaključeno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G322" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="H322" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="I322" t="str">
         <v>Da</v>
@@ -5024,7 +5027,7 @@
         <v>F-042</v>
       </c>
       <c r="L322" t="str">
-        <v>Osnovni izvještaji robnog.</v>
+        <v>Implementirani lager lista, kartica artikla i vrijednost zaliha sa presjecima po magacinu i grupi, filterima i vezom na karticu artikla.</v>
       </c>
     </row>
     <row r="323">
@@ -7041,9 +7044,47 @@
         <v>Zaglavlje za pregled; view/export scope i audit; XSD test. Portal QA ostaje otvoren.</v>
       </c>
     </row>
+    <row r="376">
+      <c r="A376" t="str">
+        <v>F-114</v>
+      </c>
+      <c r="B376" t="str">
+        <v>Korisnici, agencije i prava</v>
+      </c>
+      <c r="C376" t="str">
+        <v>Centralno slanje emaila i Reply-To agencije</v>
+      </c>
+      <c r="D376" t="str">
+        <v>Sistem šalje sa admin@summasummarum.me, dok administrator agencije podešava adresu na koju prima odgovore.</v>
+      </c>
+      <c r="E376" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F376" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G376" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H376" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I376" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J376" t="str">
+        <v>Djelimično</v>
+      </c>
+      <c r="K376" t="str">
+        <v>M-001</v>
+      </c>
+      <c r="L376" t="str">
+        <v>Admin-only podešavanje po agenciji, backend validacija, audit i probno slanje. Pozivnice koje kreira admin agencije koriste sačuvani Reply-To; produkcijski SMTP nalog mora biti ovlašćen za centralnu From adresu.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z375"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA376"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -11148,7 +11189,7 @@
 
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z342"/>
+  <dimension ref="A1:Z343"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -11188,68 +11229,68 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>UI-001</v>
+        <v>E-054</v>
       </c>
       <c r="B5" t="str">
         <v>Korisnici, agencije i prava</v>
       </c>
       <c r="C5" t="str">
-        <v>Super admin — Agencije</v>
+        <v>Email podešavanja</v>
       </c>
       <c r="D5" t="str">
-        <v>Pregled agencija, pretplata, statusa aktivacije i isteka.</v>
+        <v>Admin agencije vidi fiksnog centralnog pošiljaoca, podešava Reply-To adresu svoje agencije i može poslati probnu poruku.</v>
       </c>
       <c r="E5" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F5" t="str">
-        <v>Implementirano djelimicno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G5" t="str">
-        <v>F-001,F-003,F-004</v>
+        <v>F-114</v>
       </c>
       <c r="H5" t="str">
-        <v>Pregled agencija postoji; pretplate nisu kompletno UI zaokruzene.</v>
+        <v>/agencija/podesavanja/email</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>UI-002</v>
+        <v>UI-001</v>
       </c>
       <c r="B6" t="str">
         <v>Korisnici, agencije i prava</v>
       </c>
       <c r="C6" t="str">
-        <v>Agencijski admin — Radnici</v>
+        <v>Super admin — Agencije</v>
       </c>
       <c r="D6" t="str">
-        <v>Kreiranje radnika i dodjela prava.</v>
+        <v>Pregled agencija, pretplata, statusa aktivacije i isteka.</v>
       </c>
       <c r="E6" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F6" t="str">
-        <v>Implementirano</v>
+        <v>Implementirano djelimicno</v>
       </c>
       <c r="G6" t="str">
-        <v>F-005,F-008</v>
+        <v>F-001,F-003,F-004</v>
       </c>
       <c r="H6" t="str">
-        <v>Kreiranje radnika i dodjela prava postoje.</v>
+        <v>Pregled agencija postoji; pretplate nisu kompletno UI zaokruzene.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>UI-003</v>
+        <v>UI-002</v>
       </c>
       <c r="B7" t="str">
         <v>Korisnici, agencije i prava</v>
       </c>
       <c r="C7" t="str">
-        <v>Agencijski admin — Prava pristupa</v>
+        <v>Agencijski admin — Radnici</v>
       </c>
       <c r="D7" t="str">
-        <v>Matrica prava po firmama, modulima i akcijama.</v>
+        <v>Kreiranje radnika i dodjela prava.</v>
       </c>
       <c r="E7" t="str">
         <v>Vrlo visok</v>
@@ -11258,76 +11299,76 @@
         <v>Implementirano</v>
       </c>
       <c r="G7" t="str">
-        <v>F-007,F-008</v>
+        <v>F-005,F-008</v>
       </c>
       <c r="H7" t="str">
-        <v>Matrica ima pregled, unos, izmjenu, brisanje, knjiženje, storniranje, izvoz i administraciju; pravo pregleda određuje prikaz glavnog menija po aktivnoj firmi.</v>
+        <v>Kreiranje radnika i dodjela prava postoje.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>UI-004</v>
+        <v>UI-003</v>
       </c>
       <c r="B8" t="str">
         <v>Korisnici, agencije i prava</v>
       </c>
       <c r="C8" t="str">
-        <v>Učinak radnika</v>
+        <v>Agencijski admin — Prava pristupa</v>
       </c>
       <c r="D8" t="str">
-        <v>Dnevni/nedjeljni/mjesečni pregled aktivnosti po radniku.</v>
+        <v>Matrica prava po firmama, modulima i akcijama.</v>
       </c>
       <c r="E8" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F8" t="str">
-        <v>U izradi</v>
+        <v>Implementirano</v>
       </c>
       <c r="G8" t="str">
-        <v>F-009,F-010</v>
+        <v>F-007,F-008</v>
       </c>
       <c r="H8" t="str">
-        <v>Postoji audit/aktivnost osnova; puni ekran ucinka jos nije implementiran.</v>
+        <v>Matrica ima pregled, unos, izmjenu, brisanje, knjiženje, storniranje, izvoz i administraciju; pravo pregleda određuje prikaz glavnog menija po aktivnoj firmi.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>UI-005</v>
+        <v>UI-004</v>
       </c>
       <c r="B9" t="str">
-        <v>Firme i kontni plan</v>
+        <v>Korisnici, agencije i prava</v>
       </c>
       <c r="C9" t="str">
-        <v>Lista firmi</v>
+        <v>Učinak radnika</v>
       </c>
       <c r="D9" t="str">
-        <v>Naziv, PIB, tip, PDV status, godina, glavni radnik, status.</v>
+        <v>Dnevni/nedjeljni/mjesečni pregled aktivnosti po radniku.</v>
       </c>
       <c r="E9" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F9" t="str">
-        <v>Implementirano</v>
+        <v>U izradi</v>
       </c>
       <c r="G9" t="str">
-        <v>F-012,F-014,F-019</v>
+        <v>F-009,F-010</v>
       </c>
       <c r="H9" t="str">
-        <v>Lista firmi postoji kao /agencija/firme.</v>
+        <v>Postoji audit/aktivnost osnova; puni ekran ucinka jos nije implementiran.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>UI-006</v>
+        <v>UI-005</v>
       </c>
       <c r="B10" t="str">
         <v>Firme i kontni plan</v>
       </c>
       <c r="C10" t="str">
-        <v>Dodavanje firme</v>
+        <v>Lista firmi</v>
       </c>
       <c r="D10" t="str">
-        <v>Unos PIB-a, IRMS pretraga, provjera podataka i snimanje.</v>
+        <v>Naziv, PIB, tip, PDV status, godina, glavni radnik, status.</v>
       </c>
       <c r="E10" t="str">
         <v>Vrlo visok</v>
@@ -11336,76 +11377,76 @@
         <v>Implementirano</v>
       </c>
       <c r="G10" t="str">
-        <v>F-012,F-013</v>
+        <v>F-012,F-014,F-019</v>
       </c>
       <c r="H10" t="str">
-        <v>Dodavanje firme sa IRMS pretragom postoji kao /agencija/firme/nova.</v>
+        <v>Lista firmi postoji kao /agencija/firme.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>UI-007</v>
+        <v>UI-006</v>
       </c>
       <c r="B11" t="str">
         <v>Firme i kontni plan</v>
       </c>
       <c r="C11" t="str">
-        <v>Profil firme</v>
+        <v>Dodavanje firme</v>
       </c>
       <c r="D11" t="str">
-        <v>Tabovi: podaci, lica, banke, godine, podešavanja, radnici, klijenti, ugovor, kontni plan.</v>
+        <v>Unos PIB-a, IRMS pretraga, provjera podataka i snimanje.</v>
       </c>
       <c r="E11" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F11" t="str">
-        <v>Implementirano djelimicno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G11" t="str">
-        <v>F-012-F-023</v>
+        <v>F-012,F-013</v>
       </c>
       <c r="H11" t="str">
-        <v>Detalj firme prikazuje osnovne podatke, primarnog izvršnog direktora i JMBG, godine, bankovne račune, ugovor/cijenu i korisnike. Dodat je odvojeni opasni odjeljak za trajno brisanje firme uz obavezni unos punog naziva; ostaje poseban pregled više odgovornih/kontakt lica i fina podešavanja.</v>
+        <v>Dodavanje firme sa IRMS pretragom postoji kao /agencija/firme/nova.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>UI-008</v>
+        <v>UI-007</v>
       </c>
       <c r="B12" t="str">
         <v>Firme i kontni plan</v>
       </c>
       <c r="C12" t="str">
-        <v>Poslovne godine</v>
+        <v>Profil firme</v>
       </c>
       <c r="D12" t="str">
-        <v>Otvaranje, zaključavanje, otključavanje i arhiva godina.</v>
+        <v>Tabovi: podaci, lica, banke, godine, podešavanja, radnici, klijenti, ugovor, kontni plan.</v>
       </c>
       <c r="E12" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F12" t="str">
-        <v>Implementirano</v>
+        <v>Implementirano djelimicno</v>
       </c>
       <c r="G12" t="str">
-        <v>F-014,F-015</v>
+        <v>F-012-F-023</v>
       </c>
       <c r="H12" t="str">
-        <v>Centralna stranica poslovnih godina postoji.</v>
+        <v>Detalj firme prikazuje osnovne podatke, primarnog izvršnog direktora i JMBG, godine, bankovne račune, ugovor/cijenu i korisnike. Dodat je odvojeni opasni odjeljak za trajno brisanje firme uz obavezni unos punog naziva; ostaje poseban pregled više odgovornih/kontakt lica i fina podešavanja.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>UI-009</v>
+        <v>UI-008</v>
       </c>
       <c r="B13" t="str">
         <v>Firme i kontni plan</v>
       </c>
       <c r="C13" t="str">
-        <v>Kontni plan firme</v>
+        <v>Poslovne godine</v>
       </c>
       <c r="D13" t="str">
-        <v>Kombinovani prikaz osnovnog plana i firmi specifičnih izmjena.</v>
+        <v>Otvaranje, zaključavanje, otključavanje i arhiva godina.</v>
       </c>
       <c r="E13" t="str">
         <v>Vrlo visok</v>
@@ -11414,24 +11455,24 @@
         <v>Implementirano</v>
       </c>
       <c r="G13" t="str">
-        <v>F-021,F-022,F-023</v>
+        <v>F-014,F-015</v>
       </c>
       <c r="H13" t="str">
-        <v>Postoje dva ekrana: globalni osnovni kontni plan u podesavanjima i kontni plan firme za specificne izmjene i default konta. Kontni plan firme ima pretragu po sifri/nazivu direktno iznad tabele.</v>
+        <v>Centralna stranica poslovnih godina postoji.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>UI-010</v>
+        <v>UI-009</v>
       </c>
       <c r="B14" t="str">
-        <v>Nalozi za knjiženje</v>
+        <v>Firme i kontni plan</v>
       </c>
       <c r="C14" t="str">
-        <v>Lista naloga</v>
+        <v>Kontni plan firme</v>
       </c>
       <c r="D14" t="str">
-        <v>Pregled naloga po firmi, godini, vrsti, broju, statusu, korisniku.</v>
+        <v>Kombinovani prikaz osnovnog plana i firmi specifičnih izmjena.</v>
       </c>
       <c r="E14" t="str">
         <v>Vrlo visok</v>
@@ -11440,102 +11481,102 @@
         <v>Implementirano</v>
       </c>
       <c r="G14" t="str">
-        <v>F-024-F-031</v>
+        <v>F-021,F-022,F-023</v>
       </c>
       <c r="H14" t="str">
-        <v>Lista naloga po aktivnoj firmi/godini postoji na /agencija/nalozi, sa filterom statusa.</v>
+        <v>Globalni plan je u Podešavanjima, a kontni plan firme služi samo specifičnim izmjenama. Četiri konta za izvještaje partnera premještena su na /agencija/podesavanja/podrazumijevana-konta.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>UI-011</v>
+        <v>UI-010</v>
       </c>
       <c r="B15" t="str">
         <v>Nalozi za knjiženje</v>
       </c>
       <c r="C15" t="str">
-        <v>Unos naloga</v>
+        <v>Lista naloga</v>
       </c>
       <c r="D15" t="str">
-        <v>Zaglavlje + tabelarni unos stavki.</v>
+        <v>Pregled naloga po firmi, godini, vrsti, broju, statusu, korisniku.</v>
       </c>
       <c r="E15" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F15" t="str">
-        <v>Implementirano djelimicno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G15" t="str">
-        <v>F-026,F-027,F-029</v>
+        <v>F-024-F-031</v>
       </c>
       <c r="H15" t="str">
-        <v>Unos novog naloga postoji na /agencija/nalozi/novi; izmjena nacrta ostaje za naredni korak.</v>
+        <v>Lista naloga po aktivnoj firmi/godini postoji na /agencija/nalozi, sa filterom statusa.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>UI-012</v>
+        <v>UI-011</v>
       </c>
       <c r="B16" t="str">
         <v>Nalozi za knjiženje</v>
       </c>
       <c r="C16" t="str">
-        <v>Nacrti naloga</v>
+        <v>Unos naloga</v>
       </c>
       <c r="D16" t="str">
-        <v>Lista nacrta koji nijesu proknjiženi.</v>
+        <v>Zaglavlje + tabelarni unos stavki.</v>
       </c>
       <c r="E16" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F16" t="str">
-        <v>Implementirano</v>
+        <v>Implementirano djelimicno</v>
       </c>
       <c r="G16" t="str">
-        <v>F-028</v>
+        <v>F-026,F-027,F-029</v>
       </c>
       <c r="H16" t="str">
-        <v>Nacrti su dostupni preko /agencija/nalozi/nacrti odnosno status filtera.</v>
+        <v>Unos novog naloga postoji na /agencija/nalozi/novi; izmjena nacrta ostaje za naredni korak.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>UI-013</v>
+        <v>UI-012</v>
       </c>
       <c r="B17" t="str">
         <v>Nalozi za knjiženje</v>
       </c>
       <c r="C17" t="str">
-        <v>Početno stanje</v>
+        <v>Nacrti naloga</v>
       </c>
       <c r="D17" t="str">
-        <v>Pregled/generisanje/proknjižavanje početnog stanja.</v>
+        <v>Lista nacrta koji nijesu proknjiženi.</v>
       </c>
       <c r="E17" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F17" t="str">
         <v>Implementirano</v>
       </c>
       <c r="G17" t="str">
-        <v>F-034,F-035</v>
+        <v>F-028</v>
       </c>
       <c r="H17" t="str">
-        <v>Ekran prikazuje izvor iz prethodne godine, kontrole i pregled stavki; kreira DRAFT nalog koji se proknjižava kroz standardni detalj naloga.</v>
+        <v>Nacrti su dostupni preko /agencija/nalozi/nacrti odnosno status filtera.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>UI-014</v>
+        <v>UI-013</v>
       </c>
       <c r="B18" t="str">
         <v>Nalozi za knjiženje</v>
       </c>
       <c r="C18" t="str">
-        <v>Partneri</v>
+        <v>Početno stanje</v>
       </c>
       <c r="D18" t="str">
-        <v>Lista partnera, kupac/dobavljač oznake, PIB, kontakt podaci.</v>
+        <v>Pregled/generisanje/proknjižavanje početnog stanja.</v>
       </c>
       <c r="E18" t="str">
         <v>Vrlo visok</v>
@@ -11544,24 +11585,24 @@
         <v>Implementirano</v>
       </c>
       <c r="G18" t="str">
-        <v>F-036</v>
+        <v>F-034,F-035</v>
       </c>
       <c r="H18" t="str">
-        <v>Agencijski ekran za dodatne partnere i admin ekran za globalne partnere podrzavaju unos, IRMS pretragu i izmjenu.</v>
+        <v>Ekran prikazuje izvor iz prethodne godine, kontrole i pregled stavki; kreira DRAFT nalog koji se proknjižava kroz standardni detalj naloga.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>UI-015</v>
+        <v>UI-014</v>
       </c>
       <c r="B19" t="str">
         <v>Nalozi za knjiženje</v>
       </c>
       <c r="C19" t="str">
-        <v>Bruto bilans</v>
+        <v>Partneri</v>
       </c>
       <c r="D19" t="str">
-        <v>PS, promet, ukupno, saldo; filter po firmi, godini, poslovnoj jedinici.</v>
+        <v>Lista partnera, kupac/dobavljač oznake, PIB, kontakt podaci.</v>
       </c>
       <c r="E19" t="str">
         <v>Vrlo visok</v>
@@ -11570,76 +11611,76 @@
         <v>Implementirano</v>
       </c>
       <c r="G19" t="str">
-        <v>F-038</v>
+        <v>F-036</v>
       </c>
       <c r="H19" t="str">
-        <v>Dostupan u Nalozima i centralnim Izvještajima preko iste serverske komponente; ima filtere, nivoe zbira, drill-down na karticu konta i A4 štampu.</v>
+        <v>Agencijski ekran za dodatne partnere i admin ekran za globalne partnere podrzavaju unos, IRMS pretragu i izmjenu.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>UI-016</v>
+        <v>UI-015</v>
       </c>
       <c r="B20" t="str">
         <v>Nalozi za knjiženje</v>
       </c>
       <c r="C20" t="str">
-        <v>Kartica partnera</v>
+        <v>Bruto bilans</v>
       </c>
       <c r="D20" t="str">
-        <v>Detaljna kartica i zbirni saldo kupaca/dobavljača.</v>
+        <v>PS, promet, ukupno, saldo; filter po firmi, godini, poslovnoj jedinici.</v>
       </c>
       <c r="E20" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F20" t="str">
-        <v>Implementirano djelimicno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G20" t="str">
-        <v>F-037</v>
+        <v>F-038</v>
       </c>
       <c r="H20" t="str">
-        <v>Analiticka kartica je implementirana u /agencija/nalozi/analiticke-kartice; zbir kupaca/dobavljaca po partneru u /agencija/nalozi/kupci-dobavljaci. Ostaju stampa/export.</v>
+        <v>Dostupan u Nalozima i centralnim Izvještajima preko iste serverske komponente; ima filtere, nivoe zbira, drill-down na karticu konta i A4 štampu.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>UI-017</v>
+        <v>UI-016</v>
       </c>
       <c r="B21" t="str">
-        <v>Izvodi</v>
+        <v>Nalozi za knjiženje</v>
       </c>
       <c r="C21" t="str">
-        <v>Uvoz izvoda</v>
+        <v>Kartica partnera</v>
       </c>
       <c r="D21" t="str">
-        <v>Upload PDF/HTML/XML izvoda za aktivnu firmu/godinu i bankovni račun firme.</v>
+        <v>Detaljna kartica i zbirni saldo kupaca/dobavljača.</v>
       </c>
       <c r="E21" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F21" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Implementirano djelimicno</v>
       </c>
       <c r="G21" t="str">
-        <v>F-076</v>
+        <v>F-037</v>
       </c>
       <c r="H21" t="str">
-        <v>Na /agencija/izvodi postoji izbor bankovnog računa, konta banke, PDF/HTML/XML fajla i paste teksta; NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF rade, ostale banke ostaju otvorene.</v>
+        <v>Analitička kartica postoji u Nalozima i centralnim Izvještajima. /agencija/izvjestaji/kupci i /dobavljaci koriste podešena domaća i ino konta, tabove domaći/ino/svi, filter partnera i perioda, POSTED promet i link na karticu. Ostaju štampa/export.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>UI-018</v>
+        <v>UI-017</v>
       </c>
       <c r="B22" t="str">
         <v>Izvodi</v>
       </c>
       <c r="C22" t="str">
-        <v>Preview parsiranja</v>
+        <v>Uvoz izvoda</v>
       </c>
       <c r="D22" t="str">
-        <v>Pregled zaglavlja, parsiranih stavki, grešaka i kontrole početnog/krajnjeg stanja.</v>
+        <v>Upload PDF/HTML/XML izvoda za aktivnu firmu/godinu i bankovni račun firme.</v>
       </c>
       <c r="E22" t="str">
         <v>Vrlo visok</v>
@@ -11648,24 +11689,24 @@
         <v>Djelimično implementirano</v>
       </c>
       <c r="G22" t="str">
-        <v>F-078</v>
+        <v>F-076</v>
       </c>
       <c r="H22" t="str">
-        <v>Postoji tab Stavke izvoda sa kontrolom stanja; edit parsiranih iznosa/datuma ostaje otvoren.</v>
+        <v>Na /agencija/izvodi postoji izbor bankovnog računa, konta banke, PDF/HTML/XML fajla i paste teksta; NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF rade, ostale banke ostaju otvorene.</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>UI-019</v>
+        <v>UI-018</v>
       </c>
       <c r="B23" t="str">
         <v>Izvodi</v>
       </c>
       <c r="C23" t="str">
-        <v>Povezivanje i obrada stavki</v>
+        <v>Preview parsiranja</v>
       </c>
       <c r="D23" t="str">
-        <v>Tabela stavki sa komitentom, fakturom, predlogom knjiženja, confidence score-om i akcijama.</v>
+        <v>Pregled zaglavlja, parsiranih stavki, grešaka i kontrole početnog/krajnjeg stanja.</v>
       </c>
       <c r="E23" t="str">
         <v>Vrlo visok</v>
@@ -11674,24 +11715,24 @@
         <v>Djelimično implementirano</v>
       </c>
       <c r="G23" t="str">
-        <v>F-079,F-080,F-081,F-083</v>
+        <v>F-078</v>
       </c>
       <c r="H23" t="str">
-        <v>Postoji izbor partnera i konta, ignorisanje stavki i posebna stranica Obrada stavki; fakture, učenje računa i trajna pravila ostaju otvoreni.</v>
+        <v>Postoji tab Stavke izvoda sa kontrolom stanja; edit parsiranih iznosa/datuma ostaje otvoren.</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>UI-020</v>
+        <v>UI-019</v>
       </c>
       <c r="B24" t="str">
         <v>Izvodi</v>
       </c>
       <c r="C24" t="str">
-        <v>Preview naloga izvoda</v>
+        <v>Povezivanje i obrada stavki</v>
       </c>
       <c r="D24" t="str">
-        <v>Prije knjiženja prikazuje stavke naloga duguje/potražuje, konto, partner, opis i iznos.</v>
+        <v>Tabela stavki sa komitentom, fakturom, predlogom knjiženja, confidence score-om i akcijama.</v>
       </c>
       <c r="E24" t="str">
         <v>Vrlo visok</v>
@@ -11700,27 +11741,27 @@
         <v>Djelimično implementirano</v>
       </c>
       <c r="G24" t="str">
-        <v>F-084</v>
+        <v>F-079,F-080,F-081,F-083</v>
       </c>
       <c r="H24" t="str">
-        <v>Postoji tab Predlog naloga; banka se knjiži zbirno po ukupnom prilivu/odlivu, a stavke idu na kontra konta; knjiženje READY izvoda u IZV nalog postoji.</v>
+        <v>Postoji izbor partnera i konta, ignorisanje stavki i posebna stranica Obrada stavki; fakture, učenje računa i trajna pravila ostaju otvoreni.</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>UI-021</v>
+        <v>UI-020</v>
       </c>
       <c r="B25" t="str">
         <v>Izvodi</v>
       </c>
       <c r="C25" t="str">
-        <v>Kartica banke</v>
+        <v>Preview naloga izvoda</v>
       </c>
       <c r="D25" t="str">
-        <v>Pregled prometa bankovnog računa iz proknjiženih izvoda/naloga.</v>
+        <v>Prije knjiženja prikazuje stavke naloga duguje/potražuje, konto, partner, opis i iznos.</v>
       </c>
       <c r="E25" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F25" t="str">
         <v>Djelimično implementirano</v>
@@ -11729,50 +11770,50 @@
         <v>F-084</v>
       </c>
       <c r="H25" t="str">
+        <v>Postoji tab Predlog naloga; banka se knjiži zbirno po ukupnom prilivu/odlivu, a stavke idu na kontra konta; knjiženje READY izvoda u IZV nalog postoji.</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>UI-021</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Kartica banke</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Pregled prometa bankovnog računa iz proknjiženih izvoda/naloga.</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="G26" t="str">
+        <v>F-084</v>
+      </c>
+      <c r="H26" t="str">
         <v>Dodata stranica Kartica banke sa filterom bankovnog računa i pregledom uvezenih izvoda, priliva, odliva i naloga.</v>
-      </c>
-    </row>
-    <row r="306">
-      <c r="A306" t="str">
-        <v>E-017</v>
-      </c>
-      <c r="B306" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="C306" t="str">
-        <v>Artikli</v>
-      </c>
-      <c r="D306" t="str">
-        <v>Lista i unos artikala/usluga.</v>
-      </c>
-      <c r="E306" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F306" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="G306" t="str">
-        <v>F-039</v>
-      </c>
-      <c r="H306" t="str">
-        <v>/agencija/robno/artikli; pretraga/filteri, unos sa opcionim početnim VP/MP cijenama, izmjena, cijene i aktivacija/deaktivacija.</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="str">
-        <v>E-018</v>
+        <v>E-017</v>
       </c>
       <c r="B307" t="str">
         <v>Robno knjigovodstvo</v>
       </c>
       <c r="C307" t="str">
-        <v>Grupe artikala</v>
+        <v>Artikli</v>
       </c>
       <c r="D307" t="str">
-        <v>Šifarnik grupa artikala.</v>
+        <v>Lista i unos artikala/usluga.</v>
       </c>
       <c r="E307" t="str">
-        <v>Srednji</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F307" t="str">
         <v>Implementirano</v>
@@ -11781,125 +11822,125 @@
         <v>F-039</v>
       </c>
       <c r="H307" t="str">
-        <v>/agencija/robno/grupe; unos, izmjena, pretraga i aktivacija/deaktivacija.</v>
+        <v>/agencija/robno/artikli; pretraga/filteri, unos sa opcionim početnim VP/MP cijenama, izmjena, cijene i aktivacija/deaktivacija.</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="str">
-        <v>E-019</v>
+        <v>E-018</v>
       </c>
       <c r="B308" t="str">
         <v>Robno knjigovodstvo</v>
       </c>
       <c r="C308" t="str">
-        <v>Cijene artikala</v>
+        <v>Grupe artikala</v>
       </c>
       <c r="D308" t="str">
-        <v>Upravljanje više cijena artikla.</v>
+        <v>Šifarnik grupa artikala.</v>
       </c>
       <c r="E308" t="str">
-        <v>Visok</v>
+        <v>Srednji</v>
       </c>
       <c r="F308" t="str">
         <v>Implementirano</v>
       </c>
       <c r="G308" t="str">
-        <v>F-040</v>
+        <v>F-039</v>
       </c>
       <c r="H308" t="str">
-        <v>/agencija/robno/cijene; izbor artikla, veleprodajna/maloprodajna cijena, PDV, period važenja i istorija.</v>
+        <v>/agencija/robno/grupe; unos, izmjena, pretraga i aktivacija/deaktivacija.</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="str">
-        <v>E-020</v>
+        <v>E-019</v>
       </c>
       <c r="B309" t="str">
         <v>Robno knjigovodstvo</v>
       </c>
       <c r="C309" t="str">
-        <v>Magacini</v>
+        <v>Cijene artikala</v>
       </c>
       <c r="D309" t="str">
-        <v>Lista i podešavanje magacina.</v>
+        <v>Upravljanje više cijena artikla.</v>
       </c>
       <c r="E309" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F309" t="str">
         <v>Implementirano</v>
       </c>
       <c r="G309" t="str">
-        <v>F-041</v>
+        <v>F-040</v>
       </c>
       <c r="H309" t="str">
-        <v>/agencija/robno/magacini; unos, izmjena, status i negativan lager opciono po magacinu.</v>
+        <v>/agencija/robno/cijene; izbor artikla, veleprodajna/maloprodajna cijena, PDV, period važenja i istorija.</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="str">
-        <v>E-021</v>
+        <v>E-020</v>
       </c>
       <c r="B310" t="str">
         <v>Robno knjigovodstvo</v>
       </c>
       <c r="C310" t="str">
-        <v>Lager lista</v>
+        <v>Magacini</v>
       </c>
       <c r="D310" t="str">
-        <v>Stanje robe po magacinu.</v>
+        <v>Lista i podešavanje magacina.</v>
       </c>
       <c r="E310" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F310" t="str">
-        <v>Navigacija pripremljena</v>
+        <v>Implementirano</v>
       </c>
       <c r="G310" t="str">
-        <v>F-042,F-060</v>
+        <v>F-041</v>
       </c>
       <c r="H310" t="str">
-        <v>/agencija/robno/lager; poslovna logika nije implementirana.</v>
+        <v>/agencija/robno/magacini; unos, izmjena, status i negativan lager opciono po magacinu.</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="str">
-        <v>E-022</v>
+        <v>E-021</v>
       </c>
       <c r="B311" t="str">
         <v>Robno knjigovodstvo</v>
       </c>
       <c r="C311" t="str">
-        <v>Kartica artikla</v>
+        <v>Lager lista</v>
       </c>
       <c r="D311" t="str">
-        <v>Ulazi, izlazi i saldo artikla.</v>
+        <v>Stanje robe po magacinu.</v>
       </c>
       <c r="E311" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F311" t="str">
-        <v>Navigacija pripremljena</v>
+        <v>Implementirano</v>
       </c>
       <c r="G311" t="str">
-        <v>F-060</v>
+        <v>F-042,F-060</v>
       </c>
       <c r="H311" t="str">
-        <v>/agencija/robno/kartica-artikla; poslovna logika nije implementirana.</v>
+        <v>/agencija/robno/lager; filteri po magacinu, grupi, artiklu i znaku stanja sa količinama i nabavnom/maloprodajnom vrijednošću, RUC-om i PDV-om.</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="str">
-        <v>E-023</v>
+        <v>E-022</v>
       </c>
       <c r="B312" t="str">
         <v>Robno knjigovodstvo</v>
       </c>
       <c r="C312" t="str">
-        <v>Kalkulacije</v>
+        <v>Kartica artikla</v>
       </c>
       <c r="D312" t="str">
-        <v>Unos i završavanje kalkulacija.</v>
+        <v>Ulazi, izlazi i saldo artikla.</v>
       </c>
       <c r="E312" t="str">
         <v>Vrlo visok</v>
@@ -11908,50 +11949,50 @@
         <v>Implementirano</v>
       </c>
       <c r="G312" t="str">
-        <v>F-045</v>
+        <v>F-060</v>
       </c>
       <c r="H312" t="str">
-        <v>/agencija/robno/kalkulacije i detalj: MAPR link i pregled stavki preko pune širine, grupno povezivanje nepoznatih MAPR jedinica mjere, povezivanje postojećih ili priprema novih artikala, zaglavlje, obavezna prodajna cijena, kompaktna tabelarna izmjena, zavisni troškovi, zbirovi, završavanje u nalog/lager sa statusom čeka KUF i A4 landscape štampa. KUF knjiga ima pregled i grupno preuzimanje završenih kalkulacija.</v>
+        <v>/agencija/robno/kartica-artikla; početno stanje, prometi, tekuća količina i vrijednost uz filter magacina i perioda i linkove na izvorne dokumente.</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="str">
-        <v>E-024</v>
+        <v>E-023</v>
       </c>
       <c r="B313" t="str">
         <v>Robno knjigovodstvo</v>
       </c>
       <c r="C313" t="str">
-        <v>Uvozna kalkulacija</v>
+        <v>Kalkulacije</v>
       </c>
       <c r="D313" t="str">
-        <v>Kalkulacija sa carinskom deklaracijom.</v>
+        <v>Unos i završavanje kalkulacija.</v>
       </c>
       <c r="E313" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F313" t="str">
-        <v>Navigacija pripremljena</v>
+        <v>Implementirano</v>
       </c>
       <c r="G313" t="str">
-        <v>F-051</v>
+        <v>F-045</v>
       </c>
       <c r="H313" t="str">
-        <v>/agencija/robno/uvozne-kalkulacije; poslovna logika nije implementirana.</v>
+        <v>/agencija/robno/kalkulacije i detalj: MAPR link i pregled stavki preko pune širine, grupno povezivanje nepoznatih MAPR jedinica mjere, povezivanje postojećih ili priprema novih artikala, zaglavlje, obavezna prodajna cijena, kompaktna tabelarna izmjena, zavisni troškovi, zbirovi, završavanje u nalog/lager sa statusom čeka KUF i A4 landscape štampa. KUF knjiga ima pregled i grupno preuzimanje završenih kalkulacija.</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="str">
-        <v>E-025</v>
+        <v>E-024</v>
       </c>
       <c r="B314" t="str">
         <v>Robno knjigovodstvo</v>
       </c>
       <c r="C314" t="str">
-        <v>Povrat dobavljaču</v>
+        <v>Uvozna kalkulacija</v>
       </c>
       <c r="D314" t="str">
-        <v>Slobodan ili povezan povrat robe dobavljaču.</v>
+        <v>Kalkulacija sa carinskom deklaracijom.</v>
       </c>
       <c r="E314" t="str">
         <v>Vrlo visok</v>
@@ -11960,50 +12001,50 @@
         <v>Navigacija pripremljena</v>
       </c>
       <c r="G314" t="str">
-        <v>F-052</v>
+        <v>F-051</v>
       </c>
       <c r="H314" t="str">
-        <v>/agencija/robno/povrat-dobavljacu; poslovna logika nije implementirana.</v>
+        <v>/agencija/robno/uvozne-kalkulacije; poslovna logika nije implementirana.</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="str">
-        <v>E-026</v>
+        <v>E-025</v>
       </c>
       <c r="B315" t="str">
         <v>Robno knjigovodstvo</v>
       </c>
       <c r="C315" t="str">
-        <v>Prenos robe</v>
+        <v>Povrat dobavljaču</v>
       </c>
       <c r="D315" t="str">
-        <v>Prenos između magacina.</v>
+        <v>Slobodan ili povezan povrat robe dobavljaču.</v>
       </c>
       <c r="E315" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F315" t="str">
         <v>Navigacija pripremljena</v>
       </c>
       <c r="G315" t="str">
-        <v>F-054</v>
+        <v>F-052</v>
       </c>
       <c r="H315" t="str">
-        <v>/agencija/robno/prenos; poslovna logika nije implementirana.</v>
+        <v>/agencija/robno/povrat-dobavljacu; poslovna logika nije implementirana.</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="str">
-        <v>E-027</v>
+        <v>E-026</v>
       </c>
       <c r="B316" t="str">
         <v>Robno knjigovodstvo</v>
       </c>
       <c r="C316" t="str">
-        <v>Popis robe</v>
+        <v>Prenos robe</v>
       </c>
       <c r="D316" t="str">
-        <v>Unos stvarnog stanja, višak i manjak.</v>
+        <v>Prenos između magacina.</v>
       </c>
       <c r="E316" t="str">
         <v>Visok</v>
@@ -12012,24 +12053,24 @@
         <v>Navigacija pripremljena</v>
       </c>
       <c r="G316" t="str">
-        <v>F-055</v>
+        <v>F-054</v>
       </c>
       <c r="H316" t="str">
-        <v>/agencija/robno/popis; poslovna logika nije implementirana.</v>
+        <v>/agencija/robno/prenos; poslovna logika nije implementirana.</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="str">
-        <v>E-028</v>
+        <v>E-027</v>
       </c>
       <c r="B317" t="str">
         <v>Robno knjigovodstvo</v>
       </c>
       <c r="C317" t="str">
-        <v>Otpis robe</v>
+        <v>Popis robe</v>
       </c>
       <c r="D317" t="str">
-        <v>Otpis i razduženje robe.</v>
+        <v>Unos stvarnog stanja, višak i manjak.</v>
       </c>
       <c r="E317" t="str">
         <v>Visok</v>
@@ -12038,24 +12079,24 @@
         <v>Navigacija pripremljena</v>
       </c>
       <c r="G317" t="str">
-        <v>F-058</v>
+        <v>F-055</v>
       </c>
       <c r="H317" t="str">
-        <v>/agencija/robno/otpis; poslovna logika nije implementirana.</v>
+        <v>/agencija/robno/popis; poslovna logika nije implementirana.</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="str">
-        <v>E-029</v>
+        <v>E-028</v>
       </c>
       <c r="B318" t="str">
         <v>Robno knjigovodstvo</v>
       </c>
       <c r="C318" t="str">
-        <v>Nivelacija</v>
+        <v>Otpis robe</v>
       </c>
       <c r="D318" t="str">
-        <v>Promjena maloprodajnih cijena.</v>
+        <v>Otpis i razduženje robe.</v>
       </c>
       <c r="E318" t="str">
         <v>Visok</v>
@@ -12064,24 +12105,24 @@
         <v>Navigacija pripremljena</v>
       </c>
       <c r="G318" t="str">
-        <v>F-059</v>
+        <v>F-058</v>
       </c>
       <c r="H318" t="str">
-        <v>/agencija/robno/nivelacija; poslovna logika nije implementirana.</v>
+        <v>/agencija/robno/otpis; poslovna logika nije implementirana.</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="str">
-        <v>E-030</v>
+        <v>E-029</v>
       </c>
       <c r="B319" t="str">
         <v>Robno knjigovodstvo</v>
       </c>
       <c r="C319" t="str">
-        <v>Robni izvještaji</v>
+        <v>Nivelacija</v>
       </c>
       <c r="D319" t="str">
-        <v>Vrijednost zaliha, lager i pregledi po magacinima.</v>
+        <v>Promjena maloprodajnih cijena.</v>
       </c>
       <c r="E319" t="str">
         <v>Visok</v>
@@ -12090,24 +12131,24 @@
         <v>Navigacija pripremljena</v>
       </c>
       <c r="G319" t="str">
-        <v>F-060</v>
+        <v>F-059</v>
       </c>
       <c r="H319" t="str">
-        <v>/agencija/robno/zalihe, /agencija/robno/vrijednost-zaliha i /agencija/robno/kontrole; poslovna logika nije implementirana.</v>
+        <v>/agencija/robno/nivelacija; poslovna logika nije implementirana.</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="str">
-        <v>E-031</v>
+        <v>E-030</v>
       </c>
       <c r="B320" t="str">
         <v>Robno knjigovodstvo</v>
       </c>
       <c r="C320" t="str">
-        <v>Podešavanje negativnog lagera</v>
+        <v>Robni izvještaji</v>
       </c>
       <c r="D320" t="str">
-        <v>Blokiranje ili dozvola zaliha u minus.</v>
+        <v>Vrijednost zaliha, lager i pregledi po magacinima.</v>
       </c>
       <c r="E320" t="str">
         <v>Visok</v>
@@ -12116,128 +12157,128 @@
         <v>Djelimično implementirano</v>
       </c>
       <c r="G320" t="str">
-        <v>F-043</v>
+        <v>F-060</v>
       </c>
       <c r="H320" t="str">
-        <v>Podešavanje je implementirano na /agencija/robno/magacini po firmi i opciono po magacinu; kontrola dokumenata slijedi sa lagerom.</v>
+        <v>/agencija/robno/vrijednost-zaliha je implementirana nad trenutnim stanjem sa filterima po jedinici, magacinu, grupi, artiklu i znaku stanja, zbirima po magacinu i grupi i detaljem artikala. Lager i kartica postoje; /agencija/robno/kontrole ostaje otvorena.</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="str">
-        <v>E-032</v>
+        <v>E-031</v>
       </c>
       <c r="B321" t="str">
-        <v>Izlazne fakture</v>
+        <v>Robno knjigovodstvo</v>
       </c>
       <c r="C321" t="str">
-        <v>Izlazne fakture bez fiskalizacije</v>
+        <v>Podešavanje negativnog lagera</v>
       </c>
       <c r="D321" t="str">
-        <v>Ekran za kreiranje faktura koje mogu razdužiti magacin i kasnije se automatski knjižiti.</v>
+        <v>Blokiranje ili dozvola zaliha u minus.</v>
       </c>
       <c r="E321" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F321" t="str">
-        <v>Navigacija pripremljena</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="G321" t="str">
-        <v>M-004</v>
+        <v>F-043</v>
       </c>
       <c r="H321" t="str">
-        <v>/agencija/robno/izlazne-fakture i /agencija/robno/nova-izlazna-faktura; fiskalizacija nije dio prve verzije.</v>
+        <v>Podešavanje je implementirano na /agencija/robno/magacini po firmi i opciono po magacinu; kontrola dokumenata slijedi sa lagerom.</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="str">
-        <v>E-033</v>
+        <v>E-032</v>
       </c>
       <c r="B322" t="str">
-        <v>Podešavanja / PDV</v>
+        <v>Izlazne fakture</v>
       </c>
       <c r="C322" t="str">
-        <v>PDV stope</v>
+        <v>Izlazne fakture bez fiskalizacije</v>
       </c>
       <c r="D322" t="str">
-        <v>Ekran za unos, pregled, izmjenu i aktivaciju/deaktivaciju PDV stopa.</v>
+        <v>Ekran za kreiranje faktura koje mogu razdužiti magacin i kasnije se automatski knjižiti.</v>
       </c>
       <c r="E322" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F322" t="str">
-        <v>Implementirano</v>
+        <v>Navigacija pripremljena</v>
       </c>
       <c r="G322" t="str">
-        <v>F-062</v>
+        <v>M-004</v>
       </c>
       <c r="H322" t="str">
-        <v>/agencija/podesavanja/pdv-stope</v>
+        <v>/agencija/robno/izlazne-fakture i /agencija/robno/nova-izlazna-faktura; fiskalizacija nije dio prve verzije.</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="str">
-        <v>E-034</v>
+        <v>E-033</v>
       </c>
       <c r="B323" t="str">
-        <v>Računi / KUF</v>
+        <v>Podešavanja / PDV</v>
       </c>
       <c r="C323" t="str">
-        <v>KUF knjige i detalj KUF-a</v>
+        <v>PDV stope</v>
       </c>
       <c r="D323" t="str">
-        <v>Računi / Podešavanja prikazuju vrste KIF/KUF i šemu kontiranja po poljima. KUF i KIF imaju otvaranje knjige i unos računa; KIF konto prihoda zavisi od šeme.</v>
+        <v>Ekran za unos, pregled, izmjenu i aktivaciju/deaktivaciju PDV stopa.</v>
       </c>
       <c r="E323" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F323" t="str">
-        <v>Implementirano djelimicno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G323" t="str">
-        <v>F-063</v>
+        <v>F-062</v>
       </c>
       <c r="H323" t="str">
-        <v>/agencija/racuni/podesavanja, /agencija/racuni/kuf, /agencija/racuni/kuf/[id], /agencija/racuni/kif/[id], /agencija/racuni/import, /agencija/racuni/neproknjizeno, /agencija/racuni/pregled-kuf i /agencija/racuni/pregled-kuf/[id]. Dodato knjiženje/dopuna naloga, uvoz podešavanja i pojedinačno/višestruko lokalno čitanje MAPR QR koda iz PDF/TIFF/JPG/PNG računa. Import prikazuje progres po grupama, preskače lokalno pronađene KUF duplikate prije MAPR-a, izdvaja neuspjele fajlove/linkove sa retry/CSV akcijama i grupiše nove dobavljače bez konta po PIB-u.</v>
+        <v>/agencija/podesavanja/pdv-stope</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="str">
-        <v>E-035</v>
+        <v>E-034</v>
       </c>
       <c r="B324" t="str">
-        <v>PDV</v>
+        <v>Računi / KUF</v>
       </c>
       <c r="C324" t="str">
-        <v>PDV pregled</v>
+        <v>KUF knjige i detalj KUF-a</v>
       </c>
       <c r="D324" t="str">
-        <v>Lista mjesečnih PDV perioda za aktivnu firmu/godinu sa statusom i zbirnim iznosima.</v>
+        <v>Računi / Podešavanja prikazuju vrste KIF/KUF i šemu kontiranja po poljima. KUF i KIF imaju otvaranje knjige i unos računa; KIF konto prihoda zavisi od šeme.</v>
       </c>
       <c r="E324" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F324" t="str">
-        <v>Implementirano</v>
+        <v>Implementirano djelimicno</v>
       </c>
       <c r="G324" t="str">
-        <v>F-072</v>
+        <v>F-063</v>
       </c>
       <c r="H324" t="str">
-        <v>/agencija/pdv</v>
+        <v>/agencija/racuni/podesavanja, /agencija/racuni/kuf, /agencija/racuni/kuf/[id], /agencija/racuni/kif/[id], /agencija/racuni/import, /agencija/racuni/neproknjizeno, /agencija/racuni/pregled-kuf i /agencija/racuni/pregled-kuf/[id]. Dodato knjiženje/dopuna naloga, uvoz podešavanja i pojedinačno/višestruko lokalno čitanje MAPR QR koda iz PDF/TIFF/JPG/PNG računa. Import prikazuje progres po grupama, preskače lokalno pronađene KUF duplikate prije MAPR-a, izdvaja neuspjele fajlove/linkove sa retry/CSV akcijama i grupiše nove dobavljače bez konta po PIB-u.</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="str">
-        <v>E-036</v>
+        <v>E-035</v>
       </c>
       <c r="B325" t="str">
         <v>PDV</v>
       </c>
       <c r="C325" t="str">
-        <v>Ulazni PDV</v>
+        <v>PDV pregled</v>
       </c>
       <c r="D325" t="str">
-        <v>Dokazna evidencija KUF računa za izabrani mjesec po datumu KUF knjige.</v>
+        <v>Lista mjesečnih PDV perioda za aktivnu firmu/godinu sa statusom i zbirnim iznosima.</v>
       </c>
       <c r="E325" t="str">
         <v>Vrlo visok</v>
@@ -12246,24 +12287,24 @@
         <v>Implementirano</v>
       </c>
       <c r="G325" t="str">
-        <v>F-073</v>
+        <v>F-072</v>
       </c>
       <c r="H325" t="str">
-        <v>/agencija/pdv/ulazni</v>
+        <v>/agencija/pdv</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="str">
-        <v>E-037</v>
+        <v>E-036</v>
       </c>
       <c r="B326" t="str">
         <v>PDV</v>
       </c>
       <c r="C326" t="str">
-        <v>Izlazni PDV</v>
+        <v>Ulazni PDV</v>
       </c>
       <c r="D326" t="str">
-        <v>Dokazna evidencija KIF računa za izabrani mjesec po datumu KIF knjige.</v>
+        <v>Dokazna evidencija KUF računa za izabrani mjesec po datumu KUF knjige.</v>
       </c>
       <c r="E326" t="str">
         <v>Vrlo visok</v>
@@ -12275,50 +12316,50 @@
         <v>F-073</v>
       </c>
       <c r="H326" t="str">
-        <v>/agencija/pdv/izlazni</v>
+        <v>/agencija/pdv/ulazni</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="str">
-        <v>E-038</v>
+        <v>E-037</v>
       </c>
       <c r="B327" t="str">
         <v>PDV</v>
       </c>
       <c r="C327" t="str">
-        <v>PDV prijava</v>
+        <v>Izlazni PDV</v>
       </c>
       <c r="D327" t="str">
-        <v>IRMS-like obrazac prijave sa lijevom/desnom PDV kolonom i automatskim preračunima.</v>
+        <v>Dokazna evidencija KIF računa za izabrani mjesec po datumu KIF knjige.</v>
       </c>
       <c r="E327" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F327" t="str">
-        <v>Implementirano djelimicno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G327" t="str">
-        <v>F-074</v>
+        <v>F-073</v>
       </c>
       <c r="H327" t="str">
-        <v>/agencija/pdv/prijava</v>
+        <v>/agencija/pdv/izlazni</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="str">
-        <v>E-039</v>
+        <v>E-038</v>
       </c>
       <c r="B328" t="str">
         <v>PDV</v>
       </c>
       <c r="C328" t="str">
-        <v>PDV kontrole</v>
+        <v>PDV prijava</v>
       </c>
       <c r="D328" t="str">
-        <v>Kontrole prije XML izvoza i knjiženja prijave; uključuje neproknjižene/rasknjižene KIF/KUF stavke i poređenje sa glavnom knjigom.</v>
+        <v>IRMS-like obrazac prijave sa lijevom/desnom PDV kolonom i automatskim preračunima.</v>
       </c>
       <c r="E328" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F328" t="str">
         <v>Implementirano djelimicno</v>
@@ -12327,102 +12368,102 @@
         <v>F-074</v>
       </c>
       <c r="H328" t="str">
-        <v>/agencija/pdv/kontrole</v>
+        <v>/agencija/pdv/prijava</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="str">
-        <v>E-040</v>
+        <v>E-039</v>
       </c>
       <c r="B329" t="str">
         <v>PDV</v>
       </c>
       <c r="C329" t="str">
-        <v>Arhiva PDV prijava</v>
+        <v>PDV kontrole</v>
       </c>
       <c r="D329" t="str">
-        <v>Lista sačuvanih/proknjiženih prijava i linkovi na XML/nalog.</v>
+        <v>Kontrole prije XML izvoza i knjiženja prijave; uključuje neproknjižene/rasknjižene KIF/KUF stavke i poređenje sa glavnom knjigom.</v>
       </c>
       <c r="E329" t="str">
         <v>Visok</v>
       </c>
       <c r="F329" t="str">
-        <v>Implementirano</v>
+        <v>Implementirano djelimicno</v>
       </c>
       <c r="G329" t="str">
         <v>F-074</v>
       </c>
       <c r="H329" t="str">
-        <v>/agencija/pdv/arhiva</v>
+        <v>/agencija/pdv/kontrole</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="str">
-        <v>E-041</v>
+        <v>E-040</v>
       </c>
       <c r="B330" t="str">
         <v>PDV</v>
       </c>
       <c r="C330" t="str">
-        <v>Podešavanja PDV-a</v>
+        <v>Arhiva PDV prijava</v>
       </c>
       <c r="D330" t="str">
-        <v>Vrsta naloga i šema D/P + konto za knjiženje PDV prijave po aktivnim stopama; konto dropdown prikazuje cijeli spojeni kontni plan.</v>
+        <v>Lista sačuvanih/proknjiženih prijava i linkovi na XML/nalog.</v>
       </c>
       <c r="E330" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F330" t="str">
         <v>Implementirano</v>
       </c>
       <c r="G330" t="str">
-        <v>F-075</v>
+        <v>F-074</v>
       </c>
       <c r="H330" t="str">
-        <v>/agencija/pdv/podesavanja</v>
+        <v>/agencija/pdv/arhiva</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="str">
-        <v>E-042</v>
+        <v>E-041</v>
       </c>
       <c r="B331" t="str">
-        <v>Plate i zaposleni</v>
+        <v>PDV</v>
       </c>
       <c r="C331" t="str">
-        <v>Podešavanja plata</v>
+        <v>Podešavanja PDV-a</v>
       </c>
       <c r="D331" t="str">
-        <v>Pregled grupa podešavanja; IOPPD šifre otvaraju šifarnik osnova i pravila sa pripadajućim obračunskim podšiframa, koeficijentima, posebnim procentom osnovice i fondom sati, a podešavanje knjiženja čuva kategorijsku D/P šemu.</v>
+        <v>Vrsta naloga i šema D/P + konto za knjiženje PDV prijave po aktivnim stopama; konto dropdown prikazuje cijeli spojeni kontni plan.</v>
       </c>
       <c r="E331" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F331" t="str">
         <v>Implementirano</v>
       </c>
       <c r="G331" t="str">
-        <v>M-006</v>
+        <v>F-075</v>
       </c>
       <c r="H331" t="str">
-        <v>/agencija/plate/podesavanja</v>
+        <v>/agencija/pdv/podesavanja</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="str">
-        <v>E-043</v>
+        <v>E-042</v>
       </c>
       <c r="B332" t="str">
         <v>Plate i zaposleni</v>
       </c>
       <c r="C332" t="str">
-        <v>M-4 evidencija</v>
+        <v>Podešavanja plata</v>
       </c>
       <c r="D332" t="str">
-        <v>Godišnji kontrolni pregled osiguranika i potvrđene mjesečne uplate, uključujući preuzimanje pune uplate iz obračuna jednim klikom; matični podaci dolaze iz firme, naziv i DJP šifra opštine iz globalnog šifarnika prireza, a štampa pojedinačnog M-4, Tabele 1 i Tabele 2 prati zvanične PDF uzorke.</v>
+        <v>Pregled grupa podešavanja; IOPPD šifre otvaraju šifarnik osnova i pravila sa pripadajućim obračunskim podšiframa, koeficijentima, posebnim procentom osnovice i fondom sati, a podešavanje knjiženja čuva kategorijsku D/P šemu.</v>
       </c>
       <c r="E332" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F332" t="str">
         <v>Implementirano</v>
@@ -12431,24 +12472,24 @@
         <v>M-006</v>
       </c>
       <c r="H332" t="str">
-        <v>/agencija/plate/obrasci/m4, /stampa/plate/m4</v>
+        <v>/agencija/plate/podesavanja</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="str">
-        <v>E-044</v>
+        <v>E-043</v>
       </c>
       <c r="B333" t="str">
         <v>Plate i zaposleni</v>
       </c>
       <c r="C333" t="str">
-        <v>Obrasci plata</v>
+        <v>M-4 evidencija</v>
       </c>
       <c r="D333" t="str">
-        <v>Pregledna grupa i drugi nivo podmenija za M-4, OPP-ND i IOPPD, bez promjene postojećih funkcionalnosti obrazaca.</v>
+        <v>Godišnji kontrolni pregled osiguranika i potvrđene mjesečne uplate, uključujući preuzimanje pune uplate iz obračuna jednim klikom; matični podaci dolaze iz firme, naziv i DJP šifra opštine iz globalnog šifarnika prireza, a štampa pojedinačnog M-4, Tabele 1 i Tabele 2 prati zvanične PDF uzorke.</v>
       </c>
       <c r="E333" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F333" t="str">
         <v>Implementirano</v>
@@ -12457,47 +12498,47 @@
         <v>M-006</v>
       </c>
       <c r="H333" t="str">
-        <v>/agencija/plate/obrasci</v>
+        <v>/agencija/plate/obrasci/m4, /stampa/plate/m4</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="str">
-        <v>E-045</v>
+        <v>E-044</v>
       </c>
       <c r="B334" t="str">
         <v>Plate i zaposleni</v>
       </c>
       <c r="C334" t="str">
-        <v>OPP-ND</v>
+        <v>Obrasci plata</v>
       </c>
       <c r="D334" t="str">
-        <v>Mjesečni pregled prireza po vrstama poreza i važećoj opštinskoj stopi firme, sa službenom A4 štampom prema dostavljenom PDF obrascu.</v>
+        <v>Pregledna grupa i drugi nivo podmenija za M-4, OPP-ND i IOPPD, bez promjene postojećih funkcionalnosti obrazaca.</v>
       </c>
       <c r="E334" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F334" t="str">
         <v>Implementirano</v>
       </c>
       <c r="G334" t="str">
-        <v>F-094</v>
+        <v>M-006</v>
       </c>
       <c r="H334" t="str">
-        <v>/agencija/plate/obrasci/opp-nd, /stampa/plate/opp-nd</v>
+        <v>/agencija/plate/obrasci</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="str">
-        <v>E-046</v>
+        <v>E-045</v>
       </c>
       <c r="B335" t="str">
-        <v>Robno knjigovodstvo</v>
+        <v>Plate i zaposleni</v>
       </c>
       <c r="C335" t="str">
-        <v>Podešavanja kalkulacije</v>
+        <v>OPP-ND</v>
       </c>
       <c r="D335" t="str">
-        <v>Firm-specific D/P konta za automatsko knjiženje domaće kalkulacije.</v>
+        <v>Mjesečni pregled prireza po vrstama poreza i važećoj opštinskoj stopi firme, sa službenom A4 štampom prema dostavljenom PDF obrascu.</v>
       </c>
       <c r="E335" t="str">
         <v>Vrlo visok</v>
@@ -12506,24 +12547,24 @@
         <v>Implementirano</v>
       </c>
       <c r="G335" t="str">
-        <v>F-061</v>
+        <v>F-094</v>
       </c>
       <c r="H335" t="str">
-        <v>/agencija/robno/podesavanja; roba, ulazni PDV, dobavljač, razlika u cijeni, ukalkulisani PDV i zavisni troškovi.</v>
+        <v>/agencija/plate/obrasci/opp-nd, /stampa/plate/opp-nd</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="str">
-        <v>E-047</v>
+        <v>E-046</v>
       </c>
       <c r="B336" t="str">
-        <v>Računi / KIF</v>
+        <v>Robno knjigovodstvo</v>
       </c>
       <c r="C336" t="str">
-        <v>Unos pazara</v>
+        <v>Podešavanja kalkulacije</v>
       </c>
       <c r="D336" t="str">
-        <v>Dnevni ili mjesečni pazar sa periodom, izvještajem, kasom, osnovicama/izlaznim PDV-om, kontrolnim zbirovima i raspodjelom naplate.</v>
+        <v>Firm-specific D/P konta za automatsko knjiženje domaće kalkulacije.</v>
       </c>
       <c r="E336" t="str">
         <v>Vrlo visok</v>
@@ -12532,24 +12573,24 @@
         <v>Implementirano</v>
       </c>
       <c r="G336" t="str">
-        <v>F-095</v>
+        <v>F-061</v>
       </c>
       <c r="H336" t="str">
-        <v>/agencija/racuni/kif/[id]?unos=pazar</v>
+        <v>/agencija/robno/podesavanja; roba, ulazni PDV, dobavljač, razlika u cijeni, ukalkulisani PDV i zavisni troškovi.</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="str">
-        <v>E-048</v>
+        <v>E-047</v>
       </c>
       <c r="B337" t="str">
-        <v>POS / Kasa</v>
+        <v>Računi / KIF</v>
       </c>
       <c r="C337" t="str">
-        <v>Smjene i presjeci</v>
+        <v>Unos pazara</v>
       </c>
       <c r="D337" t="str">
-        <v>Otvaranje smjene i završni presjek prometa pri predaji kase.</v>
+        <v>Dnevni ili mjesečni pazar sa periodom, izvještajem, kasom, osnovicama/izlaznim PDV-om, kontrolnim zbirovima i raspodjelom naplate.</v>
       </c>
       <c r="E337" t="str">
         <v>Vrlo visok</v>
@@ -12558,24 +12599,24 @@
         <v>Implementirano</v>
       </c>
       <c r="G337" t="str">
-        <v>F-099</v>
+        <v>F-095</v>
       </c>
       <c r="H337" t="str">
-        <v>/agencija/pos/smjene</v>
+        <v>/agencija/racuni/kif/[id]?unos=pazar</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="str">
-        <v>E-049</v>
+        <v>E-048</v>
       </c>
       <c r="B338" t="str">
-        <v>Portal direktnog fiskalnog klijenta</v>
+        <v>POS / Kasa</v>
       </c>
       <c r="C338" t="str">
-        <v>Portal dashboard</v>
+        <v>Smjene i presjeci</v>
       </c>
       <c r="D338" t="str">
-        <v>Operativni pregled prometa, računa, storna, plaćanja, posljednjih dokumenata i upozorenja.</v>
+        <v>Otvaranje smjene i završni presjek prometa pri predaji kase.</v>
       </c>
       <c r="E338" t="str">
         <v>Vrlo visok</v>
@@ -12584,50 +12625,50 @@
         <v>Implementirano</v>
       </c>
       <c r="G338" t="str">
-        <v>F-101</v>
+        <v>F-099</v>
       </c>
       <c r="H338" t="str">
-        <v>/portal</v>
+        <v>/agencija/pos/smjene</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="str">
-        <v>E-050</v>
+        <v>E-049</v>
       </c>
       <c r="B339" t="str">
         <v>Portal direktnog fiskalnog klijenta</v>
       </c>
       <c r="C339" t="str">
-        <v>Portal POS</v>
+        <v>Portal dashboard</v>
       </c>
       <c r="D339" t="str">
-        <v>Mobile-first prodaja nad postojećim POS terminalom i servisima, u zasebnom portal layoutu.</v>
+        <v>Operativni pregled prometa, računa, storna, plaćanja, posljednjih dokumenata i upozorenja.</v>
       </c>
       <c r="E339" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F339" t="str">
-        <v>Implementirano djelimično</v>
+        <v>Implementirano</v>
       </c>
       <c r="G339" t="str">
-        <v>F-102</v>
+        <v>F-101</v>
       </c>
       <c r="H339" t="str">
-        <v>/portal/pos</v>
+        <v>/portal</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="str">
-        <v>E-051</v>
+        <v>E-050</v>
       </c>
       <c r="B340" t="str">
         <v>Portal direktnog fiskalnog klijenta</v>
       </c>
       <c r="C340" t="str">
-        <v>Portal fakture</v>
+        <v>Portal POS</v>
       </c>
       <c r="D340" t="str">
-        <v>Lista, novi nacrt, detalj, pregled i fiskalizacija klasične bezgotovinske fakture.</v>
+        <v>Mobile-first prodaja nad postojećim POS terminalom i servisima, u zasebnom portal layoutu.</v>
       </c>
       <c r="E340" t="str">
         <v>Vrlo visok</v>
@@ -12639,21 +12680,21 @@
         <v>F-102</v>
       </c>
       <c r="H340" t="str">
-        <v>/portal/fakture, /portal/fakture/nova, /portal/fakture/[id]</v>
+        <v>/portal/pos</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="str">
-        <v>E-052</v>
+        <v>E-051</v>
       </c>
       <c r="B341" t="str">
         <v>Portal direktnog fiskalnog klijenta</v>
       </c>
       <c r="C341" t="str">
-        <v>Fiskalni računi i izvještaji</v>
+        <v>Portal fakture</v>
       </c>
       <c r="D341" t="str">
-        <v>Jedinstveni pregled POS, OFFICE i storno dokumenata sa filterima, štampom, retry-em i izvještajima.</v>
+        <v>Lista, novi nacrt, detalj, pregled i fiskalizacija klasične bezgotovinske fakture.</v>
       </c>
       <c r="E341" t="str">
         <v>Vrlo visok</v>
@@ -12662,41 +12703,67 @@
         <v>Implementirano djelimično</v>
       </c>
       <c r="G341" t="str">
-        <v>F-103</v>
+        <v>F-102</v>
       </c>
       <c r="H341" t="str">
-        <v>/portal/racuni, /portal/racuni/[id], /portal/racuni/[id]/storno, /portal/izvjestaji</v>
+        <v>/portal/fakture, /portal/fakture/nova, /portal/fakture/[id]</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="str">
-        <v>E-053</v>
+        <v>E-052</v>
       </c>
       <c r="B342" t="str">
         <v>Portal direktnog fiskalnog klijenta</v>
       </c>
       <c r="C342" t="str">
-        <v>Šifarnici i operativna podešavanja</v>
+        <v>Fiskalni računi i izvještaji</v>
       </c>
       <c r="D342" t="str">
-        <v>Artikli, grupe, cijene, kupci i dozvoljena lokalna podešavanja bez fiskalne administracije.</v>
+        <v>Jedinstveni pregled POS, OFFICE i storno dokumenata sa filterima, štampom, retry-em i izvještajima.</v>
       </c>
       <c r="E342" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F342" t="str">
-        <v>Implementirano</v>
+        <v>Implementirano djelimično</v>
       </c>
       <c r="G342" t="str">
         <v>F-103</v>
       </c>
       <c r="H342" t="str">
+        <v>/portal/racuni, /portal/racuni/[id], /portal/racuni/[id]/storno, /portal/izvjestaji</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="str">
+        <v>E-053</v>
+      </c>
+      <c r="B343" t="str">
+        <v>Portal direktnog fiskalnog klijenta</v>
+      </c>
+      <c r="C343" t="str">
+        <v>Šifarnici i operativna podešavanja</v>
+      </c>
+      <c r="D343" t="str">
+        <v>Artikli, grupe, cijene, kupci i dozvoljena lokalna podešavanja bez fiskalne administracije.</v>
+      </c>
+      <c r="E343" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F343" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G343" t="str">
+        <v>F-103</v>
+      </c>
+      <c r="H343" t="str">
         <v>/portal/artikli, /portal/grupe, /portal/cijene, /portal/kupci, /portal/podesavanja</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z342"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z343"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: add payroll documents and payment orders
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -2697,7 +2697,7 @@
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA376"/>
+  <dimension ref="A1:AA377"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7082,9 +7082,47 @@
         <v>Admin-only podešavanje po agenciji, backend validacija, audit i probno slanje. Pozivnice koje kreira admin agencije koriste sačuvani Reply-To; produkcijski SMTP nalog mora biti ovlašćen za centralnu From adresu.</v>
       </c>
     </row>
+    <row r="377">
+      <c r="A377" t="str">
+        <v>F-115</v>
+      </c>
+      <c r="B377" t="str">
+        <v>Plate i zaposleni</v>
+      </c>
+      <c r="C377" t="str">
+        <v>Dokumenti obračuna plata</v>
+      </c>
+      <c r="D377" t="str">
+        <v>Obračun daje pojedinačne i zbirne platne liste, rekapitulaciju i kontrolisane naloge za plaćanje iz istih sačuvanih stavki.</v>
+      </c>
+      <c r="E377" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F377" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G377" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H377" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I377" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J377" t="str">
+        <v>Djelimično</v>
+      </c>
+      <c r="K377" t="str">
+        <v>M-006,F-089</v>
+      </c>
+      <c r="L377" t="str">
+        <v>A4 HTML/CSS štampa je dostupna uz plate/view i plate/export; obračunati dokumenti nose NACRT. Neto ide po radniku; porez, PIO, nezaposlenost i Fond rada zbirno na 820-30000-74; prirez posebno po opštini, a sindikat i Komora zasebno kada imaju iznos.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA376"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA377"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -11189,7 +11227,7 @@
 
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z343"/>
+  <dimension ref="A1:Z344"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -12761,9 +12799,35 @@
         <v>/portal/artikli, /portal/grupe, /portal/cijene, /portal/kupci, /portal/podesavanja</v>
       </c>
     </row>
+    <row r="344">
+      <c r="A344" t="str">
+        <v>E-054</v>
+      </c>
+      <c r="B344" t="str">
+        <v>Plate i zaposleni</v>
+      </c>
+      <c r="C344" t="str">
+        <v>Dokumenti obračuna</v>
+      </c>
+      <c r="D344" t="str">
+        <v>Centralne akcije na detalju obračuna vode na pojedinačne/zbirne platne liste, rekapitulaciju, pregled virmana i IOPPD.</v>
+      </c>
+      <c r="E344" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F344" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G344" t="str">
+        <v>F-115</v>
+      </c>
+      <c r="H344" t="str">
+        <v>/agencija/plate/obracun, /agencija/plate/obracun/nalozi-za-placanje, /stampa/plate/platne-liste, /stampa/plate/rekapitulacija, /stampa/plate/virmani</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z343"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z344"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: add payment orders and improve statement rules
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -2697,7 +2697,7 @@
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA377"/>
+  <dimension ref="A1:AA378"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5863,7 +5863,7 @@
         <v>F-081</v>
       </c>
       <c r="L344" t="str">
-        <v>Pravila podržavaju smjer, žiro račun, opis, šifru plaćanja, poziv na broj, prioritet, zajednički scope agencije i firm-specific override; account_code omogućava primjenu kroz firme.</v>
+        <v>Pravila podržavaju smjer, žiro račun, opis, šifru plaćanja, poziv na broj, prioritet, zajednički scope agencije i firm-specific override; account_code omogućava primjenu kroz firme. Automatsko učenje po poznatom žiro računu čuva jedno fallback pravilo po računu i smjeru bez rednog broja, opisa i šifre plaćanja. Lovćen M02 stavke bez kontra računa uče samo uslov po šifri i smjeru, bez naziva prodavnice i partnera. Neproknjižen izvod može ručno ponovo primijeniti pravila bez prepisivanja ručnog konta, a preview prikazuje konkretne razloge blokade. Regresioni testovi pokrivaju M02, fallback, firm-specific prioritet i analitičko konto.</v>
       </c>
     </row>
     <row r="345">
@@ -7117,12 +7117,50 @@
         <v>M-006,F-089</v>
       </c>
       <c r="L377" t="str">
-        <v>A4 HTML/CSS štampa je dostupna uz plate/view i plate/export; obračunati dokumenti nose NACRT. Neto ide po radniku; porez, PIO, nezaposlenost i Fond rada zbirno na 820-30000-74; prirez posebno po opštini, a sindikat i Komora zasebno kada imaju iznos.</v>
+        <v>A4 HTML/CSS štampa je dostupna uz plate/view i plate/export; obračunati dokumenti nose NACRT. Virmani prate dostavljeni PDF raspored sa tri obrasca po A4 strani i podesivom gornjom/lijevom marginom. Kompaktna priprema bez horizontalnog skrola omogućava lokalnu korekciju svih polja prije štampe, bez izmjene obračuna u bazi. Neto ide po radniku; porez, PIO, nezaposlenost i Fond rada zbirno na 820-30000-74; prirez posebno po opštini, Komora na 520-939100-43 i sindikat na 510-105-16.</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="str">
+        <v>F-116</v>
+      </c>
+      <c r="B378" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="C378" t="str">
+        <v>Opšti virmani</v>
+      </c>
+      <c r="D378" t="str">
+        <v>Ručni platni nalozi nevezani za obračun plata čuvaju se kao nacrti, odštampani zapisi ili šabloni i štampaju po tri na A4.</v>
+      </c>
+      <c r="E378" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F378" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G378" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H378" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I378" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J378" t="str">
+        <v>Djelimično</v>
+      </c>
+      <c r="K378" t="str">
+        <v>M-001,M-002,M-009</v>
+      </c>
+      <c r="L378" t="str">
+        <v>Aktivna firma predlaže nalogodavca i glavni račun; sva polja su izmjenjiva. Zasebna virmani prava štite pregled/unos/izmjenu/brisanje/izvoz. Modul ne knjiži promet niti mijenja izvode.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA377"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA378"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -11227,7 +11265,7 @@
 
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z344"/>
+  <dimension ref="A1:Z345"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -12810,7 +12848,7 @@
         <v>Dokumenti obračuna</v>
       </c>
       <c r="D344" t="str">
-        <v>Centralne akcije na detalju obračuna vode na pojedinačne/zbirne platne liste, rekapitulaciju, pregled virmana i IOPPD.</v>
+        <v>Centralne akcije na detalju obračuna vode na pojedinačne/zbirne platne liste, rekapitulaciju, kompaktno uređivanje virmana u rasporedu stvarnog obrasca i IOPPD; štampa virmana koristi tri pozicionirana obrasca po A4 strani i korekciju margina.</v>
       </c>
       <c r="E344" t="str">
         <v>Vrlo visok</v>
@@ -12825,9 +12863,35 @@
         <v>/agencija/plate/obracun, /agencija/plate/obracun/nalozi-za-placanje, /stampa/plate/platne-liste, /stampa/plate/rekapitulacija, /stampa/plate/virmani</v>
       </c>
     </row>
+    <row r="345">
+      <c r="A345" t="str">
+        <v>E-055</v>
+      </c>
+      <c r="B345" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="C345" t="str">
+        <v>Opšti virmani</v>
+      </c>
+      <c r="D345" t="str">
+        <v>Novi virman, nacrti, istorija odštampanih naloga, šabloni i grupna štampa u rasporedu stvarnog obrasca.</v>
+      </c>
+      <c r="E345" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F345" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G345" t="str">
+        <v>F-116</v>
+      </c>
+      <c r="H345" t="str">
+        <v>/agencija/virmani, /stampa/virmani</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z344"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z345"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -17471,7 +17535,7 @@
 
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB357"/>
+  <dimension ref="A1:AB358"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -19555,9 +19619,38 @@
         <v>Nije početo</v>
       </c>
     </row>
+    <row r="358">
+      <c r="A358" t="str">
+        <v>T-088</v>
+      </c>
+      <c r="B358" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="C358" t="str">
+        <v>Regresija automatskih pravila</v>
+      </c>
+      <c r="D358" t="str">
+        <v>M02 radi bez kontra žiro računa i nezavisno od trgovca; fallback po žiro računu ne zavisi od rednog broja/opisa/šifre; firm-specific pravilo ima prednost; analitičko konto bez partnera blokira knjiženje.</v>
+      </c>
+      <c r="E358" t="str">
+        <v>F-082</v>
+      </c>
+      <c r="F358" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G358" t="str">
+        <v>Codex</v>
+      </c>
+      <c r="H358">
+        <v>46289.083333333336</v>
+      </c>
+      <c r="I358" t="str">
+        <v>Pet automatizovanih testova prolazi kroz npm run test:bank-statements; u browseru potvrđen tačan razlog blokade na stavci i zbirnom upozorenju.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB357"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB358"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add agency IMAP mail rules and bank statement attachment import
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -2697,7 +2697,7 @@
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA378"/>
+  <dimension ref="A1:AA382"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7158,9 +7158,161 @@
         <v>Aktivna firma predlaže nalogodavca i glavni račun; sva polja su izmjenjiva. Zasebna virmani prava štite pregled/unos/izmjenu/brisanje/izvoz. Modul ne knjiži promet niti mijenja izvode.</v>
       </c>
     </row>
+    <row r="379">
+      <c r="A379" t="str">
+        <v>M7-IMAP-01</v>
+      </c>
+      <c r="B379" t="str">
+        <v>Modul 7</v>
+      </c>
+      <c r="C379" t="str">
+        <v>IMAP test veze</v>
+      </c>
+      <c r="D379" t="str">
+        <v>Read-only INBOX i broj poruka; bez preuzimanja i uvoza</v>
+      </c>
+      <c r="E379" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F379" t="str">
+        <v>Završeno</v>
+      </c>
+      <c r="G379" t="str">
+        <v>DA</v>
+      </c>
+      <c r="H379" t="str">
+        <v>DA</v>
+      </c>
+      <c r="I379" t="str">
+        <v>Nije potrebno</v>
+      </c>
+      <c r="J379" t="str">
+        <v>10/10; TLS i prijava potvrđeni</v>
+      </c>
+      <c r="K379" t="str">
+        <v>Serverski .env</v>
+      </c>
+      <c r="L379" t="str">
+        <v>Admin povezane agencije; IMAP_AGENCY_ID; lozinka u .env</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="str">
+        <v>M7-IMAP-02</v>
+      </c>
+      <c r="B380" t="str">
+        <v>Modul 7</v>
+      </c>
+      <c r="C380" t="str">
+        <v>Pregled mailova</v>
+      </c>
+      <c r="D380" t="str">
+        <v>INBOX lista i tekst poruke sa rucnim preuzimanjem priloga</v>
+      </c>
+      <c r="E380" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F380" t="str">
+        <v>Završeno</v>
+      </c>
+      <c r="G380" t="str">
+        <v>DA</v>
+      </c>
+      <c r="H380" t="str">
+        <v>DA</v>
+      </c>
+      <c r="I380" t="str">
+        <v>Nije potrebno</v>
+      </c>
+      <c r="J380" t="str">
+        <v>16/16 i browser QA</v>
+      </c>
+      <c r="K380" t="str">
+        <v>IMAP veza</v>
+      </c>
+      <c r="L380" t="str">
+        <v>Read-only i tenant scope; bez uvoza izvoda</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="str">
+        <v>M7-IMAP-03</v>
+      </c>
+      <c r="B381" t="str">
+        <v>Modul 7</v>
+      </c>
+      <c r="C381" t="str">
+        <v>Mail pravila po firmi</v>
+      </c>
+      <c r="D381" t="str">
+        <v>Folder i podfolderi uz filtrirani INBOX; opciona AND polja i OR pravila</v>
+      </c>
+      <c r="E381" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F381" t="str">
+        <v>Završeno</v>
+      </c>
+      <c r="G381" t="str">
+        <v>DA</v>
+      </c>
+      <c r="H381" t="str">
+        <v>DA</v>
+      </c>
+      <c r="I381" t="str">
+        <v>DA</v>
+      </c>
+      <c r="J381" t="str">
+        <v>22/22; live i rollback purge</v>
+      </c>
+      <c r="K381" t="str">
+        <v>IMAP pregled</v>
+      </c>
+      <c r="L381" t="str">
+        <v>Bez automatskog uvoza</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="str">
+        <v>M7-IMAP-04</v>
+      </c>
+      <c r="B382" t="str">
+        <v>Modul 7</v>
+      </c>
+      <c r="C382" t="str">
+        <v>Uvoz izvoda iz maila na klik</v>
+      </c>
+      <c r="D382" t="str">
+        <v>Isti parser i obrada kao ručni uvoz; račun i godina; hash i identitet; statusi priloga</v>
+      </c>
+      <c r="E382" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F382" t="str">
+        <v>Završeno</v>
+      </c>
+      <c r="G382" t="str">
+        <v>DA</v>
+      </c>
+      <c r="H382" t="str">
+        <v>DA</v>
+      </c>
+      <c r="I382" t="str">
+        <v>DA</v>
+      </c>
+      <c r="J382" t="str">
+        <v>27 testova i transakcijski rollback test</v>
+      </c>
+      <c r="K382" t="str">
+        <v>IMAP pregled i parseri</v>
+      </c>
+      <c r="L382" t="str">
+        <v>Bez zakazanog rada i automatskog knjiženja</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA378"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA382"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add client reporting portal, user permissions and bank automation
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -2729,7 +2729,7 @@
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA385"/>
+  <dimension ref="A1:AA387"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7453,12 +7453,88 @@
         <v>IMAP pregled i parseri</v>
       </c>
       <c r="L385" t="str">
-        <v>Bez zakazanog rada i automatskog knjiženja</v>
+        <v>Završeni mailovi se preskaču prije download-a; dnevna obrada dodata u M7-IMAP-05</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="str">
+        <v>M7-IMAP-05</v>
+      </c>
+      <c r="B386" t="str">
+        <v>Modul 7</v>
+      </c>
+      <c r="C386" t="str">
+        <v>Dnevna automatska obrada mail izvoda</v>
+      </c>
+      <c r="D386" t="str">
+        <v>10:00 Europe/Podgorica samo aktivne mail firme; uvoz i knjiženje READY mail izvoda</v>
+      </c>
+      <c r="E386" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F386" t="str">
+        <v>Implementirano; čeka deploy</v>
+      </c>
+      <c r="G386" t="str">
+        <v>DA</v>
+      </c>
+      <c r="H386" t="str">
+        <v>DA</v>
+      </c>
+      <c r="I386" t="str">
+        <v>Postojeći audit</v>
+      </c>
+      <c r="J386" t="str">
+        <v>DB rollback regresija</v>
+      </c>
+      <c r="K386" t="str">
+        <v>IMAP uvoz; pravila knjiženja</v>
+      </c>
+      <c r="L386" t="str">
+        <v>Runtime flag; advisory lock; dnevna evidencija; pregled rezultata</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="str">
+        <v>CLIENT-01</v>
+      </c>
+      <c r="B387" t="str">
+        <v>Klijentski portal</v>
+      </c>
+      <c r="C387" t="str">
+        <v>Read-only knjigovodstveni portal</v>
+      </c>
+      <c r="D387" t="str">
+        <v>Kupci i dobavljači preko podešenih konta; kartice; robni dokumenti i šifarnici; lager i PDV.</v>
+      </c>
+      <c r="E387" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F387" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G387" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H387" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I387" t="str">
+        <v>Nije potrebno</v>
+      </c>
+      <c r="J387" t="str">
+        <v>DB rollback; TSC; lint; desktop/mobilni render</v>
+      </c>
+      <c r="K387" t="str">
+        <v>F-006,F-018</v>
+      </c>
+      <c r="L387" t="str">
+        <v>Odvojene liste radnika i klijenata i matrice; dnevnik aktivnosti agencije sa filterima i paginacijom; bez unosa; početna ima top 10 grafikone dugovanja kupaca i dobavljača; interaktivni QA prijavljenog klijenta ostaje otvoren.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA385"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA387"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add agency workflows, deadline tracking and fiscal invoice reversal
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -2729,7 +2729,7 @@
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA387"/>
+  <dimension ref="A1:AA394"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7532,9 +7532,275 @@
         <v>Odvojene liste radnika i klijenata i matrice; dnevnik aktivnosti agencije sa filterima i paginacijom; bez unosa; početna ima top 10 grafikone dugovanja kupaca i dobavljača; interaktivni QA prijavljenog klijenta ostaje otvoren.</v>
       </c>
     </row>
+    <row r="388">
+      <c r="A388" t="str">
+        <v>OFFICE-ST-01</v>
+      </c>
+      <c r="B388" t="str">
+        <v>Robno / Prodaja</v>
+      </c>
+      <c r="C388" t="str">
+        <v>Potpuni storno izlazne fakture</v>
+      </c>
+      <c r="D388" t="str">
+        <v>Fiskalni korektivni OFFICE dokument sa vezom na original; povrat robe, korektivni nalog, KIF i štampa.</v>
+      </c>
+      <c r="E388" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F388" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G388" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H388" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I388" t="str">
+        <v>Nije potrebno</v>
+      </c>
+      <c r="J388" t="str">
+        <v>DB rollback + simulirani Fiscal API</v>
+      </c>
+      <c r="K388" t="str">
+        <v>F-097</v>
+      </c>
+      <c r="L388" t="str">
+        <v>Stabilan idempotency ključ; retry provjerava isti dokument; odvojena lokalna obrada; Live Test QA preostaje.</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="str">
+        <v>TEST-CORE-01</v>
+      </c>
+      <c r="B389" t="str">
+        <v>Računovodstveno jezgro</v>
+      </c>
+      <c r="C389" t="str">
+        <v>Regresioni testovi i CI</v>
+      </c>
+      <c r="D389" t="str">
+        <v>Nalozi; KIF/KUF; PDV; izvodi; puni OFFICE lifecycle; prava i konkurentnost</v>
+      </c>
+      <c r="E389" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F389" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G389" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H389" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I389" t="str">
+        <v>Nije potrebno</v>
+      </c>
+      <c r="J389" t="str">
+        <v>Unit + izolovana PostgreSQL baza + TSC + lint</v>
+      </c>
+      <c r="K389" t="str">
+        <v>Postojeći moduli</v>
+      </c>
+      <c r="L389" t="str">
+        <v>GitHub Linux/PG i Windows/XSD; simulirani fiskalni servis; live QA i browser E2E preostaju.</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="str">
+        <v>AGENCY-01</v>
+      </c>
+      <c r="B390" t="str">
+        <v>Podešavanja</v>
+      </c>
+      <c r="C390" t="str">
+        <v>Profil agencije i podaci ugovora</v>
+      </c>
+      <c r="D390" t="str">
+        <v>Identitet; zastupnik; kontakt; banke; sačuvane ugovorne strane</v>
+      </c>
+      <c r="E390" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F390" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G390" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H390" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I390" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J390" t="str">
+        <v>DB regresija + TypeScript + lint</v>
+      </c>
+      <c r="K390" t="str">
+        <v>Ugovori</v>
+      </c>
+      <c r="L390" t="str">
+        <v>Samo admin svoje agencije; snapshot i izričito osvježavanje; lokalna migracija; deploy preostaje.</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="str">
+        <v>CONTRACT-01</v>
+      </c>
+      <c r="B391" t="str">
+        <v>Firme / Ugovori</v>
+      </c>
+      <c r="C391" t="str">
+        <v>Predložak računovodstvenog ugovora</v>
+      </c>
+      <c r="D391" t="str">
+        <v>13 članova iz Word-a; mapiranje strana i zastupnika; naknada; datumi; rok; sud</v>
+      </c>
+      <c r="E391" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F391" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G391" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H391" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I391" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J391" t="str">
+        <v>Unit + DB + A4 vizuelna provjera</v>
+      </c>
+      <c r="K391" t="str">
+        <v>AGENCY-01</v>
+      </c>
+      <c r="L391" t="str">
+        <v>Snapshot direktora; dva načina roka plaćanja; migracija lokalno; deploy preostaje.</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="str">
+        <v>WARN-BANK-01</v>
+      </c>
+      <c r="B392" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="C392" t="str">
+        <v>Upozorenja za preskočene izvode</v>
+      </c>
+      <c r="D392" t="str">
+        <v>Pregled dostupnih firmi po računu i godini; rasponi i nepoznate oznake</v>
+      </c>
+      <c r="E392" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F392" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G392" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H392" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I392" t="str">
+        <v>Nije potrebno</v>
+      </c>
+      <c r="J392" t="str">
+        <v>Unit + DB rollback + TypeScript + lint</v>
+      </c>
+      <c r="K392" t="str">
+        <v>Modul 7</v>
+      </c>
+      <c r="L392" t="str">
+        <v>Od 1 do najvećeg broja; svi uvezeni statusi; prava radnika; link sa kontekstom.</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="str">
+        <v>STATS-01</v>
+      </c>
+      <c r="B393" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="C393" t="str">
+        <v>Statistika rada agencije</v>
+      </c>
+      <c r="D393" t="str">
+        <v>Nalozi; KIF/KUF; izvodi; plate i ugovori; zaposleni; grafikoni po mjesecima</v>
+      </c>
+      <c r="E393" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F393" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G393" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H393" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I393" t="str">
+        <v>Nije potrebno</v>
+      </c>
+      <c r="J393" t="str">
+        <v>DB rollback + TypeScript + lint + prikaz</v>
+      </c>
+      <c r="K393" t="str">
+        <v>Postojeće evidencije</v>
+      </c>
+      <c r="L393" t="str">
+        <v>Periodični dokumenti; trenutno stanje ljudi; prava po modulu.</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="str">
+        <v>DEADLINES-01</v>
+      </c>
+      <c r="B394" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="C394" t="str">
+        <v>Rokovi po firmama</v>
+      </c>
+      <c r="D394" t="str">
+        <v>Tabovi PDV i plate prethodni mjesec; završni račun prethodna godina; kontrolna lista; raniji zaostaci</v>
+      </c>
+      <c r="E394" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F394" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G394" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H394" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I394" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J394" t="str">
+        <v>Unit + DB rollback + TypeScript + lint</v>
+      </c>
+      <c r="K394" t="str">
+        <v>Postojeće evidencije</v>
+      </c>
+      <c r="L394" t="str">
+        <v>Bez emailova; scope firmi; audit i verzije; nezavisna predaja i kontrolna lista.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA387"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA394"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add employment contracts, job positions and termination documents; improve KUF entry flow
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -2729,7 +2729,7 @@
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA394"/>
+  <dimension ref="A1:AA396"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7798,9 +7798,85 @@
         <v>Bez emailova; scope firmi; audit i verzije; nezavisna predaja i kontrolna lista.</v>
       </c>
     </row>
+    <row r="395">
+      <c r="A395" t="str">
+        <v>HR-JOBS-01</v>
+      </c>
+      <c r="B395" t="str">
+        <v>Plate</v>
+      </c>
+      <c r="C395" t="str">
+        <v>Radna mjesta i ugovori o radu</v>
+      </c>
+      <c r="D395" t="str">
+        <v>Globalni šifarnik i verzije agencije; jedna kartica radnika; rasporedi 8 do 1 sat; snapshot i štampa ugovora</v>
+      </c>
+      <c r="E395" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F395" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G395" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H395" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I395" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J395" t="str">
+        <v>Unit + 13 DB skripti + TSC + lint + vizuelni pregled</v>
+      </c>
+      <c r="K395" t="str">
+        <v>Plate; Firme</v>
+      </c>
+      <c r="L395" t="str">
+        <v>Predložak iz starog sajta; pravna revizija odvojena; aneksi kasnije.</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="str">
+        <v>HR-TERM-01</v>
+      </c>
+      <c r="B396" t="str">
+        <v>Plate</v>
+      </c>
+      <c r="C396" t="str">
+        <v>Prestanak radnog odnosa</v>
+      </c>
+      <c r="D396" t="str">
+        <v>Tri vrste otkaza; datumi; snapshot; štampa iz evidencije bivših radnika</v>
+      </c>
+      <c r="E396" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F396" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G396" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H396" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I396" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J396" t="str">
+        <v>DB rollback + TSC + lint + vizuelni pregled</v>
+      </c>
+      <c r="K396" t="str">
+        <v>Plate; Firme</v>
+      </c>
+      <c r="L396" t="str">
+        <v>Bez elektronske odjave; istorija ostaje nakon reaktivacije.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA394"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA396"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Enforce analytic account length and share financial templates across agency
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -2729,7 +2729,7 @@
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA396"/>
+  <dimension ref="A1:AA397"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3688,7 +3688,7 @@
         <v>M-002</v>
       </c>
       <c r="L28" t="str">
-        <v>Globalni osnovni kontni plan usklađen je sa zadaci/kontni plan.xlsx: 1533 aktivna konta. Puni naziv dolazi iz kolone NAZIV; AK označava obaveznu analitiku, a D korišćenje radne jedinice. Konta uklonjena iz izvora se deaktiviraju radi očuvanja istorije. normalni_saldo je podrazumijevani saldo (0/1/2/5 D, 3/4/6 P), nije zabrana knjiženja. Dostupan na /agencija/podesavanja/kontni-plan.</v>
+        <v>Globalni osnovni kontni plan usklađen je sa zadaci/kontni plan.xlsx: 1533 aktivna konta. Puni naziv dolazi iz kolone NAZIV; AK označava obaveznu analitiku, a D korišćenje radne jedinice. Konta uklonjena iz izvora se deaktiviraju radi očuvanja istorije. normalni_saldo je podrazumijevani saldo (0/1/2/5 D, 3/4/6 P), nije zabrana knjiženja. Dostupan na /agencija/podesavanja/kontni-plan. Konta kraća od 4 znaka su sintetička; migracija i backend/DB zaštita; sistemske šeme 5220/5250; rollback regresija.</v>
       </c>
     </row>
     <row r="29">
@@ -7874,9 +7874,47 @@
         <v>Bez elektronske odjave; istorija ostaje nakon reaktivacije.</v>
       </c>
     </row>
+    <row r="397">
+      <c r="A397" t="str">
+        <v>FIN-AGENCY-01</v>
+      </c>
+      <c r="B397" t="str">
+        <v>Završni račun</v>
+      </c>
+      <c r="C397" t="str">
+        <v>Zajednička šema agencije</v>
+      </c>
+      <c r="D397" t="str">
+        <v>Povezivanje BU/BS/SA bez izbora firme na postojećim stranicama</v>
+      </c>
+      <c r="E397" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F397" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G397" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H397" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I397" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J397" t="str">
+        <v>DB rollback i TypeScript</v>
+      </c>
+      <c r="K397" t="str">
+        <v>M-008</v>
+      </c>
+      <c r="L397" t="str">
+        <v>Šema važi za sve firme agencije; admin prava; transakcioni audit; postojeća povezivanja prenesena.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA396"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA397"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add VAT period locking, cumulative payroll tax and rate-based posting rules
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -2729,7 +2729,7 @@
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA397"/>
+  <dimension ref="A1:AA402"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5705,7 +5705,7 @@
         <v>F-072,F-073</v>
       </c>
       <c r="L339" t="str">
-        <v>Dodat nacrt prijave, osvježavanje iz KIF/KUF, portal layout, XML export u PR_PDV_2025 formatu i osnovno zbirno knjiženje; brisanje PDV naloga vraća prijavu u nacrt. Ostaje zaključavanje i ručni QA XML upload-a.</v>
+        <v>Dodat nacrt prijave, osvježavanje iz KIF/KUF, portal layout, XML export u PR_PDV_2025 formatu i osnovno zbirno knjiženje; brisanje PDV naloga vraća prijavu u nacrt. Zaključavanje i kontrolisano otključavanje sa verzijama i DB regresijom završeni; ostaje ručni QA XML upload-a.</v>
       </c>
     </row>
     <row r="340">
@@ -7912,9 +7912,199 @@
         <v>Šema važi za sve firme agencije; admin prava; transakcioni audit; postojeća povezivanja prenesena.</v>
       </c>
     </row>
+    <row r="398">
+      <c r="A398" t="str">
+        <v>CALC-DELETE-01</v>
+      </c>
+      <c r="B398" t="str">
+        <v>Robno</v>
+      </c>
+      <c r="C398" t="str">
+        <v>Brisanje završene kalkulacije</v>
+      </c>
+      <c r="D398" t="str">
+        <v>Poništenje lagera i soft delete zasebnog naloga i KUF računa uz audit</v>
+      </c>
+      <c r="E398" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F398" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G398" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H398" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I398" t="str">
+        <v>Bez migracije</v>
+      </c>
+      <c r="J398" t="str">
+        <v>DB rollback regresija</v>
+      </c>
+      <c r="K398" t="str">
+        <v>Robno; KUF; Nalozi</v>
+      </c>
+      <c r="L398" t="str">
+        <v>Prava i zaključavanja; razlog i potvrda; blokada zavisnog prometa i plaćanja; idempotentnost.</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="str">
+        <v>PAYROLL-TEST-01</v>
+      </c>
+      <c r="B399" t="str">
+        <v>Plate</v>
+      </c>
+      <c r="C399" t="str">
+        <v>Regresioni testovi obračuna i knjiženja</v>
+      </c>
+      <c r="D399" t="str">
+        <v>Bruto/neto; sati; osnovice; dokumenti; prava; konkurentnost; audit rollback</v>
+      </c>
+      <c r="E399" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F399" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G399" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H399" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I399" t="str">
+        <v>Bez migracije</v>
+      </c>
+      <c r="J399" t="str">
+        <v>Unit i izolovana DB regresija</v>
+      </c>
+      <c r="K399" t="str">
+        <v>Plate</v>
+      </c>
+      <c r="L399" t="str">
+        <v>Zbirni porez i neto dodatak testirani; stale obračun blokiran; stvarni portal nije testiran.</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="str">
+        <v>PDV-LOCK-01</v>
+      </c>
+      <c r="B400" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C400" t="str">
+        <v>Zaključavanje i kontrolisano otključavanje</v>
+      </c>
+      <c r="D400" t="str">
+        <v>Zaštita KIF/KUF i PDV naloga; arhivske verzije; admin razlog i audit; nezavisna predaja u Rokovima</v>
+      </c>
+      <c r="E400" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F400" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G400" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H400" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I400" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J400" t="str">
+        <v>DB lifecycle + concurrency; TSC; lint</v>
+      </c>
+      <c r="K400" t="str">
+        <v>F-074</v>
+      </c>
+      <c r="L400" t="str">
+        <v>Tri migracije; purge usklađen. Plaćanja i nepovezani nalozi dozvoljeni. Ručni portal/browser QA ostaje.</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="str">
+        <v>INVOICE-RATES-01</v>
+      </c>
+      <c r="B401" t="str">
+        <v>Robno</v>
+      </c>
+      <c r="C401" t="str">
+        <v>Dinamička šema prihoda i izlaznog PDV-a</v>
+      </c>
+      <c r="D401" t="str">
+        <v>Dodavanje redova sa stopom i kontom; OFFICE i POS virman</v>
+      </c>
+      <c r="E401" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F401" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G401" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H401" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I401" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J401" t="str">
+        <v>Unit i DB lifecycle; TSC; lint</v>
+      </c>
+      <c r="K401" t="str">
+        <v>Izlazne fakture</v>
+      </c>
+      <c r="L401" t="str">
+        <v>Migracija uklanja stari unique indeks; stari nalozi se ne mijenjaju.</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="str">
+        <v>CALC-RATES-01</v>
+      </c>
+      <c r="B402" t="str">
+        <v>Robno</v>
+      </c>
+      <c r="C402" t="str">
+        <v>Dinamička šema kalkulacije</v>
+      </c>
+      <c r="D402" t="str">
+        <v>Dodavanje stavki i stopa; ulazni i ukalkulisani PDV po stopama</v>
+      </c>
+      <c r="E402" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F402" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G402" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H402" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I402" t="str">
+        <v>Postojeća migracija</v>
+      </c>
+      <c r="J402" t="str">
+        <v>Unit i DB rollback; TSC; lint</v>
+      </c>
+      <c r="K402" t="str">
+        <v>Kalkulacije</v>
+      </c>
+      <c r="L402" t="str">
+        <v>GENERAL fallback bez dupliranja; postojeći nalozi ostaju isti.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA397"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA402"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Omoguci brisanje KUF racuna sa stavkama naloga i prikazi PDV odstupanja
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -2729,7 +2729,7 @@
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA402"/>
+  <dimension ref="A1:AA403"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -8023,7 +8023,7 @@
         <v>F-074</v>
       </c>
       <c r="L400" t="str">
-        <v>Tri migracije; purge usklađen. Plaćanja i nepovezani nalozi dozvoljeni. Ručni portal/browser QA ostaje.</v>
+        <v>Tri migracije; purge usklađen. Plaćanja i nepovezani nalozi dozvoljeni. Ručni portal/browser QA ostaje. Kontrole prikazuju i razlike uz nulti KIF/KUF; tabela sa zelenim/crvenim statusom po kontu.</v>
       </c>
     </row>
     <row r="401">
@@ -8102,9 +8102,47 @@
         <v>GENERAL fallback bez dupliranja; postojeći nalozi ostaju isti.</v>
       </c>
     </row>
+    <row r="403">
+      <c r="A403" t="str">
+        <v>KUF-DELETE-01</v>
+      </c>
+      <c r="B403" t="str">
+        <v>KIF/KUF</v>
+      </c>
+      <c r="C403" t="str">
+        <v>Direktno brisanje računa i knjiženja</v>
+      </c>
+      <c r="D403" t="str">
+        <v>Kantica i modal; razlog i potvrda; uklanjanje samo povezanih stavki naloga</v>
+      </c>
+      <c r="E403" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F403" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G403" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H403" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I403" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J403" t="str">
+        <v>Izolovana DB regresija; TSC; lint</v>
+      </c>
+      <c r="K403" t="str">
+        <v>KUF; Nalozi; PDV</v>
+      </c>
+      <c r="L403" t="str">
+        <v>Veza kuf_entry_id; stare naloge ponovo knjižiti; zaključavanja i audit; purge usklađen.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA402"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA403"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Preskoci mailove bez podrzanih priloga bez upisa evidencije
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -2729,7 +2729,7 @@
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA403"/>
+  <dimension ref="A1:AA404"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -8140,9 +8140,47 @@
         <v>Veza kuf_entry_id; stare naloge ponovo knjižiti; zaključavanja i audit; purge usklađen.</v>
       </c>
     </row>
+    <row r="404">
+      <c r="A404" t="str">
+        <v>MAIL-NOISE-01</v>
+      </c>
+      <c r="B404" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="C404" t="str">
+        <v>Preskakanje logotipa bez evidencije</v>
+      </c>
+      <c r="D404" t="str">
+        <v>Mailovi bez podržanih priloga ne pune obradu ni pojedinačni audit</v>
+      </c>
+      <c r="E404" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F404" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G404" t="str">
+        <v>Nije potrebno</v>
+      </c>
+      <c r="H404" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I404" t="str">
+        <v>Bez migracije</v>
+      </c>
+      <c r="J404" t="str">
+        <v>Izolovana DB regresija</v>
+      </c>
+      <c r="K404" t="str">
+        <v>Mail import</v>
+      </c>
+      <c r="L404" t="str">
+        <v>Postojeći zapisi nijesu brisani.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA403"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA404"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Dodaj KUF filtere i ispravi MAPR import povrata i izvore dokumenata
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -5351,7 +5351,7 @@
         <v>F-062</v>
       </c>
       <c r="L329" t="str">
-        <v>KIF/KUF imaju mjesečne knjige, vrste, unos računa, PDV razradu, MAPR/SEP import, preuzimanje završenih kalkulacija, seme kontiranja, automatsko knjiženje, edit/delete neproknjiženih, print i Excel export. Kalkulacije su označene kao knjižene kroz izvorni dokument i ne ulaze ponovo u KUF nalog. Ostaju kontrole/XML/lock/testovi.</v>
+        <v>KUF pregled ima kombinovane filtere dobavljača/broja/konta/statusa/datuma/iznosa sa filtriranim zbirovima. KIF/KUF imaju mjesečne knjige, vrste, unos računa, PDV razradu, MAPR/SEP import, preuzimanje završenih kalkulacija, seme kontiranja, automatsko knjiženje, edit/delete neproknjiženih, print i Excel export. Kalkulacije su označene kao knjižene kroz izvorni dokument i ne ulaze ponovo u KUF nalog. Ostaju kontrole/XML/lock/testovi.</v>
       </c>
     </row>
     <row r="330">
@@ -5465,7 +5465,7 @@
         <v>F-063</v>
       </c>
       <c r="L332" t="str">
-        <v>KUF forma lokalno čita MAPR QR iz PDF/TIFF/JPG/PNG računa bez čuvanja originala, uz visoku PDF rezoluciju, zone, uvećavanje i kontrast. Import stranica prihvata više takvih fajlova, šalje grupe po pet uz stvarni progres i inkrementalne rezultate. KUF prije MAPR-a provjerava IIC+PIB+datum u lokalnoj bazi i preskače spoljašnji poziv za postojeće račune. Greške imaju izvještaj sa izvornim fajlom/linkom, grupni retry i CSV izvoz. Dobavljači bez zapamćenog KUF konta grupišu se po PIB-u; jedan izbor važi za sve njihove račune, ponovni import ih grupno kreira i pamti konto. Isti server-side MAPR čitač sada priprema i robnu kalkulaciju sa svim stavkama. KUF batch čuva serverski MAPR snapshot po firmi/godini i fiskalnom identitetu; izbor konta nastavlja iz baze bez novog MAPR poziva. Rollback DB test potvrđuje offline retry, prava/scope, duplikate i purge. Nakon uspješnog KUF upisa privremeni MAPR JSON se uklanja atomarno; greška ga zadržava. Migracija čisti istorijske duplikate, audit čuva samo broj; DB regresija potvrđuje životni ciklus i rollback.</v>
+        <v>KUF forma lokalno čita MAPR QR iz PDF/TIFF/JPG/PNG računa bez čuvanja originala, uz visoku PDF rezoluciju, zone, uvećavanje i kontrast. Import stranica prihvata više takvih fajlova, šalje grupe po pet uz stvarni progres i inkrementalne rezultate. KUF prije MAPR-a provjerava IIC+PIB+datum u lokalnoj bazi i preskače spoljašnji poziv za postojeće račune. Negativni MAPR računi koriste ukupnu vrijednost umjesto iznosa za plaćanje; stari negativni cache nastavlja offline iz poreskih redova. Greške prikazuju naziv dokumenta iz Excel reda ili hyperlinka; MAPR registraciono vrijeme može se razlikovati od kanonskog QR vremena uz provjeru IIC/PIB. Greške imaju izvještaj sa izvornim fajlom/linkom, grupni retry i CSV izvoz. Dobavljači bez zapamćenog KUF konta grupišu se po PIB-u; jedan izbor važi za sve njihove račune, ponovni import ih grupno kreira i pamti konto. Isti server-side MAPR čitač sada priprema i robnu kalkulaciju sa svim stavkama. KUF batch čuva serverski MAPR snapshot po firmi/godini i fiskalnom identitetu; izbor konta nastavlja iz baze bez novog MAPR poziva. Rollback DB test potvrđuje offline retry, prava/scope, duplikate i purge. Nakon uspješnog KUF upisa privremeni MAPR JSON se uklanja atomarno; greška ga zadržava. Migracija čisti istorijske duplikate, audit čuva samo broj; DB regresija potvrđuje životni ciklus i rollback.</v>
       </c>
     </row>
     <row r="333">

</xml_diff>

<commit_message>
Dodaj SEP automatiku, KIF/KUF dopune i korisnicke teme
Objedini pregled automatskih obrada, uskladi statuse sa nalozima i zakljucanim periodima, omoguci pretragu konta i potvrdu promjene radnog konteksta. Ukljuci migracije, regresione testove, dokumentaciju i planer.
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -437,7 +437,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -473,9 +473,144 @@
         <v>Korisnik potvrdio upload i Excel za septembar; bez Fiscal API-ja i automatskog KIF uvoza; JSON se ne čuva.</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>SEP podešavanja</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Ispravljeno</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Putanja u Podešavanjima i kompatibilni redirect; lokalni ključ podešen</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Linux produkcijski QA</v>
+      </c>
+      <c r="E3">
+        <v>46311.083333333336</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>KIF/KUF statusi</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Ispravljeno</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Prikaz prati status naloga; nacrt nije knjižen</v>
+      </c>
+      <c r="E4">
+        <v>46311.083333333336</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>KUF dopuna naloga</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Novi računi dopunjavaju isti POSTED nalog uz prava i zaključavanja</v>
+      </c>
+      <c r="E5">
+        <v>46311.083333333336</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>KIF dopuna i zaključan PDV</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Dopuna POSTED KIF naloga; KIF/KUF skrivaju dodavanje u zaključanom periodu</v>
+      </c>
+      <c r="E6">
+        <v>46311.083333333336</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Izbor konta</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Pretraga po šifri i nazivu u padajućim izborima svih modula; tastatura i miš</v>
+      </c>
+      <c r="E7">
+        <v>46311.083333333336</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>SEP automatika</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Opt-in po firmi; red u 04:00; IKOF prije MAPR; mjesečni KIF i POSTED nalog; Excel samo u memoriji</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Linux produkcijski živi SEP QA</v>
+      </c>
+      <c r="E8">
+        <v>46311.083333333336</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Organizacija automatike</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C9" t="str">
+        <v>SEP postavke u Podešavanja; Dashboard pregled SEP i izvoda sa filterima i ponavljanjem</v>
+      </c>
+      <c r="E9">
+        <v>46311.083333333336</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Potvrda radnog konteksta</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Modal prije promjene firme ili godine; potvrda ili odustajanje bez slučajne promjene</v>
+      </c>
+      <c r="E10">
+        <v>46311.083333333336</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Korisničke teme</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Pet paleta i svijetli/tamni režim; pamćenje po nalogu; semantičke boje svih modula; nezavisna štampa</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Dopunski browser QA ostalih uloga</v>
+      </c>
+      <c r="E11">
+        <v>46311.083333333336</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Dodaj povrat dobavljacu, dnevnik knjizenja i stampu pregleda
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -2711,7 +2711,7 @@
         <v>MVP 1/2</v>
       </c>
       <c r="H10" t="str">
-        <v>Meni i šifarnici su implementirani. Domaća kalkulacija ima MAPR unos, obračun, lager, DRAFT nalog i A4 štampu. Prenos robe, popis, otpis i nivelacija imaju nacrte, robne promete, poslovne jedinice, posebne šeme konta, DRAFT naloge i štampu; popis knjiži višak/manjak, otpis razdužuje zalihe, a nivelacija mijenja MP vrijednost, RUC i PDV bez količinske promjene. Lager lista i kartica artikla postoje u Robnom i centralnim Izvještajima. Slijede live QA, uvozna kalkulacija i povrati.</v>
+        <v>Implementirani šifarnici, domaća/MAPR kalkulacija, lager, izlazne fakture/POS, prenos, popis, otpis, nivelacija i domaći povrat dobavljaču. Povrat ima opcione izvorne veze, lager, POSTED nalog, negativan KUF/PDV, šemu/template, audit i štampu; DB rollback/purge provjereni. Postoje lager/kartica/vrijednost, brisanje kalkulacije i šeme po stopama. Otvoreni: uvoz i carinski povrat, zaseban povrat kupca, storno povrata dobavljaču, pregled razduženja, kontrole, ručna raspodjela troškova i završni live QA.</v>
       </c>
     </row>
     <row r="11">
@@ -2931,7 +2931,7 @@
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA405"/>
+  <dimension ref="A1:AA406"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4539,7 +4539,7 @@
         <v>F-036,F-027</v>
       </c>
       <c r="L45" t="str">
-        <v>Centralni izvještaji koriste četiri firm-specific konta iz Podešavanja i samo POSTED stavke; red vodi na karticu partnera. Ostaju štampa/export.</v>
+        <v>Centralni izvještaji koriste četiri firm-specific konta iz Podešavanja i samo POSTED stavke; red vodi na karticu partnera. Pregled Nalozi / Kupci-dobavljači ima A4 pejzažnu štampu sa istim kontom/datumima i zbirovima u centima; backend provjerava export pravo. Ostaju štampa centralnih izvještaja i dodatni export formati.</v>
       </c>
     </row>
     <row r="46">
@@ -4729,7 +4729,7 @@
         <v>F-039,F-041</v>
       </c>
       <c r="L308" t="str">
-        <v>Model stanja i ulazni promet iz domaće kalkulacije implementirani po firma+godina+magacin+artikal; pregled lagera tek slijedi.</v>
+        <v>Stanja i prometi po firmi, godini, magacinu i artiklu; postoje lager lista, kartica artikla i vrijednost zaliha. Domaća kalkulacija, prodaja, prenos, popis, otpis i nivelacija koriste ove evidencije.</v>
       </c>
     </row>
     <row r="309">
@@ -4787,13 +4787,13 @@
         <v>Vrlo visok</v>
       </c>
       <c r="F310" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Implementirano</v>
       </c>
       <c r="G310" t="str">
         <v>Da</v>
       </c>
       <c r="H310" t="str">
-        <v>Djelimicno</v>
+        <v>Da</v>
       </c>
       <c r="I310" t="str">
         <v>Da</v>
@@ -4805,7 +4805,7 @@
         <v>F-042</v>
       </c>
       <c r="L310" t="str">
-        <v>Ulaz iz kalkulacije ažurira ponderisanu prosječnu cijenu; razduženje po prosjeku slijedi sa izlaznim dokumentima.</v>
+        <v>Ulaz iz kalkulacije ažurira ponderisanu prosječnu cijenu; izlazne fakture, POS, prenos i otpis koriste prosječnu nabavnu cijenu. Ručni end-to-end QA postojećih tokova ostaje otvoren.</v>
       </c>
     </row>
     <row r="311">
@@ -4843,7 +4843,7 @@
         <v>F-041,F-042</v>
       </c>
       <c r="L311" t="str">
-        <v>Domaća kalkulacija ima nacrt, kompaktne stavke, brzo kreiranje artikla, MAPR pregled svih stavki sa povezivanjem ili atomarnim kreiranjem novih šifara i štampu. Pamti poslovnu jedinicu magacina, a završavanje je prenosi na DRAFT nalog CALCULATION i zadužuje lager; zatim čeka preuzimanje u KUF. Ostaje ručni end-to-end QA.</v>
+        <v>Domaća kalkulacija ima nacrt, kompaktne stavke, brzo kreiranje artikla, MAPR pregled svih stavki sa povezivanjem ili atomarnim kreiranjem novih šifara i štampu. Pamti poslovnu jedinicu magacina, a završavanje je prenosi na DRAFT nalog CALCULATION i zadužuje lager; zatim čeka preuzimanje u KUF. Ostaje ručni end-to-end QA. Izbor artikla podržava kucanje šifre/dijela naziva i tastaturu. Poslije dodavanja ostaje se kod unosa, a poslije izmjene/brisanja kod stavki. Brzi unos sada dodaje bez redirecta: Enter bira artikal i prolazi količinu/cijenu/rabat/prodajnu cijenu do potvrde; nakon upisa prazan artikal u fokusu, bez skoka na vrh. Dva stvarna browser upisa provjerena na uklonjenom QA nacrtu.</v>
       </c>
     </row>
     <row r="312">
@@ -5053,7 +5053,7 @@
         <v>Vrlo visok</v>
       </c>
       <c r="F317" t="str">
-        <v>Zaključeno</v>
+        <v>Nije implementirano</v>
       </c>
       <c r="G317" t="str">
         <v>Ne</v>
@@ -5071,7 +5071,7 @@
         <v>F-045</v>
       </c>
       <c r="L317" t="str">
-        <v>Ulazna PDV stopa stavki je 0%.</v>
+        <v>Robna stranica je placeholder. Potrebni su ino faktura i kurs, carinska deklaracija, raspodjela carine/troškova, carinski PDV i KUF veza. Postojeća KUF šema uvoza nije robni dokument.</v>
       </c>
     </row>
     <row r="318">
@@ -5091,25 +5091,25 @@
         <v>Vrlo visok</v>
       </c>
       <c r="F318" t="str">
-        <v>Zaključeno</v>
+        <v>Implementirano za domaći povrat</v>
       </c>
       <c r="G318" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="H318" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="I318" t="str">
         <v>Da</v>
       </c>
       <c r="J318" t="str">
-        <v>Ne</v>
+        <v>DB rollback + obračun + render</v>
       </c>
       <c r="K318" t="str">
         <v>F-042,F-045</v>
       </c>
       <c r="L318" t="str">
-        <v>Može biti slobodan ili povezan sa kalkulacijom.</v>
+        <v>Poseban nacrt/dokument, pozitivne količine, opcione veze na kalkulaciju/KUF/stavku; lager po prosjeku, MP/RUC/PDV, POSTED nalog i negativan SOURCE_DOCUMENT KUF bez dupliranja. Šema i template, prava/lock/audit u transakciji, štampa, idempotentnost, izvorne količine i stvarni purge test. Inostrani/carinski povrat i namjenski storno ostaju otvoreni. Izbor artikla podržava kucanje šifre/dijela naziva i tastaturu. Poslije dodavanja ostaje se kod unosa, a poslije izmjene/brisanja kod stavki.</v>
       </c>
     </row>
     <row r="319">
@@ -5129,25 +5129,25 @@
         <v>Vrlo visok</v>
       </c>
       <c r="F319" t="str">
-        <v>Zaključeno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G319" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="H319" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="I319" t="str">
         <v>Da</v>
       </c>
       <c r="J319" t="str">
-        <v>Ne</v>
+        <v>Djelimično</v>
       </c>
       <c r="K319" t="str">
         <v>F-042,F-044</v>
       </c>
       <c r="L319" t="str">
-        <v>Usluge ne razdužuju lager.</v>
+        <v>Izlazne fakture i POS razdužuju robu po prosječnoj nabavnoj cijeni uz kontrolu negativnog lagera; usluge ne mijenjaju lager. Samostalna stranica Razduženja lagera ostaje placeholder. Završni live QA ostaje otvoren.</v>
       </c>
     </row>
     <row r="320">
@@ -5451,7 +5451,7 @@
         <v>F-045,F-052,F-053,F-054,F-055,F-058,F-059</v>
       </c>
       <c r="L327" t="str">
-        <v>Domaća kalkulacija, prenos robe, popis sa razlikama, otpis i nivelacija kreiraju DRAFT naloge prema posebnim firm-specific šemama iz Robno / Podešavanja. KUF naknadno preuzima kalkulaciju bez ponovnog knjiženja. Povrati još nijesu implementirani.</v>
+        <v>Domaća kalkulacija, prenos, popis sa razlikama, otpis i nivelacija kreiraju DRAFT naloge; domaći povrat dobavljaču kreira POSTED nalog i negativan KUF u istoj transakciji. Izlazne fakture i odgovarajući POS tokovi knjiže prodaju/robu. KUF/KIF ne knjiže izvorne dokumente ponovo. Otvoreni su uvozna kalkulacija, inostrani povrat i zaseban povrat kupca; potpuni OFFICE/POS storno postoji.</v>
       </c>
     </row>
     <row r="328">
@@ -5527,7 +5527,7 @@
         <v>F-062</v>
       </c>
       <c r="L329" t="str">
-        <v>KUF pregled ima kombinovane filtere dobavljača/broja/konta/statusa/datuma/iznosa sa filtriranim zbirovima. KIF/KUF imaju mjesečne knjige, vrste, unos računa, PDV razradu, MAPR/SEP import, preuzimanje završenih kalkulacija, seme kontiranja, automatsko knjiženje, edit/delete neproknjiženih, print i Excel export. Kalkulacije su označene kao knjižene kroz izvorni dokument i ne ulaze ponovo u KUF nalog. Ostaju kontrole/XML/lock/testovi.</v>
+        <v>KUF pregled ima kombinovane filtere dobavljača/broja/konta/statusa/datuma/iznosa sa filtriranim zbirovima. KIF/KUF imaju mjesečne knjige, vrste, unos računa, PDV razradu, MAPR/SEP import, preuzimanje završenih kalkulacija, seme kontiranja, automatsko knjiženje, edit/delete neproknjiženih, print i Excel export. Kalkulacije su označene kao knjižene kroz izvorni dokument i ne ulaze ponovo u KUF nalog. Ostaju kontrole/XML/lock/testovi. Otvaranje novih KUF/KIF knjiga označava zaključane mjesece i kontrolisano blokira upis na backendu (uključujući posljednji dan); datum mora odgovarati mjesecu/godini. Rollback regresija provjerava obje akcije i render forme.</v>
       </c>
     </row>
     <row r="330">
@@ -8418,9 +8418,47 @@
         <v>Postojeći zapisi nijesu brisani.</v>
       </c>
     </row>
+    <row r="406">
+      <c r="A406" t="str">
+        <v>NAL-DNEVNIK</v>
+      </c>
+      <c r="B406" t="str">
+        <v>Nalozi za knjiženje</v>
+      </c>
+      <c r="C406" t="str">
+        <v>Dnevnik knjiženja</v>
+      </c>
+      <c r="D406" t="str">
+        <v>Sve proknjižene stavke hronološki po datumu naloga sa kontom, partnerom, dokumentom i iznosima.</v>
+      </c>
+      <c r="E406" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F406" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G406" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H406" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I406" t="str">
+        <v>Ne</v>
+      </c>
+      <c r="J406" t="str">
+        <v>Regresije; TSC; ESLint; browser</v>
+      </c>
+      <c r="K406" t="str">
+        <v>M-003</v>
+      </c>
+      <c r="L406" t="str">
+        <v>Kombinovani filteri svih kolona i perioda; 100 stavki po stranici; ukupni zbir filtriranog perioda u centima; A4 pejzažna štampa svih stavki; POSTED i tenant scope; view/export prava.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA405"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA406"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Implement advance invoices with fiscal settlement and accounting
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -2931,7 +2931,7 @@
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA406"/>
+  <dimension ref="A1:AA407"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -8456,9 +8456,47 @@
         <v>Kombinovani filteri svih kolona i perioda; 100 stavki po stranici; ukupni zbir filtriranog perioda u centima; A4 pejzažna štampa svih stavki; POSTED i tenant scope; view/export prava.</v>
       </c>
     </row>
+    <row r="407">
+      <c r="A407" t="str">
+        <v>FISCAL-ADVANCE</v>
+      </c>
+      <c r="B407" t="str">
+        <v>Fiskalizacija</v>
+      </c>
+      <c r="C407" t="str">
+        <v>Avansni računi i umanjenje</v>
+      </c>
+      <c r="D407" t="str">
+        <v>Avans, konačni račun sa vezom i negativno umanjenje u Robnom i direktnom portalu.</v>
+      </c>
+      <c r="E407" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F407" t="str">
+        <v>Implementirano djelimicno</v>
+      </c>
+      <c r="G407" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H407" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I407" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J407" t="str">
+        <v>TSC; lint; mock; DB rollback; browser</v>
+      </c>
+      <c r="K407" t="str">
+        <v>F-037</v>
+      </c>
+      <c r="L407" t="str">
+        <v>Fiskalni tok implementiran; odvojeni meni i pregled Avansni racuni u Robnom; unos preko dugmeta na pregledu; decimalni format kao obicni racuni; bez lagera za avans; sema avansnih konta po stopama i template povezana sa DRAFT nalozima i KIF SOURCE_DOCUMENT prenosom; umanjenje koristi snimak izvornih konta; odvojeni poreski mjeseci i nastavak bez novog slanja; storno-obnova sajta ostaje naredni; potreban deploy nove Fiscal API verzije.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA406"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA407"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add bulk payroll copying and controlled journal reopening
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -2931,7 +2931,7 @@
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA407"/>
+  <dimension ref="A1:AA408"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6667,7 +6667,7 @@
         <v>M-003,M-006,F-092</v>
       </c>
       <c r="L359" t="str">
-        <v>Provjeravaju se scope, pravo plate/post, zaključana godina, aktivna analitička konta, duple zbirne komponente i balans. Ponovno knjiženje je blokirano; opšte vraćanje automatskog naloga u nacrt nije dozvoljeno.</v>
+        <v>Provjeravaju se scope, pravo plate/post, zaključana godina, aktivna analitička konta, duple zbirne komponente i balans. Duplo knjiženje je blokirano. Vrati u nacrt atomski vraća nalog u DRAFT i obračun u CALCULATED; Proknjiži je ponovo dostupan uz isti nalog/broj. Backend prava oba modula; godina/PDV i zavisni mjesečni obračuni; audit rollback; realni paralelni zahtjevi i render dugmadi. Direktne izmjene/brisanje payroll naloga su blokirane.</v>
       </c>
     </row>
     <row r="360">
@@ -8494,9 +8494,47 @@
         <v>Fiskalni tok implementiran; odvojeni meni i pregled Avansni racuni u Robnom; unos preko dugmeta na pregledu; decimalni format kao obicni racuni; bez lagera za avans; sema avansnih konta po stopama i template povezana sa DRAFT nalozima i KIF SOURCE_DOCUMENT prenosom; umanjenje koristi snimak izvornih konta; odvojeni poreski mjeseci i nastavak bez novog slanja; storno-obnova sajta ostaje naredni; potreban deploy nove Fiscal API verzije.</v>
       </c>
     </row>
+    <row r="408">
+      <c r="A408" t="str">
+        <v>PAYROLL-COPY</v>
+      </c>
+      <c r="B408" t="str">
+        <v>Plate i zaposleni</v>
+      </c>
+      <c r="C408" t="str">
+        <v>Grupno kopiranje obračuna u drugi mjesec</v>
+      </c>
+      <c r="D408" t="str">
+        <v>Izvorni i ciljni mjesec; izbor firmi agencije; kopije odmah CALCULATED nezavisno od aktivne firme.</v>
+      </c>
+      <c r="E408" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F408" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G408" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H408" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I408" t="str">
+        <v>Nije potrebno</v>
+      </c>
+      <c r="J408" t="str">
+        <v>Unit; DB rollback; konkurentnost; lifecycle; browser</v>
+      </c>
+      <c r="K408" t="str">
+        <v>M-006</v>
+      </c>
+      <c r="L408" t="str">
+        <v>Preuzimaju se ulazi i fond sati; pomjeranje datuma i kraja mjeseca; važeće poreske stope; više izvora; scope/prava/verzije/periodi; bez duplikata; audit i rollback po firmi; knjiženje ostaje posebna akcija.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA407"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA408"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Store agency mail accounts encrypted in database
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -2931,7 +2931,7 @@
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA408"/>
+  <dimension ref="A1:AA409"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7576,10 +7576,10 @@
         <v>10/10; TLS i prijava potvrđeni</v>
       </c>
       <c r="K383" t="str">
-        <v>Serverski .env</v>
+        <v>Mail nalog u bazi</v>
       </c>
       <c r="L383" t="str">
-        <v>Admin povezane agencije; IMAP_AGENCY_ID; lozinka u .env</v>
+        <v>Admin agencije; sifrovana lozinka AES-256-GCM; MAIL_ENCRYPTION_KEY u env</v>
       </c>
     </row>
     <row r="384">
@@ -8532,9 +8532,47 @@
         <v>Preuzimaju se ulazi i fond sati; pomjeranje datuma i kraja mjeseca; važeće poreske stope; više izvora; scope/prava/verzije/periodi; bez duplikata; audit i rollback po firmi; knjiženje ostaje posebna akcija.</v>
       </c>
     </row>
+    <row r="409">
+      <c r="A409" t="str">
+        <v>M7-IMAP-06</v>
+      </c>
+      <c r="B409" t="str">
+        <v>Modul 7</v>
+      </c>
+      <c r="C409" t="str">
+        <v>Mail nalozi agencije u bazi</v>
+      </c>
+      <c r="D409" t="str">
+        <v>Vise naloga po agenciji i jedan izbor po firmi uz sifrovanu lozinku i prenos stare konfiguracije</v>
+      </c>
+      <c r="E409" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F409" t="str">
+        <v>Implementirano lokalno; ceka deploy</v>
+      </c>
+      <c r="G409" t="str">
+        <v>DA</v>
+      </c>
+      <c r="H409" t="str">
+        <v>DA</v>
+      </c>
+      <c r="I409" t="str">
+        <v>DA</v>
+      </c>
+      <c r="J409" t="str">
+        <v>TSC; lint; unit; DB rollback; live read-only</v>
+      </c>
+      <c r="K409" t="str">
+        <v>IMAP pregled i uvoz</v>
+      </c>
+      <c r="L409" t="str">
+        <v>Kompozitni tenant FK; bez tajni u UI i auditu; verzije; namespace istorije; opt-in automatike; idempotentan CLI; purge zadrzava agencijski nalog. Lokalno prenesene 3 firme i 39 obrada bez promjene pravila. Server nije mijenjan.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA408"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA409"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add VG and Summa fiscal report import into KIF pazar
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -2931,7 +2931,7 @@
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA409"/>
+  <dimension ref="A1:AA410"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5532,19 +5532,19 @@
     </row>
     <row r="330">
       <c r="A330" t="str">
-        <v>F-064</v>
+        <v>F-KIF-PAZAR-01</v>
       </c>
       <c r="B330" t="str">
-        <v>Računi / KIF-KUF</v>
+        <v>Računi / KIF</v>
       </c>
       <c r="C330" t="str">
-        <v>Dinamične vrste KIF/KUF knjiga</v>
+        <v>Uvoz fiskalnih izvještaja VG/Summa</v>
       </c>
       <c r="D330" t="str">
-        <v>Korisnik može otvoriti različite vrste KIF/KUF knjiga, npr. virmani, kartica, gotovina, avansi.</v>
+        <v>Uvoz periodičnog izvještaja u postojeću formu pazara i Excel download bez server arhive.</v>
       </c>
       <c r="E330" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F330" t="str">
         <v>Implementirano</v>
@@ -5559,27 +5559,27 @@
         <v>Da</v>
       </c>
       <c r="J330" t="str">
-        <v>Djelimicno</v>
+        <v>DB/SSR/live VG; browser QA ostaje</v>
       </c>
       <c r="K330" t="str">
         <v>F-063</v>
       </c>
       <c r="L330" t="str">
-        <v>Vrste se čuvaju u bazi i koriste za otvaranje knjige i izbor šeme.</v>
+        <v>KIF/KUF Podešavanja → Fiskalni portali: VG nalog šifrovan po firmi, Summa iz lokalnog POS-a. Uvezi izvještaj na postojećoj pazar formi bira kasu/period, čuva tačan PDV, popunjava formu i preuzima originalni VG ili generisani Summa Excel. Bez server fajlova, bez automatskog knjiženja. Potpis scope/verzije/izvora, locks, duplikati/preklapanje, audit, purge i paralelni uvoz provjereni. Samo POS računi i storna; OFFICE nije dio Summa izvještaja. Lokalna migracija 20261030090000; za deploy fiscal-portals:key + restart. Živa VG provjera, TSC/lint/npm test i izolovani DB testovi prošli; browser QA ostaje.</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="str">
-        <v>F-065</v>
+        <v>F-064</v>
       </c>
       <c r="B331" t="str">
         <v>Računi / KIF-KUF</v>
       </c>
       <c r="C331" t="str">
-        <v>Šema kontiranja po poljima</v>
+        <v>Dinamične vrste KIF/KUF knjiga</v>
       </c>
       <c r="D331" t="str">
-        <v>Za svako smisleno polje iznosa bira se D/P, izvor konta i konto; podržan konto iz unosa računa.</v>
+        <v>Korisnik može otvoriti različite vrste KIF/KUF knjiga, npr. virmani, kartica, gotovina, avansi.</v>
       </c>
       <c r="E331" t="str">
         <v>Vrlo visok</v>
@@ -5603,21 +5603,21 @@
         <v>F-063</v>
       </c>
       <c r="L331" t="str">
-        <v>Šema čuva pravila za ukupno, osnovice, PDV po stopama i oslobođeni promet. Pravila su odvojena po vrsti knjige; UI remount-uje redove po vrsti da se KIF/KUF šeme ne prelivaju. Podešavanja se mogu uvesti iz druge firme iste agencije. Ukupan iznos bira domaće ili ino konto prema is_foreign partnera; UKUPAN_IZNOS_INO je samo prateće pravilo bez drugog iznosa. Prazno ino konto blokira ino knjiženje; radi template i lokalni override/kopiranje. PDV tip je nezavisan; audit čuvanja atomski. TSC/lint/npm test; render; DB miješani KIF/KUF i dopuna/negativni računi; locks/scope/audit/purge; bez migracije.</v>
+        <v>Vrste se čuvaju u bazi i koriste za otvaranje knjige i izbor šeme.</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="str">
-        <v>F-066</v>
+        <v>F-065</v>
       </c>
       <c r="B332" t="str">
-        <v>Računi / KUF</v>
+        <v>Računi / KIF-KUF</v>
       </c>
       <c r="C332" t="str">
-        <v>MAPR unos i import linkova</v>
+        <v>Šema kontiranja po poljima</v>
       </c>
       <c r="D332" t="str">
-        <v>KUF i KIF mogu učitati fiskalne račune iz MAPR linka; import obrađuje više linkova u grupama.</v>
+        <v>Za svako smisleno polje iznosa bira se D/P, izvor konta i konto; podržan konto iz unosa računa.</v>
       </c>
       <c r="E332" t="str">
         <v>Vrlo visok</v>
@@ -5641,24 +5641,21 @@
         <v>F-063</v>
       </c>
       <c r="L332" t="str">
-        <v>KUF forma lokalno čita MAPR QR iz PDF/TIFF/JPG/PNG računa bez čuvanja originala, uz visoku PDF rezoluciju, zone, uvećavanje i kontrast. Import stranica prihvata više takvih fajlova, šalje grupe po pet uz stvarni progres i inkrementalne rezultate. KUF prije MAPR-a provjerava IIC+PIB+datum u lokalnoj bazi i preskače spoljašnji poziv za postojeće račune. Negativni MAPR računi koriste ukupnu vrijednost umjesto iznosa za plaćanje; stari negativni cache nastavlja offline iz poreskih redova. Greške prikazuju naziv dokumenta iz Excel reda ili hyperlinka; MAPR registraciono vrijeme može se razlikovati od kanonskog QR vremena uz provjeru IIC/PIB. Greške imaju izvještaj sa izvornim fajlom/linkom, grupni retry i CSV izvoz. Dobavljači bez zapamćenog KUF konta grupišu se po PIB-u; jedan izbor važi za sve njihove račune, ponovni import ih grupno kreira i pamti konto. Isti server-side MAPR čitač sada priprema i robnu kalkulaciju sa svim stavkama. KUF batch čuva serverski MAPR snapshot po firmi/godini i fiskalnom identitetu; izbor konta nastavlja iz baze bez novog MAPR poziva. Rollback DB test potvrđuje offline retry, prava/scope, duplikate i purge. Nakon uspješnog KUF upisa privremeni MAPR JSON se uklanja atomarno; greška ga zadržava. Migracija čisti istorijske duplikate, audit čuva samo broj; DB regresija potvrđuje životni ciklus i rollback.</v>
-      </c>
-      <c r="M332" t="str">
-        <v xml:space="preserve"> MAPR zahtjevi uklanjaju milisekunde datuma bez promjene fiskalnog identiteta; time je otklonjen HTTP 404 u SEP automatici. Greške prikazuju HTTP status; potvrđen živi read-only račun i rollback MAPR/SEP regresije. Lokalni dev restartovan zbog stare instrumentation funkcije; oba računa iz SEP greške potvrđena read-only.</v>
+        <v>Šema čuva pravila za ukupno, osnovice, PDV po stopama i oslobođeni promet. Pravila su odvojena po vrsti knjige; UI remount-uje redove po vrsti da se KIF/KUF šeme ne prelivaju. Podešavanja se mogu uvesti iz druge firme iste agencije. Ukupan iznos bira domaće ili ino konto prema is_foreign partnera; UKUPAN_IZNOS_INO je samo prateće pravilo bez drugog iznosa. Prazno ino konto blokira ino knjiženje; radi template i lokalni override/kopiranje. PDV tip je nezavisan; audit čuvanja atomski. TSC/lint/npm test; render; DB miješani KIF/KUF i dopuna/negativni računi; locks/scope/audit/purge; bez migracije.</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="str">
-        <v>F-067</v>
+        <v>F-066</v>
       </c>
       <c r="B333" t="str">
-        <v>Računi / KIF</v>
+        <v>Računi / KUF</v>
       </c>
       <c r="C333" t="str">
-        <v>SEP Excel import za KIF</v>
+        <v>MAPR unos i import linkova</v>
       </c>
       <c r="D333" t="str">
-        <v>SEP Excel se parsira u MAPR linkove i koristi za import izlaznih računa u KIF.</v>
+        <v>KUF i KIF mogu učitati fiskalne račune iz MAPR linka; import obrađuje više linkova u grupama.</v>
       </c>
       <c r="E333" t="str">
         <v>Vrlo visok</v>
@@ -5679,24 +5676,27 @@
         <v>Djelimicno</v>
       </c>
       <c r="K333" t="str">
-        <v>F-066</v>
+        <v>F-063</v>
       </c>
       <c r="L333" t="str">
-        <v>Provjereno sa testnim SEP fajlom; treba dodatna validacija edge case-ova.</v>
+        <v>KUF forma lokalno čita MAPR QR iz PDF/TIFF/JPG/PNG računa bez čuvanja originala, uz visoku PDF rezoluciju, zone, uvećavanje i kontrast. Import stranica prihvata više takvih fajlova, šalje grupe po pet uz stvarni progres i inkrementalne rezultate. KUF prije MAPR-a provjerava IIC+PIB+datum u lokalnoj bazi i preskače spoljašnji poziv za postojeće račune. Negativni MAPR računi koriste ukupnu vrijednost umjesto iznosa za plaćanje; stari negativni cache nastavlja offline iz poreskih redova. Greške prikazuju naziv dokumenta iz Excel reda ili hyperlinka; MAPR registraciono vrijeme može se razlikovati od kanonskog QR vremena uz provjeru IIC/PIB. Greške imaju izvještaj sa izvornim fajlom/linkom, grupni retry i CSV izvoz. Dobavljači bez zapamćenog KUF konta grupišu se po PIB-u; jedan izbor važi za sve njihove račune, ponovni import ih grupno kreira i pamti konto. Isti server-side MAPR čitač sada priprema i robnu kalkulaciju sa svim stavkama. KUF batch čuva serverski MAPR snapshot po firmi/godini i fiskalnom identitetu; izbor konta nastavlja iz baze bez novog MAPR poziva. Rollback DB test potvrđuje offline retry, prava/scope, duplikate i purge. Nakon uspješnog KUF upisa privremeni MAPR JSON se uklanja atomarno; greška ga zadržava. Migracija čisti istorijske duplikate, audit čuva samo broj; DB regresija potvrđuje životni ciklus i rollback.</v>
+      </c>
+      <c r="M333" t="str">
+        <v xml:space="preserve"> MAPR zahtjevi uklanjaju milisekunde datuma bez promjene fiskalnog identiteta; time je otklonjen HTTP 404 u SEP automatici. Greške prikazuju HTTP status; potvrđen živi read-only račun i rollback MAPR/SEP regresije. Lokalni dev restartovan zbog stare instrumentation funkcije; oba računa iz SEP greške potvrđena read-only.</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="str">
-        <v>F-068</v>
+        <v>F-067</v>
       </c>
       <c r="B334" t="str">
-        <v>Računi / KIF-KUF</v>
+        <v>Računi / KIF</v>
       </c>
       <c r="C334" t="str">
-        <v>Automatsko knjiženje knjige</v>
+        <v>SEP Excel import za KIF</v>
       </c>
       <c r="D334" t="str">
-        <v>Cijeli KIF/KUF se knjiži u jedan nalog po šemi, a naknadno dodati računi se dopunjavaju na isti nalog.</v>
+        <v>SEP Excel se parsira u MAPR linkove i koristi za import izlaznih računa u KIF.</v>
       </c>
       <c r="E334" t="str">
         <v>Vrlo visok</v>
@@ -5717,27 +5717,27 @@
         <v>Djelimicno</v>
       </c>
       <c r="K334" t="str">
-        <v>F-065</v>
+        <v>F-066</v>
       </c>
       <c r="L334" t="str">
-        <v>Status knjige prikazuje otvorena/djelimično knjižena/knjižena i ima link na nalog.</v>
+        <v>Provjereno sa testnim SEP fajlom; treba dodatna validacija edge case-ova.</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="str">
-        <v>F-069</v>
+        <v>F-068</v>
       </c>
       <c r="B335" t="str">
         <v>Računi / KIF-KUF</v>
       </c>
       <c r="C335" t="str">
-        <v>Štampa KIF/KUF knjige</v>
+        <v>Automatsko knjiženje knjige</v>
       </c>
       <c r="D335" t="str">
-        <v>Pregled KIF/KUF ima print varijantu bez menija, po periodu datuma knjige.</v>
+        <v>Cijeli KIF/KUF se knjiži u jedan nalog po šemi, a naknadno dodati računi se dopunjavaju na isti nalog.</v>
       </c>
       <c r="E335" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F335" t="str">
         <v>Implementirano</v>
@@ -5755,30 +5755,30 @@
         <v>Djelimicno</v>
       </c>
       <c r="K335" t="str">
-        <v>F-063</v>
+        <v>F-065</v>
       </c>
       <c r="L335" t="str">
-        <v>Format liči na službene obrasce; treba još fino podešavanje kolona za veće brojeve.</v>
+        <v>Status knjige prikazuje otvorena/djelimično knjižena/knjižena i ima link na nalog.</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="str">
-        <v>F-070</v>
+        <v>F-069</v>
       </c>
       <c r="B336" t="str">
         <v>Računi / KIF-KUF</v>
       </c>
       <c r="C336" t="str">
-        <v>Izmjena i brisanje računa</v>
+        <v>Štampa KIF/KUF knjige</v>
       </c>
       <c r="D336" t="str">
-        <v>Neproknjiženi računi u KIF/KUF se mogu mijenjati ili brisati.</v>
+        <v>Pregled KIF/KUF ima print varijantu bez menija, po periodu datuma knjige.</v>
       </c>
       <c r="E336" t="str">
         <v>Visok</v>
       </c>
       <c r="F336" t="str">
-        <v>Implementirano djelimicno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G336" t="str">
         <v>Da</v>
@@ -5796,27 +5796,27 @@
         <v>F-063</v>
       </c>
       <c r="L336" t="str">
-        <v>Za proknjižene račune ostaje definisati stroga pravila korekcije/storna.</v>
+        <v>Format liči na službene obrasce; treba još fino podešavanje kolona za veće brojeve.</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="str">
-        <v>F-071</v>
+        <v>F-070</v>
       </c>
       <c r="B337" t="str">
         <v>Računi / KIF-KUF</v>
       </c>
       <c r="C337" t="str">
-        <v>Excel export KIF/KUF pregleda</v>
+        <v>Izmjena i brisanje računa</v>
       </c>
       <c r="D337" t="str">
-        <v>KIF/KUF pregledi se izvoze u XLSX po aktivnoj firmi, poslovnoj godini i filteru datuma knjige.</v>
+        <v>Neproknjiženi računi u KIF/KUF se mogu mijenjati ili brisati.</v>
       </c>
       <c r="E337" t="str">
         <v>Visok</v>
       </c>
       <c r="F337" t="str">
-        <v>Implementirano</v>
+        <v>Implementirano djelimicno</v>
       </c>
       <c r="G337" t="str">
         <v>Da</v>
@@ -5834,24 +5834,24 @@
         <v>F-063</v>
       </c>
       <c r="L337" t="str">
-        <v>Export uključuje partnera, tip prometa, iznose, status knjiženja i PDV razradu; backend provjerava export pravo.</v>
+        <v>Za proknjižene račune ostaje definisati stroga pravila korekcije/storna.</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="str">
-        <v>F-072</v>
+        <v>F-071</v>
       </c>
       <c r="B338" t="str">
-        <v>PDV</v>
+        <v>Računi / KIF-KUF</v>
       </c>
       <c r="C338" t="str">
-        <v>PDV periodi po mjesecu</v>
+        <v>Excel export KIF/KUF pregleda</v>
       </c>
       <c r="D338" t="str">
-        <v>PDV periodi se vode za aktivnu firmu i poslovnu godinu; na PDV ekranima bira se samo mjesec.</v>
+        <v>KIF/KUF pregledi se izvoze u XLSX po aktivnoj firmi, poslovnoj godini i filteru datuma knjige.</v>
       </c>
       <c r="E338" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F338" t="str">
         <v>Implementirano</v>
@@ -5872,21 +5872,21 @@
         <v>F-063</v>
       </c>
       <c r="L338" t="str">
-        <v>Period KIF/KUF računa određuje datum knjige: kif_date odnosno kuf_date.</v>
+        <v>Export uključuje partnera, tip prometa, iznose, status knjiženja i PDV razradu; backend provjerava export pravo.</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="str">
-        <v>F-073</v>
+        <v>F-072</v>
       </c>
       <c r="B339" t="str">
         <v>PDV</v>
       </c>
       <c r="C339" t="str">
-        <v>Ulazni i izlazni PDV evidencije</v>
+        <v>PDV periodi po mjesecu</v>
       </c>
       <c r="D339" t="str">
-        <v>Ulazni PDV prikazuje KUF račune, a izlazni PDV KIF račune koji ulaze u izabrani mjesec.</v>
+        <v>PDV periodi se vode za aktivnu firmu i poslovnu godinu; na PDV ekranima bira se samo mjesec.</v>
       </c>
       <c r="E339" t="str">
         <v>Vrlo visok</v>
@@ -5907,30 +5907,30 @@
         <v>Djelimicno</v>
       </c>
       <c r="K339" t="str">
-        <v>F-063,F-072</v>
+        <v>F-063</v>
       </c>
       <c r="L339" t="str">
-        <v>Evidencije su dokazni pregled iza prijave i linkuju na KIF/KUF knjige.</v>
+        <v>Period KIF/KUF računa određuje datum knjige: kif_date odnosno kuf_date.</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="str">
-        <v>F-074</v>
+        <v>F-073</v>
       </c>
       <c r="B340" t="str">
         <v>PDV</v>
       </c>
       <c r="C340" t="str">
-        <v>PDV prijava po IRMS obrascu</v>
+        <v>Ulazni i izlazni PDV evidencije</v>
       </c>
       <c r="D340" t="str">
-        <v>Prijava se automatski puni iz KIF/KUF, ima redove obrasca i automatske preračune PDV-a i zbirnih redova.</v>
+        <v>Ulazni PDV prikazuje KUF račune, a izlazni PDV KIF račune koji ulaze u izabrani mjesec.</v>
       </c>
       <c r="E340" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F340" t="str">
-        <v>Implementirano djelimicno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G340" t="str">
         <v>Da</v>
@@ -5945,30 +5945,30 @@
         <v>Djelimicno</v>
       </c>
       <c r="K340" t="str">
-        <v>F-072,F-073</v>
+        <v>F-063,F-072</v>
       </c>
       <c r="L340" t="str">
-        <v>Dodat nacrt prijave, osvježavanje iz KIF/KUF, portal layout, XML export u PR_PDV_2025 formatu i osnovno zbirno knjiženje; brisanje PDV naloga vraća prijavu u nacrt. Zaključavanje i kontrolisano otključavanje sa verzijama i DB regresijom završeni; ostaje ručni QA XML upload-a.</v>
+        <v>Evidencije su dokazni pregled iza prijave i linkuju na KIF/KUF knjige.</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="str">
-        <v>F-075</v>
+        <v>F-074</v>
       </c>
       <c r="B341" t="str">
         <v>PDV</v>
       </c>
       <c r="C341" t="str">
-        <v>Podešavanja knjiženja PDV prijave</v>
+        <v>PDV prijava po IRMS obrascu</v>
       </c>
       <c r="D341" t="str">
-        <v>Firma za aktivnu godinu bira vrstu naloga i šemu D/P + konto za zatvaranje kartica PDV-a.</v>
+        <v>Prijava se automatski puni iz KIF/KUF, ima redove obrasca i automatske preračune PDV-a i zbirnih redova.</v>
       </c>
       <c r="E341" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F341" t="str">
-        <v>Implementirano</v>
+        <v>Implementirano djelimicno</v>
       </c>
       <c r="G341" t="str">
         <v>Da</v>
@@ -5983,62 +5983,62 @@
         <v>Djelimicno</v>
       </c>
       <c r="K341" t="str">
-        <v>F-074</v>
+        <v>F-072,F-073</v>
       </c>
       <c r="L341" t="str">
-        <v>Pravila se generišu po aktivnim PDV stopama iz baze za ulazni/izlazni PDV, plus carinski, paušalni, obaveza i kredit. Dropdown konta prikazuje cijeli spojeni kontni plan; izbor globalnog konta se pri čuvanju veže kao firmi konto. Kontrole porede PDV evidenciju sa glavnom knjigom.</v>
+        <v>Dodat nacrt prijave, osvježavanje iz KIF/KUF, portal layout, XML export u PR_PDV_2025 formatu i osnovno zbirno knjiženje; brisanje PDV naloga vraća prijavu u nacrt. Zaključavanje i kontrolisano otključavanje sa verzijama i DB regresijom završeni; ostaje ručni QA XML upload-a.</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="str">
-        <v>F-076</v>
+        <v>F-075</v>
       </c>
       <c r="B342" t="str">
-        <v>Izvodi</v>
+        <v>PDV</v>
       </c>
       <c r="C342" t="str">
-        <v>Import sesija PDF/HTML izvoda</v>
+        <v>Podešavanja knjiženja PDV prijave</v>
       </c>
       <c r="D342" t="str">
-        <v>Korisnik učitava PDF/HTML/XML izvod za aktivnu firmu/godinu i bankovni račun; sistem čuva fajl, raw text i status importa.</v>
+        <v>Firma za aktivnu godinu bira vrstu naloga i šemu D/P + konto za zatvaranje kartica PDV-a.</v>
       </c>
       <c r="E342" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F342" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Implementirano</v>
       </c>
       <c r="G342" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="H342" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="I342" t="str">
         <v>Da</v>
       </c>
       <c r="J342" t="str">
-        <v>Ne</v>
+        <v>Djelimicno</v>
       </c>
       <c r="K342" t="str">
-        <v>M-005,F-017</v>
+        <v>F-074</v>
       </c>
       <c r="L342" t="str">
-        <v>Postoji upload/paste tekst i čuvanje izvoda; podržani su NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF, a puna import sesija ostaje za kasnije.</v>
+        <v>Pravila se generišu po aktivnim PDV stopama iz baze za ulazni/izlazni PDV, plus carinski, paušalni, obaveza i kredit. Dropdown konta prikazuje cijeli spojeni kontni plan; izbor globalnog konta se pri čuvanju veže kao firmi konto. Kontrole porede PDV evidenciju sa glavnom knjigom.</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="str">
-        <v>F-077</v>
+        <v>F-076</v>
       </c>
       <c r="B343" t="str">
         <v>Izvodi</v>
       </c>
       <c r="C343" t="str">
-        <v>Parsiranje izvoda</v>
+        <v>Import sesija PDF/HTML izvoda</v>
       </c>
       <c r="D343" t="str">
-        <v>Parser čita zaglavlje i stavke, a arhitektura dozvoljava parsere po bankama.</v>
+        <v>Korisnik učitava PDF/HTML/XML izvod za aktivnu firmu/godinu i bankovni račun; sistem čuva fajl, raw text i status importa.</v>
       </c>
       <c r="E343" t="str">
         <v>Vrlo visok</v>
@@ -6059,24 +6059,24 @@
         <v>Ne</v>
       </c>
       <c r="K343" t="str">
-        <v>F-076</v>
+        <v>M-005,F-017</v>
       </c>
       <c r="L343" t="str">
-        <v>Implementirani NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF parseri; CKB ukupni priliv/odliv uzima iz zaglavlja PDF izvoda; Hipotekarna i Lovćen podržavaju kartične stavke bez žiro računa; fallback tekstualni format ostaje aktivan.</v>
+        <v>Postoji upload/paste tekst i čuvanje izvoda; podržani su NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF, a puna import sesija ostaje za kasnije.</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="str">
-        <v>F-078</v>
+        <v>F-077</v>
       </c>
       <c r="B344" t="str">
         <v>Izvodi</v>
       </c>
       <c r="C344" t="str">
-        <v>Preview parsiranja</v>
+        <v>Parsiranje izvoda</v>
       </c>
       <c r="D344" t="str">
-        <v>Korisnik vidi zaglavlje, stavke, greške, kontrolu početnog/krajnjeg stanja i može ispraviti podatke prije povezivanja.</v>
+        <v>Parser čita zaglavlje i stavke, a arhitektura dozvoljava parsere po bankama.</v>
       </c>
       <c r="E344" t="str">
         <v>Vrlo visok</v>
@@ -6097,24 +6097,24 @@
         <v>Ne</v>
       </c>
       <c r="K344" t="str">
-        <v>F-077</v>
+        <v>F-076</v>
       </c>
       <c r="L344" t="str">
-        <v>Postoji tab Stavke izvoda i kontrola stanja; korekcije iznosa/datuma ostaju za doradu.</v>
+        <v>Implementirani NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF parseri; CKB ukupni priliv/odliv uzima iz zaglavlja PDF izvoda; Hipotekarna i Lovćen podržavaju kartične stavke bez žiro računa; fallback tekstualni format ostaje aktivan.</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="str">
-        <v>F-079</v>
+        <v>F-078</v>
       </c>
       <c r="B345" t="str">
         <v>Izvodi</v>
       </c>
       <c r="C345" t="str">
-        <v>Prepoznavanje komitenta po žiro računu</v>
+        <v>Preview parsiranja</v>
       </c>
       <c r="D345" t="str">
-        <v>Komitent se primarno prepoznaje po normalizovanom žiro računu; naziv iz banke je samo pomoćni signal.</v>
+        <v>Korisnik vidi zaglavlje, stavke, greške, kontrolu početnog/krajnjeg stanja i može ispraviti podatke prije povezivanja.</v>
       </c>
       <c r="E345" t="str">
         <v>Vrlo visok</v>
@@ -6135,24 +6135,24 @@
         <v>Ne</v>
       </c>
       <c r="K345" t="str">
-        <v>F-078</v>
+        <v>F-077</v>
       </c>
       <c r="L345" t="str">
-        <v>Automatski predlog po partner_bank_accounts i komitent_ziro_racuni postoji; ručno povezivanje partnera na stavci izvoda pamti račun kao agencijski zajednički račun kad je moguće.</v>
+        <v>Postoji tab Stavke izvoda i kontrola stanja; korekcije iznosa/datuma ostaju za doradu.</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="str">
-        <v>F-080</v>
+        <v>F-079</v>
       </c>
       <c r="B346" t="str">
         <v>Izvodi</v>
       </c>
       <c r="C346" t="str">
-        <v>Povezivanje sa KIF/KUF fakturama</v>
+        <v>Prepoznavanje komitenta po žiro računu</v>
       </c>
       <c r="D346" t="str">
-        <v>Stavka izvoda može zatvoriti jednu ili više KIF/KUF faktura; jedna faktura može biti plaćena kroz više uplata.</v>
+        <v>Komitent se primarno prepoznaje po normalizovanom žiro računu; naziv iz banke je samo pomoćni signal.</v>
       </c>
       <c r="E346" t="str">
         <v>Vrlo visok</v>
@@ -6161,36 +6161,36 @@
         <v>Djelimično implementirano</v>
       </c>
       <c r="G346" t="str">
-        <v>Da</v>
+        <v>Ne</v>
       </c>
       <c r="H346" t="str">
-        <v>Da</v>
+        <v>Ne</v>
       </c>
       <c r="I346" t="str">
         <v>Da</v>
       </c>
       <c r="J346" t="str">
-        <v>Djelimicno</v>
+        <v>Ne</v>
       </c>
       <c r="K346" t="str">
-        <v>F-063,F-079</v>
+        <v>F-078</v>
       </c>
       <c r="L346" t="str">
-        <v>Osnovna alokacija jedne stavke izvoda na jedan otvoreni KIF/KUF račun je implementirana kroz bank_statement_line_allocations; status plaćanja se osvježava na UNPAID/PARTIALLY_PAID/PAID/OVERPAID. Split jedne uplate na više računa ostaje dorada.</v>
+        <v>Automatski predlog po partner_bank_accounts i komitent_ziro_racuni postoji; ručno povezivanje partnera na stavci izvoda pamti račun kao agencijski zajednički račun kad je moguće.</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="str">
-        <v>F-081</v>
+        <v>F-080</v>
       </c>
       <c r="B347" t="str">
         <v>Izvodi</v>
       </c>
       <c r="C347" t="str">
-        <v>Ručno kontiranje stavke</v>
+        <v>Povezivanje sa KIF/KUF fakturama</v>
       </c>
       <c r="D347" t="str">
-        <v>Stavke koje nisu kupci/dobavljači mogu se ručno kontirati kroz konto duguje, konto potražuje, partner po potrebi i opis.</v>
+        <v>Stavka izvoda može zatvoriti jednu ili više KIF/KUF faktura; jedna faktura može biti plaćena kroz više uplata.</v>
       </c>
       <c r="E347" t="str">
         <v>Vrlo visok</v>
@@ -6199,39 +6199,39 @@
         <v>Djelimično implementirano</v>
       </c>
       <c r="G347" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="H347" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="I347" t="str">
         <v>Da</v>
       </c>
       <c r="J347" t="str">
-        <v>Ne</v>
+        <v>Djelimicno</v>
       </c>
       <c r="K347" t="str">
-        <v>F-078</v>
+        <v>F-063,F-079</v>
       </c>
       <c r="L347" t="str">
-        <v>Tab Predlog naloga omogućava izbor partnera i duguje/potražuje konta; izbor konta ide preko šifre i automatskog firma_konta linka; interni prenosi između sopstvenih računa firme se prepoznaju po kontra računu.</v>
+        <v>Osnovna alokacija jedne stavke izvoda na jedan otvoreni KIF/KUF račun je implementirana kroz bank_statement_line_allocations; status plaćanja se osvježava na UNPAID/PARTIALLY_PAID/PAID/OVERPAID. Split jedne uplate na više računa ostaje dorada.</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="str">
-        <v>F-082</v>
+        <v>F-081</v>
       </c>
       <c r="B348" t="str">
         <v>Izvodi</v>
       </c>
       <c r="C348" t="str">
-        <v>Pravila knjiženja i učenje</v>
+        <v>Ručno kontiranje stavke</v>
       </c>
       <c r="D348" t="str">
-        <v>Korisnik može ručno riješenu stavku zapamtiti kao pravilo knjiženja; pravila imaju match uslove, priority, auto_apply i requires_review.</v>
+        <v>Stavke koje nisu kupci/dobavljači mogu se ručno kontirati kroz konto duguje, konto potražuje, partner po potrebi i opis.</v>
       </c>
       <c r="E348" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F348" t="str">
         <v>Djelimično implementirano</v>
@@ -6249,30 +6249,30 @@
         <v>Ne</v>
       </c>
       <c r="K348" t="str">
-        <v>F-081</v>
+        <v>F-078</v>
       </c>
       <c r="L348" t="str">
-        <v>Pravila podržavaju smjer, žiro račun, opis, šifru plaćanja, poziv na broj, prioritet, zajednički scope agencije i firm-specific override; account_code omogućava primjenu kroz firme. Automatsko učenje po poznatom žiro računu čuva jedno fallback pravilo po računu i smjeru bez rednog broja, opisa i šifre plaćanja. Lovćen M02 stavke bez kontra računa uče samo uslov po šifri i smjeru, bez naziva prodavnice i partnera. Neproknjižen izvod može ručno ponovo primijeniti pravila bez prepisivanja ručnog konta, a preview prikazuje konkretne razloge blokade. Regresioni testovi pokrivaju M02, fallback, firm-specific prioritet i analitičko konto.</v>
+        <v>Tab Predlog naloga omogućava izbor partnera i duguje/potražuje konta; izbor konta ide preko šifre i automatskog firma_konta linka; interni prenosi između sopstvenih računa firme se prepoznaju po kontra računu.</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="str">
-        <v>F-083</v>
+        <v>F-082</v>
       </c>
       <c r="B349" t="str">
         <v>Izvodi</v>
       </c>
       <c r="C349" t="str">
-        <v>Confidence score i grupna potvrda</v>
+        <v>Pravila knjiženja i učenje</v>
       </c>
       <c r="D349" t="str">
-        <v>Sistem boduje predloge po računu, fakturi, iznosu i nazivu; grupno se mogu potvrditi samo sigurne READY stavke.</v>
+        <v>Korisnik može ručno riješenu stavku zapamtiti kao pravilo knjiženja; pravila imaju match uslove, priority, auto_apply i requires_review.</v>
       </c>
       <c r="E349" t="str">
         <v>Visok</v>
       </c>
       <c r="F349" t="str">
-        <v>Specifikacija spremna</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="G349" t="str">
         <v>Ne</v>
@@ -6287,30 +6287,30 @@
         <v>Ne</v>
       </c>
       <c r="K349" t="str">
-        <v>F-079,F-080,F-082</v>
+        <v>F-081</v>
       </c>
       <c r="L349" t="str">
-        <v>Predlog: &gt;=90 za grupnu potvrdu.</v>
+        <v>Pravila podržavaju smjer, žiro račun, opis, šifru plaćanja, poziv na broj, prioritet, zajednički scope agencije i firm-specific override; account_code omogućava primjenu kroz firme. Automatsko učenje po poznatom žiro računu čuva jedno fallback pravilo po računu i smjeru bez rednog broja, opisa i šifre plaćanja. Lovćen M02 stavke bez kontra računa uče samo uslov po šifri i smjeru, bez naziva prodavnice i partnera. Neproknjižen izvod može ručno ponovo primijeniti pravila bez prepisivanja ručnog konta, a preview prikazuje konkretne razloge blokade. Regresioni testovi pokrivaju M02, fallback, firm-specific prioritet i analitičko konto.</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="str">
-        <v>F-084</v>
+        <v>F-083</v>
       </c>
       <c r="B350" t="str">
         <v>Izvodi</v>
       </c>
       <c r="C350" t="str">
-        <v>Preview i knjiženje naloga</v>
+        <v>Confidence score i grupna potvrda</v>
       </c>
       <c r="D350" t="str">
-        <v>Kada su sve stavke READY ili IGNORED, sistem prikazuje preview naloga i knjiži jedan izvod u jedan nalog.</v>
+        <v>Sistem boduje predloge po računu, fakturi, iznosu i nazivu; grupno se mogu potvrditi samo sigurne READY stavke.</v>
       </c>
       <c r="E350" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F350" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Specifikacija spremna</v>
       </c>
       <c r="G350" t="str">
         <v>Ne</v>
@@ -6325,30 +6325,30 @@
         <v>Ne</v>
       </c>
       <c r="K350" t="str">
-        <v>F-078,F-080,F-081</v>
+        <v>F-079,F-080,F-082</v>
       </c>
       <c r="L350" t="str">
-        <v>Postoji preview i knjiženje READY izvoda u poseban proknjižen IZV nalog; banka se knjiži zbirno po ukupnom prilivu/odlivu, pojedinačne stavke idu samo na kontra konta; preview sada omogućava osnovno zatvaranje KIF/KUF računa.</v>
+        <v>Predlog: &gt;=90 za grupnu potvrdu.</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="str">
-        <v>F-085</v>
+        <v>F-084</v>
       </c>
       <c r="B351" t="str">
         <v>Izvodi</v>
       </c>
       <c r="C351" t="str">
-        <v>Vraćanje izvoda u nacrt</v>
+        <v>Preview i knjiženje naloga</v>
       </c>
       <c r="D351" t="str">
-        <v>Proknjižen izvod se ne mijenja direktno; vraćanje u nacrt poništava ili označava povezani nalog i efekat zatvaranja faktura.</v>
+        <v>Kada su sve stavke READY ili IGNORED, sistem prikazuje preview naloga i knjiži jedan izvod u jedan nalog.</v>
       </c>
       <c r="E351" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F351" t="str">
-        <v>Specifikacija spremna</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="G351" t="str">
         <v>Ne</v>
@@ -6363,62 +6363,62 @@
         <v>Ne</v>
       </c>
       <c r="K351" t="str">
-        <v>F-084</v>
+        <v>F-078,F-080,F-081</v>
       </c>
       <c r="L351" t="str">
-        <v>Provjeriti prava, zaključanu godinu i upisati audit log.</v>
+        <v>Postoji preview i knjiženje READY izvoda u poseban proknjižen IZV nalog; banka se knjiži zbirno po ukupnom prilivu/odlivu, pojedinačne stavke idu samo na kontra konta; preview sada omogućava osnovno zatvaranje KIF/KUF računa.</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="str">
-        <v>F-086</v>
+        <v>F-085</v>
       </c>
       <c r="B352" t="str">
-        <v>Zavrsni racun</v>
+        <v>Izvodi</v>
       </c>
       <c r="C352" t="str">
-        <v>Bilans uspjeha</v>
+        <v>Vraćanje izvoda u nacrt</v>
       </c>
       <c r="D352" t="str">
-        <v>Bilans uspjeha se racuna iz POSTED naloga po podesivoj semi pozicija, prikazuje tekucu i prethodnu godinu i stampa formalni obrazac.</v>
+        <v>Proknjižen izvod se ne mijenja direktno; vraćanje u nacrt poništava ili označava povezani nalog i efekat zatvaranja faktura.</v>
       </c>
       <c r="E352" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F352" t="str">
-        <v>Djelimicno implementirano</v>
+        <v>Specifikacija spremna</v>
       </c>
       <c r="G352" t="str">
-        <v>Da</v>
+        <v>Ne</v>
       </c>
       <c r="H352" t="str">
-        <v>Da</v>
+        <v>Ne</v>
       </c>
       <c r="I352" t="str">
         <v>Da</v>
       </c>
       <c r="J352" t="str">
-        <v>Djelimicno</v>
+        <v>Ne</v>
       </c>
       <c r="K352" t="str">
-        <v>M-003,M-008,F-038</v>
+        <v>F-084</v>
       </c>
       <c r="L352" t="str">
-        <v>Sistemska sema je seedovana u finansijski_izvjestaj_sabloni/pozicije; firma moze izmijeniti konta, izuzetke i formule kroz podesavanja. Trajne rucne korekcije po AOP/koloni postoje; arhiva ostaje za doradu.</v>
+        <v>Provjeriti prava, zaključanu godinu i upisati audit log.</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="str">
-        <v>F-087</v>
+        <v>F-086</v>
       </c>
       <c r="B353" t="str">
         <v>Zavrsni racun</v>
       </c>
       <c r="C353" t="str">
-        <v>Bilans stanja</v>
+        <v>Bilans uspjeha</v>
       </c>
       <c r="D353" t="str">
-        <v>Bilans stanja se racuna iz POSTED naloga po podesivoj semi pozicija, prikazuje tekucu godinu, prethodnu godinu - krajnje stanje i prethodnu godinu - pocetno stanje.</v>
+        <v>Bilans uspjeha se racuna iz POSTED naloga po podesivoj semi pozicija, prikazuje tekucu i prethodnu godinu i stampa formalni obrazac.</v>
       </c>
       <c r="E353" t="str">
         <v>Vrlo visok</v>
@@ -6442,24 +6442,24 @@
         <v>M-003,M-008,F-038</v>
       </c>
       <c r="L353" t="str">
-        <v>Dodati sistemski sablon, obracun, podesavanja po firmi, trajne rucne korekcije po AOP/koloni i HTML/CSS print obrazac. Arhiva ostaje za doradu.</v>
+        <v>Sistemska sema je seedovana u finansijski_izvjestaj_sabloni/pozicije; firma moze izmijeniti konta, izuzetke i formule kroz podesavanja. Trajne rucne korekcije po AOP/koloni postoje; arhiva ostaje za doradu.</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="str">
-        <v>F-088</v>
+        <v>F-087</v>
       </c>
       <c r="B354" t="str">
         <v>Zavrsni racun</v>
       </c>
       <c r="C354" t="str">
-        <v>Statisticki aneks</v>
+        <v>Bilans stanja</v>
       </c>
       <c r="D354" t="str">
-        <v>Statisticki aneks se racuna iz POSTED naloga po podesivoj semi pozicija, prikazuje tekucu i prethodnu godinu i stampa formalni obrazac.</v>
+        <v>Bilans stanja se racuna iz POSTED naloga po podesivoj semi pozicija, prikazuje tekucu godinu, prethodnu godinu - krajnje stanje i prethodnu godinu - pocetno stanje.</v>
       </c>
       <c r="E354" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F354" t="str">
         <v>Djelimicno implementirano</v>
@@ -6480,27 +6480,27 @@
         <v>M-003,M-008,F-038</v>
       </c>
       <c r="L354" t="str">
-        <v>Dodat sistemski sablon, obracun, podesavanja po firmi, trajne rucne korekcije po AOP/koloni i HTML/CSS print obrazac.</v>
+        <v>Dodati sistemski sablon, obracun, podesavanja po firmi, trajne rucne korekcije po AOP/koloni i HTML/CSS print obrazac. Arhiva ostaje za doradu.</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="str">
-        <v>F-089</v>
+        <v>F-088</v>
       </c>
       <c r="B355" t="str">
-        <v>Plate i zaposleni</v>
+        <v>Zavrsni racun</v>
       </c>
       <c r="C355" t="str">
-        <v>Šifarnik opština i prireza</v>
+        <v>Statisticki aneks</v>
       </c>
       <c r="D355" t="str">
-        <v>Globalni šifarnik povezuje opštinu sa DJP šifrom, stopom prireza, šifrom plaćanja i raspoloživim žiro računom za prirez; iste podatke koriste obračun plata i M-4.</v>
+        <v>Statisticki aneks se racuna iz POSTED naloga po podesivoj semi pozicija, prikazuje tekucu i prethodnu godinu i stampa formalni obrazac.</v>
       </c>
       <c r="E355" t="str">
         <v>Visok</v>
       </c>
       <c r="F355" t="str">
-        <v>Implementirano</v>
+        <v>Djelimicno implementirano</v>
       </c>
       <c r="G355" t="str">
         <v>Da</v>
@@ -6512,27 +6512,27 @@
         <v>Da</v>
       </c>
       <c r="J355" t="str">
-        <v>Da</v>
+        <v>Djelimicno</v>
       </c>
       <c r="K355" t="str">
-        <v>M-006</v>
+        <v>M-003,M-008,F-038</v>
       </c>
       <c r="L355" t="str">
-        <v>Unesena je 21 opština iz 001LP.mdb/B_Opstine. Prazni žiro računi iz izvora ostavljeni su prazni do pouzdanijeg zvaničnog izvora.</v>
+        <v>Dodat sistemski sablon, obracun, podesavanja po firmi, trajne rucne korekcije po AOP/koloni i HTML/CSS print obrazac.</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="str">
-        <v>F-090</v>
+        <v>F-089</v>
       </c>
       <c r="B356" t="str">
         <v>Plate i zaposleni</v>
       </c>
       <c r="C356" t="str">
-        <v>Obračunske podšifre i koeficijenti</v>
+        <v>Šifarnik opština i prireza</v>
       </c>
       <c r="D356" t="str">
-        <v>Šifra primanja može imati roditeljsku IOPPD osnovu, koeficijent iznosa ili staža, posebni procenat poreske osnovice i oznaku fonda sati.</v>
+        <v>Globalni šifarnik povezuje opštinu sa DJP šifrom, stopom prireza, šifrom plaćanja i raspoloživim žiro računom za prirez; iste podatke koriste obračun plata i M-4.</v>
       </c>
       <c r="E356" t="str">
         <v>Visok</v>
@@ -6556,24 +6556,24 @@
         <v>M-006</v>
       </c>
       <c r="L356" t="str">
-        <v>Dodato je 25 podšifara iz 001LP.mdb/A_SifR. Koeficijenti tipa IZNOS primjenjuju se u obračunu; STAZ je informativan za uvećano trajanje i ne množi zaradu. Važeće stope ostaju u novim vremenskim šifarnicima.</v>
+        <v>Unesena je 21 opština iz 001LP.mdb/B_Opstine. Prazni žiro računi iz izvora ostavljeni su prazni do pouzdanijeg zvaničnog izvora.</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="str">
-        <v>F-091</v>
+        <v>F-090</v>
       </c>
       <c r="B357" t="str">
-        <v>Firme i kontni plan</v>
+        <v>Plate i zaposleni</v>
       </c>
       <c r="C357" t="str">
-        <v>Trajno brisanje testne firme</v>
+        <v>Obračunske podšifre i koeficijenti</v>
       </c>
       <c r="D357" t="str">
-        <v>Admin agencije može trajno obrisati firmu i sve podatke koji pripadaju samo toj firmi tek nakon unosa potpuno istog punog naziva.</v>
+        <v>Šifra primanja može imati roditeljsku IOPPD osnovu, koeficijent iznosa ili staža, posebni procenat poreske osnovice i oznaku fonda sati.</v>
       </c>
       <c r="E357" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F357" t="str">
         <v>Implementirano</v>
@@ -6591,24 +6591,24 @@
         <v>Da</v>
       </c>
       <c r="K357" t="str">
-        <v>M-002</v>
+        <v>M-006</v>
       </c>
       <c r="L357" t="str">
-        <v>Brisanje je jedna backend transakcija sa agencijskim scope-om, audit zapisom i čišćenjem aktivnog konteksta. Obuhvata lokalne fiskalne/POS podatke; podaci poslati u zasebni Fiscal API ili Poresku upravu ostaju. Provjera db:check-company-purge pokriva tabele sa firma_id, uz obaveznu ručnu FK provjeru podređenih tabela pri svakoj promjeni šeme.</v>
+        <v>Dodato je 25 podšifara iz 001LP.mdb/A_SifR. Koeficijenti tipa IZNOS primjenjuju se u obračunu; STAZ je informativan za uvećano trajanje i ne množi zaradu. Važeće stope ostaju u novim vremenskim šifarnicima.</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="str">
-        <v>F-092</v>
+        <v>F-091</v>
       </c>
       <c r="B358" t="str">
-        <v>Plate i zaposleni</v>
+        <v>Firme i kontni plan</v>
       </c>
       <c r="C358" t="str">
-        <v>Podešavanje knjiženja po kategoriji</v>
+        <v>Trajno brisanje testne firme</v>
       </c>
       <c r="D358" t="str">
-        <v>Firma za aktivnu poslovnu godinu bira vrstu naloga i posebna duguje/potražuje konta za neto, porez, prirez, svaki doprinos i ostale komponente redovnog rada, ugovora o djelu, zakupa i ostalih ugovora.</v>
+        <v>Admin agencije može trajno obrisati firmu i sve podatke koji pripadaju samo toj firmi tek nakon unosa potpuno istog punog naziva.</v>
       </c>
       <c r="E358" t="str">
         <v>Vrlo visok</v>
@@ -6626,27 +6626,27 @@
         <v>Da</v>
       </c>
       <c r="J358" t="str">
-        <v>Djelimično</v>
+        <v>Da</v>
       </c>
       <c r="K358" t="str">
-        <v>M-003,M-006,F-024</v>
+        <v>M-002</v>
       </c>
       <c r="L358" t="str">
-        <v>Početna redovna šema izvedena je iz 001LP.mdb/ZAR_Kontir i ZAR_TipZB i prilagođena važećem kontnom planu. Šemu koristi automatsko knjiženje obračuna.</v>
+        <v>Brisanje je jedna backend transakcija sa agencijskim scope-om, audit zapisom i čišćenjem aktivnog konteksta. Obuhvata lokalne fiskalne/POS podatke; podaci poslati u zasebni Fiscal API ili Poresku upravu ostaju. Provjera db:check-company-purge pokriva tabele sa firma_id, uz obaveznu ručnu FK provjeru podređenih tabela pri svakoj promjeni šeme.</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="str">
-        <v>F-093</v>
+        <v>F-092</v>
       </c>
       <c r="B359" t="str">
         <v>Plate i zaposleni</v>
       </c>
       <c r="C359" t="str">
-        <v>Proknjižavanje obračuna plata</v>
+        <v>Podešavanje knjiženja po kategoriji</v>
       </c>
       <c r="D359" t="str">
-        <v>Akcija Proknjiži na obrađenom obračunu transakcijski kreira numerisan, izbalansiran i odmah POSTED PAYROLL nalog iz kategorijske D/P šeme i povezuje ga sa obračunom.</v>
+        <v>Firma za aktivnu poslovnu godinu bira vrstu naloga i posebna duguje/potražuje konta za neto, porez, prirez, svaki doprinos i ostale komponente redovnog rada, ugovora o djelu, zakupa i ostalih ugovora.</v>
       </c>
       <c r="E359" t="str">
         <v>Vrlo visok</v>
@@ -6667,24 +6667,24 @@
         <v>Djelimično</v>
       </c>
       <c r="K359" t="str">
-        <v>M-003,M-006,F-092</v>
+        <v>M-003,M-006,F-024</v>
       </c>
       <c r="L359" t="str">
-        <v>Provjeravaju se scope, pravo plate/post, zaključana godina, aktivna analitička konta, duple zbirne komponente i balans. Duplo knjiženje je blokirano. Vrati u nacrt atomski vraća nalog u DRAFT i obračun u CALCULATED; Proknjiži je ponovo dostupan uz isti nalog/broj. Backend prava oba modula; godina/PDV i zavisni mjesečni obračuni; audit rollback; realni paralelni zahtjevi i render dugmadi. Direktne izmjene/brisanje payroll naloga su blokirane.</v>
+        <v>Početna redovna šema izvedena je iz 001LP.mdb/ZAR_Kontir i ZAR_TipZB i prilagođena važećem kontnom planu. Šemu koristi automatsko knjiženje obračuna.</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="str">
-        <v>F-094</v>
+        <v>F-093</v>
       </c>
       <c r="B360" t="str">
         <v>Plate i zaposleni</v>
       </c>
       <c r="C360" t="str">
-        <v>OPP-ND prijava prireza</v>
+        <v>Proknjižavanje obračuna plata</v>
       </c>
       <c r="D360" t="str">
-        <v>Mjesečna prijava razvrstava porez na lična primanja, samostalnu djelatnost, imovinu/imovinska prava i kapital, primjenjuje važeću stopu prireza opštine firme i generiše službeni A4 obrazac.</v>
+        <v>Akcija Proknjiži na obrađenom obračunu transakcijski kreira numerisan, izbalansiran i odmah POSTED PAYROLL nalog iz kategorijske D/P šeme i povezuje ga sa obračunom.</v>
       </c>
       <c r="E360" t="str">
         <v>Vrlo visok</v>
@@ -6702,27 +6702,27 @@
         <v>Da</v>
       </c>
       <c r="J360" t="str">
-        <v>Da</v>
+        <v>Djelimično</v>
       </c>
       <c r="K360" t="str">
-        <v>M-006,F-089</v>
+        <v>M-003,M-006,F-092</v>
       </c>
       <c r="L360" t="str">
-        <v>Redovan rad ide u lična primanja, ugovor o djelu i ostali ugovori u samostalnu djelatnost, a zakup u imovinu. Kapital ostaje prazan dok ne postoji odgovarajuća vrsta obračuna. Vizuelni render provjeren je prema zvaničnom PDF-u.</v>
+        <v>Provjeravaju se scope, pravo plate/post, zaključana godina, aktivna analitička konta, duple zbirne komponente i balans. Duplo knjiženje je blokirano. Vrati u nacrt atomski vraća nalog u DRAFT i obračun u CALCULATED; Proknjiži je ponovo dostupan uz isti nalog/broj. Backend prava oba modula; godina/PDV i zavisni mjesečni obračuni; audit rollback; realni paralelni zahtjevi i render dugmadi. Direktne izmjene/brisanje payroll naloga su blokirane.</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="str">
-        <v>F-095</v>
+        <v>F-094</v>
       </c>
       <c r="B361" t="str">
-        <v>Računi / KIF-KUF</v>
+        <v>Plate i zaposleni</v>
       </c>
       <c r="C361" t="str">
-        <v>Unos i knjiženje pazara</v>
+        <v>OPP-ND prijava prireza</v>
       </c>
       <c r="D361" t="str">
-        <v>KIF prihvata dnevni ili mjesečni zbirni pazar sa PDV razradom i načinima naplate; pazar ulazi u PDV i knjiži se kroz posebna konta naplate.</v>
+        <v>Mjesečna prijava razvrstava porez na lična primanja, samostalnu djelatnost, imovinu/imovinska prava i kapital, primjenjuje važeću stopu prireza opštine firme i generiše službeni A4 obrazac.</v>
       </c>
       <c r="E361" t="str">
         <v>Vrlo visok</v>
@@ -6740,27 +6740,27 @@
         <v>Da</v>
       </c>
       <c r="J361" t="str">
-        <v>Djelimično</v>
+        <v>Da</v>
       </c>
       <c r="K361" t="str">
-        <v>M-010,F-062,F-068</v>
+        <v>M-006,F-089</v>
       </c>
       <c r="L361" t="str">
-        <v>Podržani su gotovina, kartice, virman i ostalo; prihodi/PDV koriste KIF šemu, a konta naplate se podešavaju po firmi.</v>
+        <v>Redovan rad ide u lična primanja, ugovor o djelu i ostali ugovori u samostalnu djelatnost, a zakup u imovinu. Kapital ostaje prazan dok ne postoji odgovarajuća vrsta obračuna. Vizuelni render provjeren je prema zvaničnom PDF-u.</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="str">
-        <v>F-096</v>
+        <v>F-095</v>
       </c>
       <c r="B362" t="str">
-        <v>POS / Kasa</v>
+        <v>Računi / KIF-KUF</v>
       </c>
       <c r="C362" t="str">
-        <v>Računovodstveni tok po načinu plaćanja</v>
+        <v>Unos i knjiženje pazara</v>
       </c>
       <c r="D362" t="str">
-        <v>Fiskalizovani POS virman ulazi pojedinačno u KIF i koristi nalog po šemi izlaznih računa; gotovina i kartica ulaze u zbirni dnevni ili mjesečni pazar.</v>
+        <v>KIF prihvata dnevni ili mjesečni zbirni pazar sa PDV razradom i načinima naplate; pazar ulazi u PDV i knjiži se kroz posebna konta naplate.</v>
       </c>
       <c r="E362" t="str">
         <v>Vrlo visok</v>
@@ -6781,24 +6781,24 @@
         <v>Djelimično</v>
       </c>
       <c r="K362" t="str">
-        <v>M-010,F-062,F-095</v>
+        <v>M-010,F-062,F-068</v>
       </c>
       <c r="L362" t="str">
-        <v>Virman tok ostaje pojedinačan. Zbirna obrada gotovine i kartica kreira idempotentan PAZAR u otvorenom KIF-u, čuva članstvo računa i prati status do zajedničkog KIF naloga i njegovog knjiženja. Automatski POS KIF zapis zaštićen je od ručne izmjene i brisanja.</v>
+        <v>Podržani su gotovina, kartice, virman i ostalo; prihodi/PDV koriste KIF šemu, a konta naplate se podešavaju po firmi.</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="str">
-        <v>F-097</v>
+        <v>F-096</v>
       </c>
       <c r="B363" t="str">
         <v>POS / Kasa</v>
       </c>
       <c r="C363" t="str">
-        <v>Potpuni storno POS računa</v>
+        <v>Računovodstveni tok po načinu plaćanja</v>
       </c>
       <c r="D363" t="str">
-        <v>Fiskalizovani POS račun može se potpuno stornirati povezanim negativnim korektivnim dokumentom bez brisanja originala.</v>
+        <v>Fiskalizovani POS virman ulazi pojedinačno u KIF i koristi nalog po šemi izlaznih računa; gotovina i kartica ulaze u zbirni dnevni ili mjesečni pazar.</v>
       </c>
       <c r="E363" t="str">
         <v>Vrlo visok</v>
@@ -6819,24 +6819,24 @@
         <v>Djelimično</v>
       </c>
       <c r="K363" t="str">
-        <v>M-011,F-096</v>
+        <v>M-010,F-062,F-095</v>
       </c>
       <c r="L363" t="str">
-        <v>Agencijski POS i direktni portal koriste isti tenant-aware servis. Obavezni su razlog i potvrda; uključeni su Fiscal API storno, povrat robe, audit i retry. Agencijski tok zadržava računovodstvenu obradu, a direktni FISCAL_ONLY tok ne kreira KIF ni nalog. Djelimični povrat čeka API podršku.</v>
+        <v>Virman tok ostaje pojedinačan. Zbirna obrada gotovine i kartica kreira idempotentan PAZAR u otvorenom KIF-u, čuva članstvo računa i prati status do zajedničkog KIF naloga i njegovog knjiženja. Automatski POS KIF zapis zaštićen je od ručne izmjene i brisanja.</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="str">
-        <v>F-098</v>
+        <v>F-097</v>
       </c>
       <c r="B364" t="str">
         <v>POS / Kasa</v>
       </c>
       <c r="C364" t="str">
-        <v>POS izvještaji i termalna štampa</v>
+        <v>Potpuni storno POS računa</v>
       </c>
       <c r="D364" t="str">
-        <v>Promet po periodu i kasi sa neto stornima, plaćanjima, PDV-om i artiklima; fiskalni račun se štampa na 58/80 mm papiru.</v>
+        <v>Fiskalizovani POS račun može se potpuno stornirati povezanim negativnim korektivnim dokumentom bez brisanja originala.</v>
       </c>
       <c r="E364" t="str">
         <v>Vrlo visok</v>
@@ -6857,24 +6857,24 @@
         <v>Djelimično</v>
       </c>
       <c r="K364" t="str">
-        <v>M-011,F-097</v>
+        <v>M-011,F-096</v>
       </c>
       <c r="L364" t="str">
-        <v>Browser štampa fiskalnog računa čuva dvojezičnu srpsko-englesku A4 opciju i prikazuje QR, IKOF/JIKR, kupca i vezu storna. Izvještaj ima zasebnu štampu; direktni portal auditira otvaranje A4 i 58/80 mm štampe. Stvarni termalni printer i reprint audit agencijskog POS-a ostaju za ručni QA.</v>
+        <v>Agencijski POS i direktni portal koriste isti tenant-aware servis. Obavezni su razlog i potvrda; uključeni su Fiscal API storno, povrat robe, audit i retry. Agencijski tok zadržava računovodstvenu obradu, a direktni FISCAL_ONLY tok ne kreira KIF ni nalog. Djelimični povrat čeka API podršku.</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="str">
-        <v>F-099</v>
+        <v>F-098</v>
       </c>
       <c r="B365" t="str">
         <v>POS / Kasa</v>
       </c>
       <c r="C365" t="str">
-        <v>Smjenski presjek i predaja kase</v>
+        <v>POS izvještaji i termalna štampa</v>
       </c>
       <c r="D365" t="str">
-        <v>Radnik otvara smjenu sa preuzetom gotovinom, a pri predaji zatvara smjenu i čuva presjek prometa do tog trenutka.</v>
+        <v>Promet po periodu i kasi sa neto stornima, plaćanjima, PDV-om i artiklima; fiskalni račun se štampa na 58/80 mm papiru.</v>
       </c>
       <c r="E365" t="str">
         <v>Vrlo visok</v>
@@ -6895,24 +6895,24 @@
         <v>Djelimično</v>
       </c>
       <c r="K365" t="str">
-        <v>M-011,F-098</v>
+        <v>M-011,F-097</v>
       </c>
       <c r="L365" t="str">
-        <v>Jedna otvorena smjena po kasi; presjek čuva račune, plaćanja, ukupan promet i očekivanu gotovinu. Ne mijenja dnevni ili mjesečni KIF zbir.</v>
+        <v>Browser štampa fiskalnog računa čuva dvojezičnu srpsko-englesku A4 opciju i prikazuje QR, IKOF/JIKR, kupca i vezu storna. Izvještaj ima zasebnu štampu; direktni portal auditira otvaranje A4 i 58/80 mm štampe. Stvarni termalni printer i reprint audit agencijskog POS-a ostaju za ručni QA.</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="str">
-        <v>F-100</v>
+        <v>F-099</v>
       </c>
       <c r="B366" t="str">
-        <v>Portal direktnog fiskalnog klijenta</v>
+        <v>POS / Kasa</v>
       </c>
       <c r="C366" t="str">
-        <v>Siguran portal shell i automatski kontekst</v>
+        <v>Smjenski presjek i predaja kase</v>
       </c>
       <c r="D366" t="str">
-        <v>Direktni korisnik poslije prijave ulazi na /portal, dobija svoju jedinu firmu i važeću poslovnu godinu, ne vidi sistemski tenant i ne može otvoriti /agencija prostor.</v>
+        <v>Radnik otvara smjenu sa preuzetom gotovinom, a pri predaji zatvara smjenu i čuva presjek prometa do tog trenutka.</v>
       </c>
       <c r="E366" t="str">
         <v>Vrlo visok</v>
@@ -6930,27 +6930,27 @@
         <v>Da</v>
       </c>
       <c r="J366" t="str">
-        <v>Da</v>
+        <v>Djelimično</v>
       </c>
       <c r="K366" t="str">
-        <v>M-001,M-002,M-012</v>
+        <v>M-011,F-098</v>
       </c>
       <c r="L366" t="str">
-        <v>Centralni backend guard razlikuje direktnog korisnika preko sistemskog tenant-a, KorisnikFirma access_type-a i eksplicitnih prava; cookie nije dokaz ovlašćenja.</v>
+        <v>Jedna otvorena smjena po kasi; presjek čuva račune, plaćanja, ukupan promet i očekivanu gotovinu. Ne mijenja dnevni ili mjesečni KIF zbir.</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="str">
-        <v>F-101</v>
+        <v>F-100</v>
       </c>
       <c r="B367" t="str">
         <v>Portal direktnog fiskalnog klijenta</v>
       </c>
       <c r="C367" t="str">
-        <v>Operativni dashboard</v>
+        <v>Siguran portal shell i automatski kontekst</v>
       </c>
       <c r="D367" t="str">
-        <v>Početna prikazuje današnji neto fiskalizovani promet, broj računa i storna, prosjek, načine plaćanja, posljednje račune i upozorenja sa correlation ID-em.</v>
+        <v>Direktni korisnik poslije prijave ulazi na /portal, dobija svoju jedinu firmu i važeću poslovnu godinu, ne vidi sistemski tenant i ne može otvoriti /agencija prostor.</v>
       </c>
       <c r="E367" t="str">
         <v>Vrlo visok</v>
@@ -6968,33 +6968,33 @@
         <v>Da</v>
       </c>
       <c r="J367" t="str">
-        <v>Djelimično</v>
+        <v>Da</v>
       </c>
       <c r="K367" t="str">
-        <v>F-100,F-097,F-098</v>
+        <v>M-001,M-002,M-012</v>
       </c>
       <c r="L367" t="str">
-        <v>Metrike koriste Europe/Podgorica, centnu aritmetiku i uključuju original plus negativni korektivni dokument radi ispravnog neto prometa.</v>
+        <v>Centralni backend guard razlikuje direktnog korisnika preko sistemskog tenant-a, KorisnikFirma access_type-a i eksplicitnih prava; cookie nije dokaz ovlašćenja.</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="str">
-        <v>F-102</v>
+        <v>F-101</v>
       </c>
       <c r="B368" t="str">
         <v>Portal direktnog fiskalnog klijenta</v>
       </c>
       <c r="C368" t="str">
-        <v>POS i klasične bezgotovinske fakture</v>
+        <v>Operativni dashboard</v>
       </c>
       <c r="D368" t="str">
-        <v>Portal omogućava mobile-first POS i dokument-oriented OFFICE fakturu nad istim prodajnim dokumentom i postojećim Fiscal API tokom.</v>
+        <v>Početna prikazuje današnji neto fiskalizovani promet, broj računa i storna, prosjek, načine plaćanja, posljednje račune i upozorenja sa correlation ID-em.</v>
       </c>
       <c r="E368" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F368" t="str">
-        <v>Implementirano djelimično</v>
+        <v>Implementirano</v>
       </c>
       <c r="G368" t="str">
         <v>Da</v>
@@ -7009,30 +7009,30 @@
         <v>Djelimično</v>
       </c>
       <c r="K368" t="str">
-        <v>F-100,M-004,M-011</v>
+        <v>F-100,F-097,F-098</v>
       </c>
       <c r="L368" t="str">
-        <v>Oba toka koriste idempotency, eksplicitnu Production potvrdu, status recovery i štampu. POS puni storno koristi isti servis kao agencijski POS; direct FISCAL_ONLY uspjeh ne kreira KIF ni nalog. Ostaje ručni end-to-end QA.</v>
+        <v>Metrike koriste Europe/Podgorica, centnu aritmetiku i uključuju original plus negativni korektivni dokument radi ispravnog neto prometa.</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="str">
-        <v>F-103</v>
+        <v>F-102</v>
       </c>
       <c r="B369" t="str">
         <v>Portal direktnog fiskalnog klijenta</v>
       </c>
       <c r="C369" t="str">
-        <v>Fiskalni računi izvještaji šifarnici i podešavanja</v>
+        <v>POS i klasične bezgotovinske fakture</v>
       </c>
       <c r="D369" t="str">
-        <v>Jedinstveni pregled POS/OFFICE/storno dokumenata, prodajni izvještaji, artikli, cijene, kupci i samo dozvoljena operativna podešavanja.</v>
+        <v>Portal omogućava mobile-first POS i dokument-oriented OFFICE fakturu nad istim prodajnim dokumentom i postojećim Fiscal API tokom.</v>
       </c>
       <c r="E369" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F369" t="str">
-        <v>Implementirano</v>
+        <v>Implementirano djelimično</v>
       </c>
       <c r="G369" t="str">
         <v>Da</v>
@@ -7047,24 +7047,24 @@
         <v>Djelimično</v>
       </c>
       <c r="K369" t="str">
-        <v>F-100,F-101,F-102</v>
+        <v>F-100,M-004,M-011</v>
       </c>
       <c r="L369" t="str">
-        <v>Operativna podešavanja obuhvataju kontakt, glavni račun, kasu, magacin, plaćanje, rok, štampu, smjene, lager i Test depozit. Fiskalna administracija ostaje platformskom adminu; produkcijski depozit čeka API rutu.</v>
+        <v>Oba toka koriste idempotency, eksplicitnu Production potvrdu, status recovery i štampu. POS puni storno koristi isti servis kao agencijski POS; direct FISCAL_ONLY uspjeh ne kreira KIF ni nalog. Ostaje ručni end-to-end QA.</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="str">
-        <v>F-104</v>
+        <v>F-103</v>
       </c>
       <c r="B370" t="str">
-        <v>Plate i zaposleni</v>
+        <v>Portal direktnog fiskalnog klijenta</v>
       </c>
       <c r="C370" t="str">
-        <v>Pojedinačni period i sati radnika</v>
+        <v>Fiskalni računi izvještaji šifarnici i podešavanja</v>
       </c>
       <c r="D370" t="str">
-        <v>Obračunska stavka ima datum od/do unutar mjeseca i trajanja zaposlenja; sistem predlaže sate prema radnim danima i fondu, a računovođa može sa auditom ručno promijeniti ili vratiti automatske sate.</v>
+        <v>Jedinstveni pregled POS/OFFICE/storno dokumenata, prodajni izvještaji, artikli, cijene, kupci i samo dozvoljena operativna podešavanja.</v>
       </c>
       <c r="E370" t="str">
         <v>Vrlo visok</v>
@@ -7082,30 +7082,30 @@
         <v>Da</v>
       </c>
       <c r="J370" t="str">
-        <v>Da</v>
+        <v>Djelimično</v>
       </c>
       <c r="K370" t="str">
-        <v>M-006</v>
+        <v>F-100,F-101,F-102</v>
       </c>
       <c r="L370" t="str">
-        <v>Priprema uključuje i radnike koji počnu ili završe radni odnos tokom mjeseca. Testovi pokrivaju početak 17-og, prestanak prije kraja, nekoliko dana rada i period van mjeseca; kalendar praznika i nestandardnih smjena ostaje dorada.</v>
+        <v>Operativna podešavanja obuhvataju kontakt, glavni račun, kasu, magacin, plaćanje, rok, štampu, smjene, lager i Test depozit. Fiskalna administracija ostaje platformskom adminu; produkcijski depozit čeka API rutu.</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="str">
-        <v>F-105</v>
+        <v>F-104</v>
       </c>
       <c r="B371" t="str">
-        <v>Korisnici, agencije i prava</v>
+        <v>Plate i zaposleni</v>
       </c>
       <c r="C371" t="str">
-        <v>Sklopivi agencijski meni</v>
+        <v>Pojedinačni period i sati radnika</v>
       </c>
       <c r="D371" t="str">
-        <v>Glavni agencijski meni se na desktopu sklapa na ikonice i pamti izbor; na telefonu se otvara kao pristupačan bočni panel preko sadržaja.</v>
+        <v>Obračunska stavka ima datum od/do unutar mjeseca i trajanja zaposlenja; sistem predlaže sate prema radnim danima i fondu, a računovođa može sa auditom ručno promijeniti ili vratiti automatske sate.</v>
       </c>
       <c r="E371" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F371" t="str">
         <v>Implementirano</v>
@@ -7117,30 +7117,30 @@
         <v>Da</v>
       </c>
       <c r="I371" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="J371" t="str">
         <v>Da</v>
       </c>
       <c r="K371" t="str">
-        <v>M-001</v>
+        <v>M-006</v>
       </c>
       <c r="L371" t="str">
-        <v>Sadržaj koristi oslobođenu širinu; dostupni su ujednačene SVG ikonice, aktivna stavka, title opisi, aria oznake, Escape i backdrop zatvaranje te reduced-motion stilovi. TypeScript i lint su čisti; browser QA je potvrđen u otvorenom i sklopljenom stanju.</v>
+        <v>Priprema uključuje i radnike koji počnu ili završe radni odnos tokom mjeseca. Testovi pokrivaju početak 17-og, prestanak prije kraja, nekoliko dana rada i period van mjeseca; kalendar praznika i nestandardnih smjena ostaje dorada.</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="str">
-        <v>F-106</v>
+        <v>F-105</v>
       </c>
       <c r="B372" t="str">
-        <v>Izvještaji i dashboard</v>
+        <v>Korisnici, agencije i prava</v>
       </c>
       <c r="C372" t="str">
-        <v>Operativne stavke početnog dashboarda</v>
+        <v>Sklopivi agencijski meni</v>
       </c>
       <c r="D372" t="str">
-        <v>Početna za aktivnu firmu/godinu prikazuje nacrte naloga, kalkulacije koje čekaju KUF i izlazne račune koji čekaju KIF, umjesto audit logova.</v>
+        <v>Glavni agencijski meni se na desktopu sklapa na ikonice i pamti izbor; na telefonu se otvara kao pristupačan bočni panel preko sadržaja.</v>
       </c>
       <c r="E372" t="str">
         <v>Visok</v>
@@ -7155,33 +7155,33 @@
         <v>Da</v>
       </c>
       <c r="I372" t="str">
-        <v>Da</v>
+        <v>Ne</v>
       </c>
       <c r="J372" t="str">
         <v>Da</v>
       </c>
       <c r="K372" t="str">
-        <v>M-003,M-004,M-009,M-010</v>
+        <v>M-001</v>
       </c>
       <c r="L372" t="str">
-        <v>Brojači i najnovije stavke koriste stvarne statuse DRAFT/WAITING_KUF/WAITING_KIF, tenant scope i prava pregleda; redovi vode direktno na izvorni dokument. Browser QA je potvrđen.</v>
+        <v>Sadržaj koristi oslobođenu širinu; dostupni su ujednačene SVG ikonice, aktivna stavka, title opisi, aria oznake, Escape i backdrop zatvaranje te reduced-motion stilovi. TypeScript i lint su čisti; browser QA je potvrđen u otvorenom i sklopljenom stanju.</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="str">
-        <v>F-107</v>
+        <v>F-106</v>
       </c>
       <c r="B373" t="str">
-        <v>Robno i izvještaji</v>
+        <v>Izvještaji i dashboard</v>
       </c>
       <c r="C373" t="str">
-        <v>Lager lista i kartica artikla</v>
+        <v>Operativne stavke početnog dashboarda</v>
       </c>
       <c r="D373" t="str">
-        <v>Lager lista prikazuje stanje i vrijednosti po magacinu/artiklu, a kartica hronološke ulaze, izlaze i saldo za izabrani period.</v>
+        <v>Početna za aktivnu firmu/godinu prikazuje nacrte naloga, kalkulacije koje čekaju KUF i izlazne račune koji čekaju KIF, umjesto audit logova.</v>
       </c>
       <c r="E373" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F373" t="str">
         <v>Implementirano</v>
@@ -7199,27 +7199,27 @@
         <v>Da</v>
       </c>
       <c r="K373" t="str">
-        <v>M-004,M-009</v>
+        <v>M-003,M-004,M-009,M-010</v>
       </c>
       <c r="L373" t="str">
-        <v>Iste serverske komponente koriste se u Robnom i centralnim Izvještajima. Filteri obuhvataju magacin, grupu, artikal, znak stanja i period; kartica računa početno stanje prije perioda i povezuje izvorne dokumente.</v>
+        <v>Brojači i najnovije stavke koriste stvarne statuse DRAFT/WAITING_KUF/WAITING_KIF, tenant scope i prava pregleda; redovi vode direktno na izvorni dokument. Browser QA je potvrđen.</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="str">
-        <v>F-108</v>
+        <v>F-107</v>
       </c>
       <c r="B374" t="str">
-        <v>Izvještaji i dashboard</v>
+        <v>Robno i izvještaji</v>
       </c>
       <c r="C374" t="str">
-        <v>Centralne kartice konta i partnera, PDV i plate</v>
+        <v>Lager lista i kartica artikla</v>
       </c>
       <c r="D374" t="str">
-        <v>Centralni meni izvještaja otvara postojeće funkcionalne kartice glavne knjige, mjesečni PDV pregled i pregled izvještaja plata bez dupliranja poslovne računice.</v>
+        <v>Lager lista prikazuje stanje i vrijednosti po magacinu/artiklu, a kartica hronološke ulaze, izlaze i saldo za izabrani period.</v>
       </c>
       <c r="E374" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F374" t="str">
         <v>Implementirano</v>
@@ -7237,24 +7237,24 @@
         <v>Da</v>
       </c>
       <c r="K374" t="str">
-        <v>M-003,M-006,M-007,M-009</v>
+        <v>M-004,M-009</v>
       </c>
       <c r="L374" t="str">
-        <v>Kartica konta ima lijevi pretraživ spisak, izbor samo konta sa POSTED prometom ili svih aktivnih konta i desni detalj sa periodom/partnerom; na telefonu radi kao lista pa detalj. Isti master-detail prikaz koristi i ruta pod Nalozima. Partnerska kartica koristi analitička konta i partnera, PDV postojeće periode/prijave, a plate obračune, M-4, OPP-ND i IOPPD.</v>
+        <v>Iste serverske komponente koriste se u Robnom i centralnim Izvještajima. Filteri obuhvataju magacin, grupu, artikal, znak stanja i period; kartica računa početno stanje prije perioda i povezuje izvorne dokumente.</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="str">
-        <v>F-109</v>
+        <v>F-108</v>
       </c>
       <c r="B375" t="str">
-        <v>Nalozi / Izvještaji</v>
+        <v>Izvještaji i dashboard</v>
       </c>
       <c r="C375" t="str">
-        <v>Ispravna štampa bruto bilansa</v>
+        <v>Centralne kartice konta i partnera, PDV i plate</v>
       </c>
       <c r="D375" t="str">
-        <v>Bruto bilans se štampa na A4 landscape sa osam stabilnih kolona, neprelomivim iznosima i ponovljenim zaglavljem tabele.</v>
+        <v>Centralni meni izvještaja otvara postojeće funkcionalne kartice glavne knjige, mjesečni PDV pregled i pregled izvještaja plata bez dupliranja poslovne računice.</v>
       </c>
       <c r="E375" t="str">
         <v>Visok</v>
@@ -7269,30 +7269,30 @@
         <v>Da</v>
       </c>
       <c r="I375" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="J375" t="str">
         <v>Da</v>
       </c>
       <c r="K375" t="str">
-        <v>M-003,F-038</v>
+        <v>M-003,M-006,M-007,M-009</v>
       </c>
       <c r="L375" t="str">
-        <v>Zasebni stil i colgroup odvajaju bruto bilans od sedmokolonskog Bilansa stanja: konto 8%, naziv 26%, šest iznosa po 11%; redovi se ne cijepaju preko stranice.</v>
+        <v>Kartica konta ima lijevi pretraživ spisak, izbor samo konta sa POSTED prometom ili svih aktivnih konta i desni detalj sa periodom/partnerom; na telefonu radi kao lista pa detalj. Isti master-detail prikaz koristi i ruta pod Nalozima. Partnerska kartica koristi analitička konta i partnera, PDV postojeće periode/prijave, a plate obračune, M-4, OPP-ND i IOPPD.</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="str">
-        <v>F-110</v>
+        <v>F-109</v>
       </c>
       <c r="B376" t="str">
         <v>Nalozi / Izvještaji</v>
       </c>
       <c r="C376" t="str">
-        <v>Štampa kartice konta</v>
+        <v>Ispravna štampa bruto bilansa</v>
       </c>
       <c r="D376" t="str">
-        <v>Izabrana kartica konta štampa se sa aktivnim partnerom i periodom, početnim saldom, prometom, tekućim saldom i završnim zbirom.</v>
+        <v>Bruto bilans se štampa na A4 landscape sa osam stabilnih kolona, neprelomivim iznosima i ponovljenim zaglavljem tabele.</v>
       </c>
       <c r="E376" t="str">
         <v>Visok</v>
@@ -7313,27 +7313,27 @@
         <v>Da</v>
       </c>
       <c r="K376" t="str">
-        <v>M-003,F-037,F-108</v>
+        <v>M-003,F-038</v>
       </c>
       <c r="L376" t="str">
-        <v>Čista A4 landscape ruta prikazuje samo POSTED stavke aktivne firme i godine, provjerava tenant/account/partner scope i ponavlja zaglavlje tabele preko stranica.</v>
+        <v>Zasebni stil i colgroup odvajaju bruto bilans od sedmokolonskog Bilansa stanja: konto 8%, naziv 26%, šest iznosa po 11%; redovi se ne cijepaju preko stranice.</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="str">
-        <v>F-111</v>
+        <v>F-110</v>
       </c>
       <c r="B377" t="str">
-        <v>Završni račun</v>
+        <v>Nalozi / Izvještaji</v>
       </c>
       <c r="C377" t="str">
-        <v>Kontrole spremnosti završnog računa</v>
+        <v>Štampa kartice konta</v>
       </c>
       <c r="D377" t="str">
-        <v>Jedinstven ekran provjerava glavnu knjigu, pomoćne evidencije, šeme i zaključna knjiženja prije arhiviranja i zaključivanja godine.</v>
+        <v>Izabrana kartica konta štampa se sa aktivnim partnerom i periodom, početnim saldom, prometom, tekućim saldom i završnim zbirom.</v>
       </c>
       <c r="E377" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F377" t="str">
         <v>Implementirano</v>
@@ -7351,24 +7351,24 @@
         <v>Da</v>
       </c>
       <c r="K377" t="str">
-        <v>M-003,M-005,M-006,M-007,M-008,M-010</v>
+        <v>M-003,F-037,F-108</v>
       </c>
       <c r="L377" t="str">
-        <v>Read-only tenant-aware kontrolni centar razdvaja greške/upozorenja/uspjehe i vodi direktno na razrješenje; provjerava POSTED balans, analitiku, nacrte, KIF/KUF, izvode, plate, PDV, šablone, 5990/6990, klase 5/6, korekcije, arhivu i matične podatke. Izvorna PDV konta moraju imati saldo 0,00, klasa 5 dugovni/nulti, a klasa 6 potražni/nulti saldo; sporna konta vode na karticu.</v>
+        <v>Čista A4 landscape ruta prikazuje samo POSTED stavke aktivne firme i godine, provjerava tenant/account/partner scope i ponavlja zaglavlje tabele preko stranica.</v>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="str">
-        <v>F-112</v>
+        <v>F-111</v>
       </c>
       <c r="B378" t="str">
-        <v>Nalozi / Izvještaji</v>
+        <v>Završni račun</v>
       </c>
       <c r="C378" t="str">
-        <v>Poslovne jedinice kroz dokumente i knjiženja</v>
+        <v>Kontrole spremnosti završnog računa</v>
       </c>
       <c r="D378" t="str">
-        <v>Organizaciona dimenzija prati magacin, dokument i stavku naloga te omogućava rezultat po jedinicama.</v>
+        <v>Jedinstven ekran provjerava glavnu knjigu, pomoćne evidencije, šeme i zaključna knjiženja prije arhiviranja i zaključivanja godine.</v>
       </c>
       <c r="E378" t="str">
         <v>Vrlo visok</v>
@@ -7383,33 +7383,33 @@
         <v>Da</v>
       </c>
       <c r="I378" t="str">
-        <v>Da</v>
+        <v>Ne</v>
       </c>
       <c r="J378" t="str">
-        <v>Djelimično</v>
+        <v>Da</v>
       </c>
       <c r="K378" t="str">
-        <v>F-026,F-029,F-041</v>
+        <v>M-003,M-005,M-006,M-007,M-008,M-010</v>
       </c>
       <c r="L378" t="str">
-        <v>Kalkulacije i izlazni/POS računi nasljeđuju jedinicu magacina; ručni KIF/KUF, pazar, izvod i plata imaju izbor. KIF/KUF knjiženje čuva jedinicu po stavci, izvještaj računa klasu 6 minus klasu 5, a završna kontrola prijavljuje obaveznu jedinicu koja nedostaje. Izbor se automatski skriva kada firma nema aktivnih jedinica.</v>
+        <v>Read-only tenant-aware kontrolni centar razdvaja greške/upozorenja/uspjehe i vodi direktno na razrješenje; provjerava POSTED balans, analitiku, nacrte, KIF/KUF, izvode, plate, PDV, šablone, 5990/6990, klase 5/6, korekcije, arhivu i matične podatke. Izvorna PDV konta moraju imati saldo 0,00, klasa 5 dugovni/nulti, a klasa 6 potražni/nulti saldo; sporna konta vode na karticu.</v>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="str">
-        <v>F-113</v>
+        <v>F-112</v>
       </c>
       <c r="B379" t="str">
-        <v>Završni račun</v>
+        <v>Nalozi / Izvještaji</v>
       </c>
       <c r="C379" t="str">
-        <v>XML izvoz finansijskih iskaza</v>
+        <v>Poslovne jedinice kroz dokumente i knjiženja</v>
       </c>
       <c r="D379" t="str">
-        <v>BS/BU/SA sa korekcijama i uporednim kolonama; ostale sekcije nulte prema potvrđenom obimu.</v>
+        <v>Organizaciona dimenzija prati magacin, dokument i stavku naloga te omogućava rezultat po jedinicama.</v>
       </c>
       <c r="E379" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F379" t="str">
         <v>Implementirano</v>
@@ -7421,30 +7421,30 @@
         <v>Da</v>
       </c>
       <c r="I379" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="J379" t="str">
-        <v>Da</v>
+        <v>Djelimično</v>
       </c>
       <c r="K379" t="str">
-        <v>M-008</v>
+        <v>F-026,F-029,F-041</v>
       </c>
       <c r="L379" t="str">
-        <v>Zaglavlje za pregled; view/export scope i audit; XSD test. Portal QA ostaje otvoren.</v>
+        <v>Kalkulacije i izlazni/POS računi nasljeđuju jedinicu magacina; ručni KIF/KUF, pazar, izvod i plata imaju izbor. KIF/KUF knjiženje čuva jedinicu po stavci, izvještaj računa klasu 6 minus klasu 5, a završna kontrola prijavljuje obaveznu jedinicu koja nedostaje. Izbor se automatski skriva kada firma nema aktivnih jedinica.</v>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="str">
-        <v>F-114</v>
+        <v>F-113</v>
       </c>
       <c r="B380" t="str">
-        <v>Korisnici, agencije i prava</v>
+        <v>Završni račun</v>
       </c>
       <c r="C380" t="str">
-        <v>Centralno slanje emaila i Reply-To agencije</v>
+        <v>XML izvoz finansijskih iskaza</v>
       </c>
       <c r="D380" t="str">
-        <v>Sistem šalje sa admin@summasummarum.me, dok administrator agencije podešava adresu na koju prima odgovore.</v>
+        <v>BS/BU/SA sa korekcijama i uporednim kolonama; ostale sekcije nulte prema potvrđenom obimu.</v>
       </c>
       <c r="E380" t="str">
         <v>Visok</v>
@@ -7459,33 +7459,33 @@
         <v>Da</v>
       </c>
       <c r="I380" t="str">
-        <v>Da</v>
+        <v>Ne</v>
       </c>
       <c r="J380" t="str">
-        <v>Djelimično</v>
+        <v>Da</v>
       </c>
       <c r="K380" t="str">
-        <v>M-001</v>
+        <v>M-008</v>
       </c>
       <c r="L380" t="str">
-        <v>Admin-only podešavanje po agenciji, backend validacija, audit i probno slanje. Pozivnice koje kreira admin agencije koriste sačuvani Reply-To; produkcijski SMTP nalog mora biti ovlašćen za centralnu From adresu.</v>
+        <v>Zaglavlje za pregled; view/export scope i audit; XSD test. Portal QA ostaje otvoren.</v>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="str">
-        <v>F-115</v>
+        <v>F-114</v>
       </c>
       <c r="B381" t="str">
-        <v>Plate i zaposleni</v>
+        <v>Korisnici, agencije i prava</v>
       </c>
       <c r="C381" t="str">
-        <v>Dokumenti obračuna plata</v>
+        <v>Centralno slanje emaila i Reply-To agencije</v>
       </c>
       <c r="D381" t="str">
-        <v>Obračun daje pojedinačne i zbirne platne liste, rekapitulaciju i kontrolisane naloge za plaćanje iz istih sačuvanih stavki.</v>
+        <v>Sistem šalje sa admin@summasummarum.me, dok administrator agencije podešava adresu na koju prima odgovore.</v>
       </c>
       <c r="E381" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F381" t="str">
         <v>Implementirano</v>
@@ -7503,27 +7503,27 @@
         <v>Djelimično</v>
       </c>
       <c r="K381" t="str">
-        <v>M-006,F-089</v>
+        <v>M-001</v>
       </c>
       <c r="L381" t="str">
-        <v>A4 HTML/CSS štampa je dostupna uz plate/view i plate/export; obračunati dokumenti nose NACRT. Virmani prate dostavljeni PDF raspored sa tri obrasca po A4 strani i podesivom gornjom/lijevom marginom. Kompaktna priprema bez horizontalnog skrola omogućava lokalnu korekciju svih polja prije štampe, bez izmjene obračuna u bazi. Neto ide po radniku; porez, PIO, nezaposlenost i Fond rada zbirno na 820-30000-74; prirez posebno po opštini, Komora na 520-939100-43 i sindikat na 510-105-16.</v>
+        <v>Admin-only podešavanje po agenciji, backend validacija, audit i probno slanje. Pozivnice koje kreira admin agencije koriste sačuvani Reply-To; produkcijski SMTP nalog mora biti ovlašćen za centralnu From adresu.</v>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="str">
-        <v>F-116</v>
+        <v>F-115</v>
       </c>
       <c r="B382" t="str">
-        <v>Dashboard</v>
+        <v>Plate i zaposleni</v>
       </c>
       <c r="C382" t="str">
-        <v>Opšti virmani</v>
+        <v>Dokumenti obračuna plata</v>
       </c>
       <c r="D382" t="str">
-        <v>Ručni platni nalozi nevezani za obračun plata čuvaju se kao nacrti, odštampani zapisi ili šabloni i štampaju po tri na A4.</v>
+        <v>Obračun daje pojedinačne i zbirne platne liste, rekapitulaciju i kontrolisane naloge za plaćanje iz istih sačuvanih stavki.</v>
       </c>
       <c r="E382" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F382" t="str">
         <v>Implementirano</v>
@@ -7541,62 +7541,62 @@
         <v>Djelimično</v>
       </c>
       <c r="K382" t="str">
-        <v>M-001,M-002,M-009</v>
+        <v>M-006,F-089</v>
       </c>
       <c r="L382" t="str">
-        <v>Aktivna firma predlaže nalogodavca i glavni račun; sva polja su izmjenjiva. Zasebna virmani prava štite pregled/unos/izmjenu/brisanje/izvoz. Modul ne knjiži promet niti mijenja izvode.</v>
+        <v>A4 HTML/CSS štampa je dostupna uz plate/view i plate/export; obračunati dokumenti nose NACRT. Virmani prate dostavljeni PDF raspored sa tri obrasca po A4 strani i podesivom gornjom/lijevom marginom. Kompaktna priprema bez horizontalnog skrola omogućava lokalnu korekciju svih polja prije štampe, bez izmjene obračuna u bazi. Neto ide po radniku; porez, PIO, nezaposlenost i Fond rada zbirno na 820-30000-74; prirez posebno po opštini, Komora na 520-939100-43 i sindikat na 510-105-16.</v>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="str">
-        <v>M7-IMAP-01</v>
+        <v>F-116</v>
       </c>
       <c r="B383" t="str">
-        <v>Modul 7</v>
+        <v>Dashboard</v>
       </c>
       <c r="C383" t="str">
-        <v>IMAP test veze</v>
+        <v>Opšti virmani</v>
       </c>
       <c r="D383" t="str">
-        <v>Read-only INBOX i broj poruka; bez preuzimanja i uvoza</v>
+        <v>Ručni platni nalozi nevezani za obračun plata čuvaju se kao nacrti, odštampani zapisi ili šabloni i štampaju po tri na A4.</v>
       </c>
       <c r="E383" t="str">
         <v>Visok</v>
       </c>
       <c r="F383" t="str">
-        <v>Završeno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G383" t="str">
-        <v>DA</v>
+        <v>Da</v>
       </c>
       <c r="H383" t="str">
-        <v>DA</v>
+        <v>Da</v>
       </c>
       <c r="I383" t="str">
-        <v>Nije potrebno</v>
+        <v>Da</v>
       </c>
       <c r="J383" t="str">
-        <v>10/10; TLS i prijava potvrđeni</v>
+        <v>Djelimično</v>
       </c>
       <c r="K383" t="str">
-        <v>Mail nalog u bazi</v>
+        <v>M-001,M-002,M-009</v>
       </c>
       <c r="L383" t="str">
-        <v>Admin agencije; sifrovana lozinka AES-256-GCM; MAIL_ENCRYPTION_KEY u env</v>
+        <v>Aktivna firma predlaže nalogodavca i glavni račun; sva polja su izmjenjiva. Zasebna virmani prava štite pregled/unos/izmjenu/brisanje/izvoz. Modul ne knjiži promet niti mijenja izvode.</v>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="str">
-        <v>M7-IMAP-02</v>
+        <v>M7-IMAP-01</v>
       </c>
       <c r="B384" t="str">
         <v>Modul 7</v>
       </c>
       <c r="C384" t="str">
-        <v>Pregled mailova</v>
+        <v>IMAP test veze</v>
       </c>
       <c r="D384" t="str">
-        <v>INBOX lista i tekst poruke sa rucnim preuzimanjem priloga</v>
+        <v>Read-only INBOX i broj poruka; bez preuzimanja i uvoza</v>
       </c>
       <c r="E384" t="str">
         <v>Visok</v>
@@ -7614,27 +7614,27 @@
         <v>Nije potrebno</v>
       </c>
       <c r="J384" t="str">
-        <v>16/16 i browser QA</v>
+        <v>10/10; TLS i prijava potvrđeni</v>
       </c>
       <c r="K384" t="str">
-        <v>IMAP veza</v>
+        <v>Mail nalog u bazi</v>
       </c>
       <c r="L384" t="str">
-        <v>Read-only i tenant scope; bez uvoza izvoda</v>
+        <v>Admin agencije; sifrovana lozinka AES-256-GCM; MAIL_ENCRYPTION_KEY u env</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="str">
-        <v>M7-IMAP-03</v>
+        <v>M7-IMAP-02</v>
       </c>
       <c r="B385" t="str">
         <v>Modul 7</v>
       </c>
       <c r="C385" t="str">
-        <v>Mail pravila po firmi</v>
+        <v>Pregled mailova</v>
       </c>
       <c r="D385" t="str">
-        <v>Folder i podfolderi uz filtrirani INBOX; opciona AND polja i OR pravila</v>
+        <v>INBOX lista i tekst poruke sa rucnim preuzimanjem priloga</v>
       </c>
       <c r="E385" t="str">
         <v>Visok</v>
@@ -7649,30 +7649,30 @@
         <v>DA</v>
       </c>
       <c r="I385" t="str">
-        <v>DA</v>
+        <v>Nije potrebno</v>
       </c>
       <c r="J385" t="str">
-        <v>22/22; live i rollback purge</v>
+        <v>16/16 i browser QA</v>
       </c>
       <c r="K385" t="str">
-        <v>IMAP pregled</v>
+        <v>IMAP veza</v>
       </c>
       <c r="L385" t="str">
-        <v>Bez automatskog uvoza</v>
+        <v>Read-only i tenant scope; bez uvoza izvoda</v>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="str">
-        <v>M7-IMAP-04</v>
+        <v>M7-IMAP-03</v>
       </c>
       <c r="B386" t="str">
         <v>Modul 7</v>
       </c>
       <c r="C386" t="str">
-        <v>Uvoz izvoda iz maila na klik</v>
+        <v>Mail pravila po firmi</v>
       </c>
       <c r="D386" t="str">
-        <v>Isti parser i obrada kao ručni uvoz; račun i godina; hash i identitet; statusi priloga</v>
+        <v>Folder i podfolderi uz filtrirani INBOX; opciona AND polja i OR pravila</v>
       </c>
       <c r="E386" t="str">
         <v>Visok</v>
@@ -7690,33 +7690,33 @@
         <v>DA</v>
       </c>
       <c r="J386" t="str">
-        <v>27 testova i transakcijski rollback test</v>
+        <v>22/22; live i rollback purge</v>
       </c>
       <c r="K386" t="str">
-        <v>IMAP pregled i parseri</v>
+        <v>IMAP pregled</v>
       </c>
       <c r="L386" t="str">
-        <v>Završeni mailovi se preskaču prije download-a; dnevna obrada dodata u M7-IMAP-05</v>
+        <v>Bez automatskog uvoza</v>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="str">
-        <v>M7-IMAP-05</v>
+        <v>M7-IMAP-04</v>
       </c>
       <c r="B387" t="str">
         <v>Modul 7</v>
       </c>
       <c r="C387" t="str">
-        <v>Dnevna automatska obrada mail izvoda</v>
+        <v>Uvoz izvoda iz maila na klik</v>
       </c>
       <c r="D387" t="str">
-        <v>10:00 Europe/Podgorica samo aktivne mail firme; uvoz i knjiženje READY mail izvoda</v>
+        <v>Isti parser i obrada kao ručni uvoz; račun i godina; hash i identitet; statusi priloga</v>
       </c>
       <c r="E387" t="str">
         <v>Visok</v>
       </c>
       <c r="F387" t="str">
-        <v>Implementirano; čeka deploy</v>
+        <v>Završeno</v>
       </c>
       <c r="G387" t="str">
         <v>DA</v>
@@ -7725,71 +7725,71 @@
         <v>DA</v>
       </c>
       <c r="I387" t="str">
-        <v>Postojeći audit</v>
+        <v>DA</v>
       </c>
       <c r="J387" t="str">
-        <v>DB rollback regresija</v>
+        <v>27 testova i transakcijski rollback test</v>
       </c>
       <c r="K387" t="str">
-        <v>IMAP uvoz; pravila knjiženja</v>
+        <v>IMAP pregled i parseri</v>
       </c>
       <c r="L387" t="str">
-        <v>Runtime flag; advisory lock; dnevna evidencija; pregled rezultata</v>
+        <v>Završeni mailovi se preskaču prije download-a; dnevna obrada dodata u M7-IMAP-05</v>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="str">
-        <v>CLIENT-01</v>
+        <v>M7-IMAP-05</v>
       </c>
       <c r="B388" t="str">
-        <v>Klijentski portal</v>
+        <v>Modul 7</v>
       </c>
       <c r="C388" t="str">
-        <v>Read-only knjigovodstveni portal</v>
+        <v>Dnevna automatska obrada mail izvoda</v>
       </c>
       <c r="D388" t="str">
-        <v>Kupci i dobavljači preko podešenih konta; kartice; robni dokumenti i šifarnici; lager i PDV.</v>
+        <v>10:00 Europe/Podgorica samo aktivne mail firme; uvoz i knjiženje READY mail izvoda</v>
       </c>
       <c r="E388" t="str">
         <v>Visok</v>
       </c>
       <c r="F388" t="str">
-        <v>Implementirano</v>
+        <v>Implementirano; čeka deploy</v>
       </c>
       <c r="G388" t="str">
-        <v>Da</v>
+        <v>DA</v>
       </c>
       <c r="H388" t="str">
-        <v>Da</v>
+        <v>DA</v>
       </c>
       <c r="I388" t="str">
-        <v>Nije potrebno</v>
+        <v>Postojeći audit</v>
       </c>
       <c r="J388" t="str">
-        <v>DB rollback; TSC; lint; desktop/mobilni render</v>
+        <v>DB rollback regresija</v>
       </c>
       <c r="K388" t="str">
-        <v>F-006,F-018</v>
+        <v>IMAP uvoz; pravila knjiženja</v>
       </c>
       <c r="L388" t="str">
-        <v>Odvojene liste radnika i klijenata i matrice; dnevnik aktivnosti agencije sa filterima i paginacijom; bez unosa; početna ima top 10 grafikone dugovanja kupaca i dobavljača; interaktivni QA prijavljenog klijenta ostaje otvoren.</v>
+        <v>Runtime flag; advisory lock; dnevna evidencija; pregled rezultata</v>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="str">
-        <v>OFFICE-ST-01</v>
+        <v>CLIENT-01</v>
       </c>
       <c r="B389" t="str">
-        <v>Robno / Prodaja</v>
+        <v>Klijentski portal</v>
       </c>
       <c r="C389" t="str">
-        <v>Potpuni storno izlazne fakture</v>
+        <v>Read-only knjigovodstveni portal</v>
       </c>
       <c r="D389" t="str">
-        <v>Fiskalni korektivni OFFICE dokument sa vezom na original; povrat robe, korektivni nalog, KIF i štampa.</v>
+        <v>Kupci i dobavljači preko podešenih konta; kartice; robni dokumenti i šifarnici; lager i PDV.</v>
       </c>
       <c r="E389" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F389" t="str">
         <v>Implementirano</v>
@@ -7804,27 +7804,27 @@
         <v>Nije potrebno</v>
       </c>
       <c r="J389" t="str">
-        <v>DB rollback + simulirani Fiscal API</v>
+        <v>DB rollback; TSC; lint; desktop/mobilni render</v>
       </c>
       <c r="K389" t="str">
-        <v>F-097</v>
+        <v>F-006,F-018</v>
       </c>
       <c r="L389" t="str">
-        <v>Stabilan idempotency ključ; retry provjerava isti dokument; odvojena lokalna obrada; Live Test QA preostaje.</v>
+        <v>Odvojene liste radnika i klijenata i matrice; dnevnik aktivnosti agencije sa filterima i paginacijom; bez unosa; početna ima top 10 grafikone dugovanja kupaca i dobavljača; interaktivni QA prijavljenog klijenta ostaje otvoren.</v>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="str">
-        <v>TEST-CORE-01</v>
+        <v>OFFICE-ST-01</v>
       </c>
       <c r="B390" t="str">
-        <v>Računovodstveno jezgro</v>
+        <v>Robno / Prodaja</v>
       </c>
       <c r="C390" t="str">
-        <v>Regresioni testovi i CI</v>
+        <v>Potpuni storno izlazne fakture</v>
       </c>
       <c r="D390" t="str">
-        <v>Nalozi; KIF/KUF; PDV; izvodi; puni OFFICE lifecycle; prava i konkurentnost</v>
+        <v>Fiskalni korektivni OFFICE dokument sa vezom na original; povrat robe, korektivni nalog, KIF i štampa.</v>
       </c>
       <c r="E390" t="str">
         <v>Vrlo visok</v>
@@ -7842,30 +7842,30 @@
         <v>Nije potrebno</v>
       </c>
       <c r="J390" t="str">
-        <v>Unit + izolovana PostgreSQL baza + TSC + lint</v>
+        <v>DB rollback + simulirani Fiscal API</v>
       </c>
       <c r="K390" t="str">
-        <v>Postojeći moduli</v>
+        <v>F-097</v>
       </c>
       <c r="L390" t="str">
-        <v>GitHub Linux/PG i Windows/XSD; simulirani fiskalni servis; live QA i browser E2E preostaju.</v>
+        <v>Stabilan idempotency ključ; retry provjerava isti dokument; odvojena lokalna obrada; Live Test QA preostaje.</v>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="str">
-        <v>AGENCY-01</v>
+        <v>TEST-CORE-01</v>
       </c>
       <c r="B391" t="str">
-        <v>Podešavanja</v>
+        <v>Računovodstveno jezgro</v>
       </c>
       <c r="C391" t="str">
-        <v>Profil agencije i podaci ugovora</v>
+        <v>Regresioni testovi i CI</v>
       </c>
       <c r="D391" t="str">
-        <v>Identitet; zastupnik; kontakt; banke; sačuvane ugovorne strane</v>
+        <v>Nalozi; KIF/KUF; PDV; izvodi; puni OFFICE lifecycle; prava i konkurentnost</v>
       </c>
       <c r="E391" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F391" t="str">
         <v>Implementirano</v>
@@ -7877,30 +7877,30 @@
         <v>Da</v>
       </c>
       <c r="I391" t="str">
-        <v>Da</v>
+        <v>Nije potrebno</v>
       </c>
       <c r="J391" t="str">
-        <v>DB regresija + TypeScript + lint</v>
+        <v>Unit + izolovana PostgreSQL baza + TSC + lint</v>
       </c>
       <c r="K391" t="str">
-        <v>Ugovori</v>
+        <v>Postojeći moduli</v>
       </c>
       <c r="L391" t="str">
-        <v>Samo admin svoje agencije; snapshot i izričito osvježavanje; lokalna migracija; deploy preostaje.</v>
+        <v>GitHub Linux/PG i Windows/XSD; simulirani fiskalni servis; live QA i browser E2E preostaju.</v>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="str">
-        <v>CONTRACT-01</v>
+        <v>AGENCY-01</v>
       </c>
       <c r="B392" t="str">
-        <v>Firme / Ugovori</v>
+        <v>Podešavanja</v>
       </c>
       <c r="C392" t="str">
-        <v>Predložak računovodstvenog ugovora</v>
+        <v>Profil agencije i podaci ugovora</v>
       </c>
       <c r="D392" t="str">
-        <v>13 članova iz Word-a; mapiranje strana i zastupnika; naknada; datumi; rok; sud</v>
+        <v>Identitet; zastupnik; kontakt; banke; sačuvane ugovorne strane</v>
       </c>
       <c r="E392" t="str">
         <v>Visok</v>
@@ -7918,27 +7918,27 @@
         <v>Da</v>
       </c>
       <c r="J392" t="str">
-        <v>Unit + DB + A4 vizuelna provjera</v>
+        <v>DB regresija + TypeScript + lint</v>
       </c>
       <c r="K392" t="str">
-        <v>AGENCY-01</v>
+        <v>Ugovori</v>
       </c>
       <c r="L392" t="str">
-        <v>Snapshot direktora; dva načina roka plaćanja; migracija lokalno; deploy preostaje.</v>
+        <v>Samo admin svoje agencije; snapshot i izričito osvježavanje; lokalna migracija; deploy preostaje.</v>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="str">
-        <v>WARN-BANK-01</v>
+        <v>CONTRACT-01</v>
       </c>
       <c r="B393" t="str">
-        <v>Izvodi</v>
+        <v>Firme / Ugovori</v>
       </c>
       <c r="C393" t="str">
-        <v>Upozorenja za preskočene izvode</v>
+        <v>Predložak računovodstvenog ugovora</v>
       </c>
       <c r="D393" t="str">
-        <v>Pregled dostupnih firmi po računu i godini; rasponi i nepoznate oznake</v>
+        <v>13 članova iz Word-a; mapiranje strana i zastupnika; naknada; datumi; rok; sud</v>
       </c>
       <c r="E393" t="str">
         <v>Visok</v>
@@ -7953,30 +7953,30 @@
         <v>Da</v>
       </c>
       <c r="I393" t="str">
-        <v>Nije potrebno</v>
+        <v>Da</v>
       </c>
       <c r="J393" t="str">
-        <v>Unit + DB rollback + TypeScript + lint</v>
+        <v>Unit + DB + A4 vizuelna provjera</v>
       </c>
       <c r="K393" t="str">
-        <v>Modul 7</v>
+        <v>AGENCY-01</v>
       </c>
       <c r="L393" t="str">
-        <v>Od 1 do najvećeg broja; svi uvezeni statusi; prava radnika; link sa kontekstom.</v>
+        <v>Snapshot direktora; dva načina roka plaćanja; migracija lokalno; deploy preostaje.</v>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="str">
-        <v>STATS-01</v>
+        <v>WARN-BANK-01</v>
       </c>
       <c r="B394" t="str">
-        <v>Dashboard</v>
+        <v>Izvodi</v>
       </c>
       <c r="C394" t="str">
-        <v>Statistika rada agencije</v>
+        <v>Upozorenja za preskočene izvode</v>
       </c>
       <c r="D394" t="str">
-        <v>Nalozi; KIF/KUF; izvodi; plate i ugovori; zaposleni; grafikoni po mjesecima</v>
+        <v>Pregled dostupnih firmi po računu i godini; rasponi i nepoznate oznake</v>
       </c>
       <c r="E394" t="str">
         <v>Visok</v>
@@ -7994,27 +7994,27 @@
         <v>Nije potrebno</v>
       </c>
       <c r="J394" t="str">
-        <v>DB rollback + TypeScript + lint + prikaz</v>
+        <v>Unit + DB rollback + TypeScript + lint</v>
       </c>
       <c r="K394" t="str">
-        <v>Postojeće evidencije</v>
+        <v>Modul 7</v>
       </c>
       <c r="L394" t="str">
-        <v>Periodični dokumenti; trenutno stanje ljudi; prava po modulu.</v>
+        <v>Od 1 do najvećeg broja; svi uvezeni statusi; prava radnika; link sa kontekstom.</v>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="str">
-        <v>DEADLINES-01</v>
+        <v>STATS-01</v>
       </c>
       <c r="B395" t="str">
         <v>Dashboard</v>
       </c>
       <c r="C395" t="str">
-        <v>Rokovi po firmama</v>
+        <v>Statistika rada agencije</v>
       </c>
       <c r="D395" t="str">
-        <v>Tabovi PDV i plate prethodni mjesec; završni račun prethodna godina; kontrolna lista; raniji zaostaci</v>
+        <v>Nalozi; KIF/KUF; izvodi; plate i ugovori; zaposleni; grafikoni po mjesecima</v>
       </c>
       <c r="E395" t="str">
         <v>Visok</v>
@@ -8029,30 +8029,30 @@
         <v>Da</v>
       </c>
       <c r="I395" t="str">
-        <v>Da</v>
+        <v>Nije potrebno</v>
       </c>
       <c r="J395" t="str">
-        <v>Unit + DB rollback + TypeScript + lint</v>
+        <v>DB rollback + TypeScript + lint + prikaz</v>
       </c>
       <c r="K395" t="str">
         <v>Postojeće evidencije</v>
       </c>
       <c r="L395" t="str">
-        <v>Bez emailova; scope firmi; audit i verzije; nezavisna predaja i kontrolna lista.</v>
+        <v>Periodični dokumenti; trenutno stanje ljudi; prava po modulu.</v>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="str">
-        <v>HR-JOBS-01</v>
+        <v>DEADLINES-01</v>
       </c>
       <c r="B396" t="str">
-        <v>Plate</v>
+        <v>Dashboard</v>
       </c>
       <c r="C396" t="str">
-        <v>Radna mjesta i ugovori o radu</v>
+        <v>Rokovi po firmama</v>
       </c>
       <c r="D396" t="str">
-        <v>Globalni šifarnik i verzije agencije; jedna kartica radnika; rasporedi 8 do 1 sat; snapshot i štampa ugovora</v>
+        <v>Tabovi PDV i plate prethodni mjesec; završni račun prethodna godina; kontrolna lista; raniji zaostaci</v>
       </c>
       <c r="E396" t="str">
         <v>Visok</v>
@@ -8070,27 +8070,27 @@
         <v>Da</v>
       </c>
       <c r="J396" t="str">
-        <v>Unit + 13 DB skripti + TSC + lint + vizuelni pregled</v>
+        <v>Unit + DB rollback + TypeScript + lint</v>
       </c>
       <c r="K396" t="str">
-        <v>Plate; Firme</v>
+        <v>Postojeće evidencije</v>
       </c>
       <c r="L396" t="str">
-        <v>Predložak iz starog sajta; pravna revizija odvojena; aneksi kasnije.</v>
+        <v>Bez emailova; scope firmi; audit i verzije; nezavisna predaja i kontrolna lista.</v>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="str">
-        <v>HR-TERM-01</v>
+        <v>HR-JOBS-01</v>
       </c>
       <c r="B397" t="str">
         <v>Plate</v>
       </c>
       <c r="C397" t="str">
-        <v>Prestanak radnog odnosa</v>
+        <v>Radna mjesta i ugovori o radu</v>
       </c>
       <c r="D397" t="str">
-        <v>Tri vrste otkaza; datumi; snapshot; štampa iz evidencije bivših radnika</v>
+        <v>Globalni šifarnik i verzije agencije; jedna kartica radnika; rasporedi 8 do 1 sat; snapshot i štampa ugovora</v>
       </c>
       <c r="E397" t="str">
         <v>Visok</v>
@@ -8108,27 +8108,27 @@
         <v>Da</v>
       </c>
       <c r="J397" t="str">
-        <v>DB rollback + TSC + lint + vizuelni pregled</v>
+        <v>Unit + 13 DB skripti + TSC + lint + vizuelni pregled</v>
       </c>
       <c r="K397" t="str">
         <v>Plate; Firme</v>
       </c>
       <c r="L397" t="str">
-        <v>Bez elektronske odjave; istorija ostaje nakon reaktivacije.</v>
+        <v>Predložak iz starog sajta; pravna revizija odvojena; aneksi kasnije.</v>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="str">
-        <v>FIN-AGENCY-01</v>
+        <v>HR-TERM-01</v>
       </c>
       <c r="B398" t="str">
-        <v>Završni račun</v>
+        <v>Plate</v>
       </c>
       <c r="C398" t="str">
-        <v>Zajednička šema agencije</v>
+        <v>Prestanak radnog odnosa</v>
       </c>
       <c r="D398" t="str">
-        <v>Povezivanje BU/BS/SA bez izbora firme na postojećim stranicama</v>
+        <v>Tri vrste otkaza; datumi; snapshot; štampa iz evidencije bivših radnika</v>
       </c>
       <c r="E398" t="str">
         <v>Visok</v>
@@ -8146,27 +8146,27 @@
         <v>Da</v>
       </c>
       <c r="J398" t="str">
-        <v>DB rollback i TypeScript</v>
+        <v>DB rollback + TSC + lint + vizuelni pregled</v>
       </c>
       <c r="K398" t="str">
-        <v>M-008</v>
+        <v>Plate; Firme</v>
       </c>
       <c r="L398" t="str">
-        <v>Šema važi za sve firme agencije; admin prava; transakcioni audit; postojeća povezivanja prenesena.</v>
+        <v>Bez elektronske odjave; istorija ostaje nakon reaktivacije.</v>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="str">
-        <v>CALC-DELETE-01</v>
+        <v>FIN-AGENCY-01</v>
       </c>
       <c r="B399" t="str">
-        <v>Robno</v>
+        <v>Završni račun</v>
       </c>
       <c r="C399" t="str">
-        <v>Brisanje završene kalkulacije</v>
+        <v>Zajednička šema agencije</v>
       </c>
       <c r="D399" t="str">
-        <v>Poništenje lagera i soft delete zasebnog naloga i KUF računa uz audit</v>
+        <v>Povezivanje BU/BS/SA bez izbora firme na postojećim stranicama</v>
       </c>
       <c r="E399" t="str">
         <v>Visok</v>
@@ -8181,30 +8181,30 @@
         <v>Da</v>
       </c>
       <c r="I399" t="str">
-        <v>Bez migracije</v>
+        <v>Da</v>
       </c>
       <c r="J399" t="str">
-        <v>DB rollback regresija</v>
+        <v>DB rollback i TypeScript</v>
       </c>
       <c r="K399" t="str">
-        <v>Robno; KUF; Nalozi</v>
+        <v>M-008</v>
       </c>
       <c r="L399" t="str">
-        <v>Prava i zaključavanja; razlog i potvrda; blokada zavisnog prometa i plaćanja; idempotentnost.</v>
+        <v>Šema važi za sve firme agencije; admin prava; transakcioni audit; postojeća povezivanja prenesena.</v>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="str">
-        <v>PAYROLL-TEST-01</v>
+        <v>CALC-DELETE-01</v>
       </c>
       <c r="B400" t="str">
-        <v>Plate</v>
+        <v>Robno</v>
       </c>
       <c r="C400" t="str">
-        <v>Regresioni testovi obračuna i knjiženja</v>
+        <v>Brisanje završene kalkulacije</v>
       </c>
       <c r="D400" t="str">
-        <v>Bruto/neto; sati; osnovice; dokumenti; prava; konkurentnost; audit rollback</v>
+        <v>Poništenje lagera i soft delete zasebnog naloga i KUF računa uz audit</v>
       </c>
       <c r="E400" t="str">
         <v>Visok</v>
@@ -8222,30 +8222,30 @@
         <v>Bez migracije</v>
       </c>
       <c r="J400" t="str">
-        <v>Unit i izolovana DB regresija</v>
+        <v>DB rollback regresija</v>
       </c>
       <c r="K400" t="str">
-        <v>Plate</v>
+        <v>Robno; KUF; Nalozi</v>
       </c>
       <c r="L400" t="str">
-        <v>Zbirni porez i neto dodatak testirani; stale obračun blokiran; stvarni portal nije testiran.</v>
+        <v>Prava i zaključavanja; razlog i potvrda; blokada zavisnog prometa i plaćanja; idempotentnost.</v>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="str">
-        <v>PDV-LOCK-01</v>
+        <v>PAYROLL-TEST-01</v>
       </c>
       <c r="B401" t="str">
-        <v>PDV</v>
+        <v>Plate</v>
       </c>
       <c r="C401" t="str">
-        <v>Zaključavanje i kontrolisano otključavanje</v>
+        <v>Regresioni testovi obračuna i knjiženja</v>
       </c>
       <c r="D401" t="str">
-        <v>Zaštita KIF/KUF i PDV naloga; arhivske verzije; admin razlog i audit; nezavisna predaja u Rokovima</v>
+        <v>Bruto/neto; sati; osnovice; dokumenti; prava; konkurentnost; audit rollback</v>
       </c>
       <c r="E401" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F401" t="str">
         <v>Implementirano</v>
@@ -8257,33 +8257,33 @@
         <v>Da</v>
       </c>
       <c r="I401" t="str">
-        <v>Da</v>
+        <v>Bez migracije</v>
       </c>
       <c r="J401" t="str">
-        <v>DB lifecycle + concurrency; TSC; lint</v>
+        <v>Unit i izolovana DB regresija</v>
       </c>
       <c r="K401" t="str">
-        <v>F-074</v>
+        <v>Plate</v>
       </c>
       <c r="L401" t="str">
-        <v>Tri migracije; purge usklađen. Plaćanja i nepovezani nalozi dozvoljeni. Ručni portal/browser QA ostaje. Kontrole prikazuju i razlike uz nulti KIF/KUF; tabela sa zelenim/crvenim statusom po kontu.</v>
+        <v>Zbirni porez i neto dodatak testirani; stale obračun blokiran; stvarni portal nije testiran.</v>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="str">
-        <v>INVOICE-RATES-01</v>
+        <v>PDV-LOCK-01</v>
       </c>
       <c r="B402" t="str">
-        <v>Robno</v>
+        <v>PDV</v>
       </c>
       <c r="C402" t="str">
-        <v>Dinamička šema prihoda i izlaznog PDV-a</v>
+        <v>Zaključavanje i kontrolisano otključavanje</v>
       </c>
       <c r="D402" t="str">
-        <v>Dodavanje redova sa stopom i kontom; OFFICE i POS virman</v>
+        <v>Zaštita KIF/KUF i PDV naloga; arhivske verzije; admin razlog i audit; nezavisna predaja u Rokovima</v>
       </c>
       <c r="E402" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F402" t="str">
         <v>Implementirano</v>
@@ -8298,27 +8298,27 @@
         <v>Da</v>
       </c>
       <c r="J402" t="str">
-        <v>Unit i DB lifecycle; TSC; lint</v>
+        <v>DB lifecycle + concurrency; TSC; lint</v>
       </c>
       <c r="K402" t="str">
-        <v>Izlazne fakture</v>
+        <v>F-074</v>
       </c>
       <c r="L402" t="str">
-        <v>Migracija uklanja stari unique indeks; stari nalozi se ne mijenjaju.</v>
+        <v>Tri migracije; purge usklađen. Plaćanja i nepovezani nalozi dozvoljeni. Ručni portal/browser QA ostaje. Kontrole prikazuju i razlike uz nulti KIF/KUF; tabela sa zelenim/crvenim statusom po kontu.</v>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="str">
-        <v>CALC-RATES-01</v>
+        <v>INVOICE-RATES-01</v>
       </c>
       <c r="B403" t="str">
         <v>Robno</v>
       </c>
       <c r="C403" t="str">
-        <v>Dinamička šema kalkulacije</v>
+        <v>Dinamička šema prihoda i izlaznog PDV-a</v>
       </c>
       <c r="D403" t="str">
-        <v>Dodavanje stavki i stopa; ulazni i ukalkulisani PDV po stopama</v>
+        <v>Dodavanje redova sa stopom i kontom; OFFICE i POS virman</v>
       </c>
       <c r="E403" t="str">
         <v>Visok</v>
@@ -8333,30 +8333,30 @@
         <v>Da</v>
       </c>
       <c r="I403" t="str">
-        <v>Postojeća migracija</v>
+        <v>Da</v>
       </c>
       <c r="J403" t="str">
-        <v>Unit i DB rollback; TSC; lint</v>
+        <v>Unit i DB lifecycle; TSC; lint</v>
       </c>
       <c r="K403" t="str">
-        <v>Kalkulacije</v>
+        <v>Izlazne fakture</v>
       </c>
       <c r="L403" t="str">
-        <v>GENERAL fallback bez dupliranja; postojeći nalozi ostaju isti.</v>
+        <v>Migracija uklanja stari unique indeks; stari nalozi se ne mijenjaju.</v>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="str">
-        <v>KUF-DELETE-01</v>
+        <v>CALC-RATES-01</v>
       </c>
       <c r="B404" t="str">
-        <v>KIF/KUF</v>
+        <v>Robno</v>
       </c>
       <c r="C404" t="str">
-        <v>Direktno brisanje računa i knjiženja</v>
+        <v>Dinamička šema kalkulacije</v>
       </c>
       <c r="D404" t="str">
-        <v>Kantica i modal; razlog i potvrda; uklanjanje samo povezanih stavki naloga</v>
+        <v>Dodavanje stavki i stopa; ulazni i ukalkulisani PDV po stopama</v>
       </c>
       <c r="E404" t="str">
         <v>Visok</v>
@@ -8371,30 +8371,30 @@
         <v>Da</v>
       </c>
       <c r="I404" t="str">
-        <v>Da</v>
+        <v>Postojeća migracija</v>
       </c>
       <c r="J404" t="str">
-        <v>Izolovana DB regresija; TSC; lint</v>
+        <v>Unit i DB rollback; TSC; lint</v>
       </c>
       <c r="K404" t="str">
-        <v>KUF; Nalozi; PDV</v>
+        <v>Kalkulacije</v>
       </c>
       <c r="L404" t="str">
-        <v>Veza kuf_entry_id; stare naloge ponovo knjižiti; zaključavanja i audit; purge usklađen.</v>
+        <v>GENERAL fallback bez dupliranja; postojeći nalozi ostaju isti.</v>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="str">
-        <v>MAIL-NOISE-01</v>
+        <v>KUF-DELETE-01</v>
       </c>
       <c r="B405" t="str">
-        <v>Izvodi</v>
+        <v>KIF/KUF</v>
       </c>
       <c r="C405" t="str">
-        <v>Preskakanje logotipa bez evidencije</v>
+        <v>Direktno brisanje računa i knjiženja</v>
       </c>
       <c r="D405" t="str">
-        <v>Mailovi bez podržanih priloga ne pune obradu ni pojedinačni audit</v>
+        <v>Kantica i modal; razlog i potvrda; uklanjanje samo povezanih stavki naloga</v>
       </c>
       <c r="E405" t="str">
         <v>Visok</v>
@@ -8403,36 +8403,36 @@
         <v>Implementirano</v>
       </c>
       <c r="G405" t="str">
-        <v>Nije potrebno</v>
+        <v>Da</v>
       </c>
       <c r="H405" t="str">
         <v>Da</v>
       </c>
       <c r="I405" t="str">
-        <v>Bez migracije</v>
+        <v>Da</v>
       </c>
       <c r="J405" t="str">
-        <v>Izolovana DB regresija</v>
+        <v>Izolovana DB regresija; TSC; lint</v>
       </c>
       <c r="K405" t="str">
-        <v>Mail import</v>
+        <v>KUF; Nalozi; PDV</v>
       </c>
       <c r="L405" t="str">
-        <v>Postojeći zapisi nijesu brisani.</v>
+        <v>Veza kuf_entry_id; stare naloge ponovo knjižiti; zaključavanja i audit; purge usklađen.</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="str">
-        <v>NAL-DNEVNIK</v>
+        <v>MAIL-NOISE-01</v>
       </c>
       <c r="B406" t="str">
-        <v>Nalozi za knjiženje</v>
+        <v>Izvodi</v>
       </c>
       <c r="C406" t="str">
-        <v>Dnevnik knjiženja</v>
+        <v>Preskakanje logotipa bez evidencije</v>
       </c>
       <c r="D406" t="str">
-        <v>Sve proknjižene stavke hronološki po datumu naloga sa kontom, partnerom, dokumentom i iznosima.</v>
+        <v>Mailovi bez podržanih priloga ne pune obradu ni pojedinačni audit</v>
       </c>
       <c r="E406" t="str">
         <v>Visok</v>
@@ -8441,42 +8441,42 @@
         <v>Implementirano</v>
       </c>
       <c r="G406" t="str">
-        <v>Da</v>
+        <v>Nije potrebno</v>
       </c>
       <c r="H406" t="str">
         <v>Da</v>
       </c>
       <c r="I406" t="str">
-        <v>Ne</v>
+        <v>Bez migracije</v>
       </c>
       <c r="J406" t="str">
-        <v>Regresije; TSC; ESLint; browser</v>
+        <v>Izolovana DB regresija</v>
       </c>
       <c r="K406" t="str">
-        <v>M-003</v>
+        <v>Mail import</v>
       </c>
       <c r="L406" t="str">
-        <v>Kombinovani filteri svih kolona i perioda; 100 stavki po stranici; ukupni zbir filtriranog perioda u centima; A4 pejzažna štampa svih stavki; POSTED i tenant scope; view/export prava.</v>
+        <v>Postojeći zapisi nijesu brisani.</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="str">
-        <v>FISCAL-ADVANCE</v>
+        <v>NAL-DNEVNIK</v>
       </c>
       <c r="B407" t="str">
-        <v>Fiskalizacija</v>
+        <v>Nalozi za knjiženje</v>
       </c>
       <c r="C407" t="str">
-        <v>Avansni računi i umanjenje</v>
+        <v>Dnevnik knjiženja</v>
       </c>
       <c r="D407" t="str">
-        <v>Avans, konačni račun sa vezom i negativno umanjenje u Robnom i direktnom portalu.</v>
+        <v>Sve proknjižene stavke hronološki po datumu naloga sa kontom, partnerom, dokumentom i iznosima.</v>
       </c>
       <c r="E407" t="str">
         <v>Visok</v>
       </c>
       <c r="F407" t="str">
-        <v>Implementirano djelimicno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G407" t="str">
         <v>Da</v>
@@ -8485,36 +8485,36 @@
         <v>Da</v>
       </c>
       <c r="I407" t="str">
-        <v>Da</v>
+        <v>Ne</v>
       </c>
       <c r="J407" t="str">
-        <v>TSC; lint; mock; DB rollback; browser</v>
+        <v>Regresije; TSC; ESLint; browser</v>
       </c>
       <c r="K407" t="str">
-        <v>F-037</v>
+        <v>M-003</v>
       </c>
       <c r="L407" t="str">
-        <v>Fiskalni tok implementiran; odvojeni meni i pregled Avansni racuni u Robnom; unos preko dugmeta na pregledu; decimalni format kao obicni racuni; bez lagera za avans; sema avansnih konta po stopama i template povezana sa DRAFT nalozima i KIF SOURCE_DOCUMENT prenosom; umanjenje koristi snimak izvornih konta; odvojeni poreski mjeseci i nastavak bez novog slanja; storno-obnova sajta ostaje naredni; potreban deploy nove Fiscal API verzije.</v>
+        <v>Kombinovani filteri svih kolona i perioda; 100 stavki po stranici; ukupni zbir filtriranog perioda u centima; A4 pejzažna štampa svih stavki; POSTED i tenant scope; view/export prava.</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="str">
-        <v>PAYROLL-COPY</v>
+        <v>FISCAL-ADVANCE</v>
       </c>
       <c r="B408" t="str">
-        <v>Plate i zaposleni</v>
+        <v>Fiskalizacija</v>
       </c>
       <c r="C408" t="str">
-        <v>Grupno kopiranje obračuna u drugi mjesec</v>
+        <v>Avansni računi i umanjenje</v>
       </c>
       <c r="D408" t="str">
-        <v>Izvorni i ciljni mjesec; izbor firmi agencije; kopije odmah CALCULATED nezavisno od aktivne firme.</v>
+        <v>Avans, konačni račun sa vezom i negativno umanjenje u Robnom i direktnom portalu.</v>
       </c>
       <c r="E408" t="str">
         <v>Visok</v>
       </c>
       <c r="F408" t="str">
-        <v>Implementirano</v>
+        <v>Implementirano djelimicno</v>
       </c>
       <c r="G408" t="str">
         <v>Da</v>
@@ -8523,59 +8523,97 @@
         <v>Da</v>
       </c>
       <c r="I408" t="str">
-        <v>Nije potrebno</v>
+        <v>Da</v>
       </c>
       <c r="J408" t="str">
-        <v>Unit; DB rollback; konkurentnost; lifecycle; browser</v>
+        <v>TSC; lint; mock; DB rollback; browser</v>
       </c>
       <c r="K408" t="str">
-        <v>M-006</v>
+        <v>F-037</v>
       </c>
       <c r="L408" t="str">
-        <v>Preuzimaju se ulazi i fond sati; pomjeranje datuma i kraja mjeseca; važeće poreske stope; više izvora; scope/prava/verzije/periodi; bez duplikata; audit i rollback po firmi; knjiženje ostaje posebna akcija.</v>
+        <v>Fiskalni tok implementiran; odvojeni meni i pregled Avansni racuni u Robnom; unos preko dugmeta na pregledu; decimalni format kao obicni racuni; bez lagera za avans; sema avansnih konta po stopama i template povezana sa DRAFT nalozima i KIF SOURCE_DOCUMENT prenosom; umanjenje koristi snimak izvornih konta; odvojeni poreski mjeseci i nastavak bez novog slanja; storno-obnova sajta ostaje naredni; potreban deploy nove Fiscal API verzije.</v>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="str">
-        <v>M7-IMAP-06</v>
+        <v>PAYROLL-COPY</v>
       </c>
       <c r="B409" t="str">
-        <v>Modul 7</v>
+        <v>Plate i zaposleni</v>
       </c>
       <c r="C409" t="str">
-        <v>Mail nalozi agencije u bazi</v>
+        <v>Grupno kopiranje obračuna u drugi mjesec</v>
       </c>
       <c r="D409" t="str">
-        <v>Vise naloga po agenciji i jedan izbor po firmi uz sifrovanu lozinku i prenos stare konfiguracije</v>
+        <v>Izvorni i ciljni mjesec; izbor firmi agencije; kopije odmah CALCULATED nezavisno od aktivne firme.</v>
       </c>
       <c r="E409" t="str">
         <v>Visok</v>
       </c>
       <c r="F409" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G409" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H409" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I409" t="str">
+        <v>Nije potrebno</v>
+      </c>
+      <c r="J409" t="str">
+        <v>Unit; DB rollback; konkurentnost; lifecycle; browser</v>
+      </c>
+      <c r="K409" t="str">
+        <v>M-006</v>
+      </c>
+      <c r="L409" t="str">
+        <v>Preuzimaju se ulazi i fond sati; pomjeranje datuma i kraja mjeseca; važeće poreske stope; više izvora; scope/prava/verzije/periodi; bez duplikata; audit i rollback po firmi; knjiženje ostaje posebna akcija.</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="str">
+        <v>M7-IMAP-06</v>
+      </c>
+      <c r="B410" t="str">
+        <v>Modul 7</v>
+      </c>
+      <c r="C410" t="str">
+        <v>Mail nalozi agencije u bazi</v>
+      </c>
+      <c r="D410" t="str">
+        <v>Vise naloga po agenciji i jedan izbor po firmi uz sifrovanu lozinku i prenos stare konfiguracije</v>
+      </c>
+      <c r="E410" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F410" t="str">
         <v>Implementirano lokalno; ceka deploy</v>
       </c>
-      <c r="G409" t="str">
+      <c r="G410" t="str">
         <v>DA</v>
       </c>
-      <c r="H409" t="str">
+      <c r="H410" t="str">
         <v>DA</v>
       </c>
-      <c r="I409" t="str">
+      <c r="I410" t="str">
         <v>DA</v>
       </c>
-      <c r="J409" t="str">
+      <c r="J410" t="str">
         <v>TSC; lint; unit; DB rollback; live read-only</v>
       </c>
-      <c r="K409" t="str">
+      <c r="K410" t="str">
         <v>IMAP pregled i uvoz</v>
       </c>
-      <c r="L409" t="str">
+      <c r="L410" t="str">
         <v>Kompozitni tenant FK; bez tajni u UI i auditu; verzije; namespace istorije; opt-in automatike; idempotentan CLI; purge zadrzava agencijski nalog. Lokalno prenesene 3 firme i 39 obrada bez promjene pravila. Server nije mijenjan.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA409"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA410"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add bank statement reopening and bulk journal account replacement
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -2931,7 +2931,7 @@
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA410"/>
+  <dimension ref="A1:AA412"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6214,7 +6214,7 @@
         <v>F-063,F-079</v>
       </c>
       <c r="L347" t="str">
-        <v>Osnovna alokacija jedne stavke izvoda na jedan otvoreni KIF/KUF račun je implementirana kroz bank_statement_line_allocations; status plaćanja se osvježava na UNPAID/PARTIALLY_PAID/PAID/OVERPAID. Split jedne uplate na više računa ostaje dorada.</v>
+        <v>Osnovna alokacija jedne stavke izvoda na jedan otvoreni KIF/KUF račun je implementirana kroz bank_statement_line_allocations; status plaćanja se osvježava na UNPAID/PARTIALLY_PAID/PAID/OVERPAID. Split jedne uplate na više računa ostaje dorada. Od 31.10.2026. samo POSTED izvod i POSTED nalog aktiviraju plaćanje; draft čuva izbor bez zatvaranja fakture.</v>
       </c>
     </row>
     <row r="348">
@@ -6371,60 +6371,60 @@
     </row>
     <row r="352">
       <c r="A352" t="str">
-        <v>F-085</v>
+        <v>F-IZV-REOPEN-01</v>
       </c>
       <c r="B352" t="str">
         <v>Izvodi</v>
       </c>
       <c r="C352" t="str">
-        <v>Vraćanje izvoda u nacrt</v>
+        <v>Rasknjižavanje i ispravka izvoda</v>
       </c>
       <c r="D352" t="str">
-        <v>Proknjižen izvod se ne mijenja direktno; vraćanje u nacrt poništava ili označava povezani nalog i efekat zatvaranja faktura.</v>
+        <v>Vrati izvod i nalog u nacrt; ispravi konta i veze; ponovo proknjiži isti nalog i broj.</v>
       </c>
       <c r="E352" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F352" t="str">
-        <v>Specifikacija spremna</v>
+        <v>Implementirano</v>
       </c>
       <c r="G352" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="H352" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="I352" t="str">
-        <v>Da</v>
+        <v>Postojeća šema</v>
       </c>
       <c r="J352" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="K352" t="str">
-        <v>F-084</v>
+        <v>F-080,F-084</v>
       </c>
       <c r="L352" t="str">
-        <v>Provjeriti prava, zaključanu godinu i upisati audit log.</v>
+        <v>31.10.2026. Prava, scope, godina/PDV, zavisnosti, atomski audit, aktivne alokacije samo na POSTED, stale edit i konkurentni zahtjevi; mail automatika ne preuzima rasknjižen izvod.</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="str">
-        <v>F-086</v>
+        <v>F-NAL-ZAMJENA-01</v>
       </c>
       <c r="B353" t="str">
-        <v>Zavrsni racun</v>
+        <v>Nalozi</v>
       </c>
       <c r="C353" t="str">
-        <v>Bilans uspjeha</v>
+        <v>Grupna zamjena konta</v>
       </c>
       <c r="D353" t="str">
-        <v>Bilans uspjeha se racuna iz POSTED naloga po podesivoj semi pozicija, prikazuje tekucu i prethodnu godinu i stampa formalni obrazac.</v>
+        <v>Pregled i potvrda zamjene konta u POSTED nalozima tačne vrste i perioda aktivne firme/godine.</v>
       </c>
       <c r="E353" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F353" t="str">
-        <v>Djelimicno implementirano</v>
+        <v>Implementirano</v>
       </c>
       <c r="G353" t="str">
         <v>Da</v>
@@ -6433,71 +6433,71 @@
         <v>Da</v>
       </c>
       <c r="I353" t="str">
-        <v>Da</v>
+        <v>Postojeća šema</v>
       </c>
       <c r="J353" t="str">
-        <v>Djelimicno</v>
+        <v>Da</v>
       </c>
       <c r="K353" t="str">
-        <v>M-003,M-008,F-038</v>
+        <v>F-IZV-REOPEN-01</v>
       </c>
       <c r="L353" t="str">
-        <v>Sistemska sema je seedovana u finansijski_izvjestaj_sabloni/pozicije; firma moze izmijeniti konta, izuzetke i formule kroz podesavanja. Trajne rucne korekcije po AOP/koloni postoje; arhiva ostaje za doradu.</v>
+        <v>31.10.2026. Isti nalozi/iznosi/partneri; izvorna konta izvoda usklađena; prava/zaključavanja/zavisnosti; potpis i hash pregleda; audit rollback, 263 stavke, concurrency i trajnost kroz repost. Bez nove tabele/ključa.</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="str">
-        <v>F-087</v>
+        <v>F-085</v>
       </c>
       <c r="B354" t="str">
-        <v>Zavrsni racun</v>
+        <v>Izvodi</v>
       </c>
       <c r="C354" t="str">
-        <v>Bilans stanja</v>
+        <v>Vraćanje izvoda u nacrt</v>
       </c>
       <c r="D354" t="str">
-        <v>Bilans stanja se racuna iz POSTED naloga po podesivoj semi pozicija, prikazuje tekucu godinu, prethodnu godinu - krajnje stanje i prethodnu godinu - pocetno stanje.</v>
+        <v>Proknjižen izvod se ne mijenja direktno; vraćanje u nacrt poništava ili označava povezani nalog i efekat zatvaranja faktura.</v>
       </c>
       <c r="E354" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F354" t="str">
-        <v>Djelimicno implementirano</v>
+        <v>Specifikacija spremna</v>
       </c>
       <c r="G354" t="str">
-        <v>Da</v>
+        <v>Ne</v>
       </c>
       <c r="H354" t="str">
-        <v>Da</v>
+        <v>Ne</v>
       </c>
       <c r="I354" t="str">
         <v>Da</v>
       </c>
       <c r="J354" t="str">
-        <v>Djelimicno</v>
+        <v>Ne</v>
       </c>
       <c r="K354" t="str">
-        <v>M-003,M-008,F-038</v>
+        <v>F-084</v>
       </c>
       <c r="L354" t="str">
-        <v>Dodati sistemski sablon, obracun, podesavanja po firmi, trajne rucne korekcije po AOP/koloni i HTML/CSS print obrazac. Arhiva ostaje za doradu.</v>
+        <v>Provjeriti prava, zaključanu godinu i upisati audit log.</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="str">
-        <v>F-088</v>
+        <v>F-086</v>
       </c>
       <c r="B355" t="str">
         <v>Zavrsni racun</v>
       </c>
       <c r="C355" t="str">
-        <v>Statisticki aneks</v>
+        <v>Bilans uspjeha</v>
       </c>
       <c r="D355" t="str">
-        <v>Statisticki aneks se racuna iz POSTED naloga po podesivoj semi pozicija, prikazuje tekucu i prethodnu godinu i stampa formalni obrazac.</v>
+        <v>Bilans uspjeha se racuna iz POSTED naloga po podesivoj semi pozicija, prikazuje tekucu i prethodnu godinu i stampa formalni obrazac.</v>
       </c>
       <c r="E355" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F355" t="str">
         <v>Djelimicno implementirano</v>
@@ -6518,27 +6518,27 @@
         <v>M-003,M-008,F-038</v>
       </c>
       <c r="L355" t="str">
-        <v>Dodat sistemski sablon, obracun, podesavanja po firmi, trajne rucne korekcije po AOP/koloni i HTML/CSS print obrazac.</v>
+        <v>Sistemska sema je seedovana u finansijski_izvjestaj_sabloni/pozicije; firma moze izmijeniti konta, izuzetke i formule kroz podesavanja. Trajne rucne korekcije po AOP/koloni postoje; arhiva ostaje za doradu.</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="str">
-        <v>F-089</v>
+        <v>F-087</v>
       </c>
       <c r="B356" t="str">
-        <v>Plate i zaposleni</v>
+        <v>Zavrsni racun</v>
       </c>
       <c r="C356" t="str">
-        <v>Šifarnik opština i prireza</v>
+        <v>Bilans stanja</v>
       </c>
       <c r="D356" t="str">
-        <v>Globalni šifarnik povezuje opštinu sa DJP šifrom, stopom prireza, šifrom plaćanja i raspoloživim žiro računom za prirez; iste podatke koriste obračun plata i M-4.</v>
+        <v>Bilans stanja se racuna iz POSTED naloga po podesivoj semi pozicija, prikazuje tekucu godinu, prethodnu godinu - krajnje stanje i prethodnu godinu - pocetno stanje.</v>
       </c>
       <c r="E356" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F356" t="str">
-        <v>Implementirano</v>
+        <v>Djelimicno implementirano</v>
       </c>
       <c r="G356" t="str">
         <v>Da</v>
@@ -6550,33 +6550,33 @@
         <v>Da</v>
       </c>
       <c r="J356" t="str">
-        <v>Da</v>
+        <v>Djelimicno</v>
       </c>
       <c r="K356" t="str">
-        <v>M-006</v>
+        <v>M-003,M-008,F-038</v>
       </c>
       <c r="L356" t="str">
-        <v>Unesena je 21 opština iz 001LP.mdb/B_Opstine. Prazni žiro računi iz izvora ostavljeni su prazni do pouzdanijeg zvaničnog izvora.</v>
+        <v>Dodati sistemski sablon, obracun, podesavanja po firmi, trajne rucne korekcije po AOP/koloni i HTML/CSS print obrazac. Arhiva ostaje za doradu.</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="str">
-        <v>F-090</v>
+        <v>F-088</v>
       </c>
       <c r="B357" t="str">
-        <v>Plate i zaposleni</v>
+        <v>Zavrsni racun</v>
       </c>
       <c r="C357" t="str">
-        <v>Obračunske podšifre i koeficijenti</v>
+        <v>Statisticki aneks</v>
       </c>
       <c r="D357" t="str">
-        <v>Šifra primanja može imati roditeljsku IOPPD osnovu, koeficijent iznosa ili staža, posebni procenat poreske osnovice i oznaku fonda sati.</v>
+        <v>Statisticki aneks se racuna iz POSTED naloga po podesivoj semi pozicija, prikazuje tekucu i prethodnu godinu i stampa formalni obrazac.</v>
       </c>
       <c r="E357" t="str">
         <v>Visok</v>
       </c>
       <c r="F357" t="str">
-        <v>Implementirano</v>
+        <v>Djelimicno implementirano</v>
       </c>
       <c r="G357" t="str">
         <v>Da</v>
@@ -6588,30 +6588,30 @@
         <v>Da</v>
       </c>
       <c r="J357" t="str">
-        <v>Da</v>
+        <v>Djelimicno</v>
       </c>
       <c r="K357" t="str">
-        <v>M-006</v>
+        <v>M-003,M-008,F-038</v>
       </c>
       <c r="L357" t="str">
-        <v>Dodato je 25 podšifara iz 001LP.mdb/A_SifR. Koeficijenti tipa IZNOS primjenjuju se u obračunu; STAZ je informativan za uvećano trajanje i ne množi zaradu. Važeće stope ostaju u novim vremenskim šifarnicima.</v>
+        <v>Dodat sistemski sablon, obracun, podesavanja po firmi, trajne rucne korekcije po AOP/koloni i HTML/CSS print obrazac.</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="str">
-        <v>F-091</v>
+        <v>F-089</v>
       </c>
       <c r="B358" t="str">
-        <v>Firme i kontni plan</v>
+        <v>Plate i zaposleni</v>
       </c>
       <c r="C358" t="str">
-        <v>Trajno brisanje testne firme</v>
+        <v>Šifarnik opština i prireza</v>
       </c>
       <c r="D358" t="str">
-        <v>Admin agencije može trajno obrisati firmu i sve podatke koji pripadaju samo toj firmi tek nakon unosa potpuno istog punog naziva.</v>
+        <v>Globalni šifarnik povezuje opštinu sa DJP šifrom, stopom prireza, šifrom plaćanja i raspoloživim žiro računom za prirez; iste podatke koriste obračun plata i M-4.</v>
       </c>
       <c r="E358" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F358" t="str">
         <v>Implementirano</v>
@@ -6629,27 +6629,27 @@
         <v>Da</v>
       </c>
       <c r="K358" t="str">
-        <v>M-002</v>
+        <v>M-006</v>
       </c>
       <c r="L358" t="str">
-        <v>Brisanje je jedna backend transakcija sa agencijskim scope-om, audit zapisom i čišćenjem aktivnog konteksta. Obuhvata lokalne fiskalne/POS podatke; podaci poslati u zasebni Fiscal API ili Poresku upravu ostaju. Provjera db:check-company-purge pokriva tabele sa firma_id, uz obaveznu ručnu FK provjeru podređenih tabela pri svakoj promjeni šeme.</v>
+        <v>Unesena je 21 opština iz 001LP.mdb/B_Opstine. Prazni žiro računi iz izvora ostavljeni su prazni do pouzdanijeg zvaničnog izvora.</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="str">
-        <v>F-092</v>
+        <v>F-090</v>
       </c>
       <c r="B359" t="str">
         <v>Plate i zaposleni</v>
       </c>
       <c r="C359" t="str">
-        <v>Podešavanje knjiženja po kategoriji</v>
+        <v>Obračunske podšifre i koeficijenti</v>
       </c>
       <c r="D359" t="str">
-        <v>Firma za aktivnu poslovnu godinu bira vrstu naloga i posebna duguje/potražuje konta za neto, porez, prirez, svaki doprinos i ostale komponente redovnog rada, ugovora o djelu, zakupa i ostalih ugovora.</v>
+        <v>Šifra primanja može imati roditeljsku IOPPD osnovu, koeficijent iznosa ili staža, posebni procenat poreske osnovice i oznaku fonda sati.</v>
       </c>
       <c r="E359" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F359" t="str">
         <v>Implementirano</v>
@@ -6664,27 +6664,27 @@
         <v>Da</v>
       </c>
       <c r="J359" t="str">
-        <v>Djelimično</v>
+        <v>Da</v>
       </c>
       <c r="K359" t="str">
-        <v>M-003,M-006,F-024</v>
+        <v>M-006</v>
       </c>
       <c r="L359" t="str">
-        <v>Početna redovna šema izvedena je iz 001LP.mdb/ZAR_Kontir i ZAR_TipZB i prilagođena važećem kontnom planu. Šemu koristi automatsko knjiženje obračuna.</v>
+        <v>Dodato je 25 podšifara iz 001LP.mdb/A_SifR. Koeficijenti tipa IZNOS primjenjuju se u obračunu; STAZ je informativan za uvećano trajanje i ne množi zaradu. Važeće stope ostaju u novim vremenskim šifarnicima.</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="str">
-        <v>F-093</v>
+        <v>F-091</v>
       </c>
       <c r="B360" t="str">
-        <v>Plate i zaposleni</v>
+        <v>Firme i kontni plan</v>
       </c>
       <c r="C360" t="str">
-        <v>Proknjižavanje obračuna plata</v>
+        <v>Trajno brisanje testne firme</v>
       </c>
       <c r="D360" t="str">
-        <v>Akcija Proknjiži na obrađenom obračunu transakcijski kreira numerisan, izbalansiran i odmah POSTED PAYROLL nalog iz kategorijske D/P šeme i povezuje ga sa obračunom.</v>
+        <v>Admin agencije može trajno obrisati firmu i sve podatke koji pripadaju samo toj firmi tek nakon unosa potpuno istog punog naziva.</v>
       </c>
       <c r="E360" t="str">
         <v>Vrlo visok</v>
@@ -6702,27 +6702,27 @@
         <v>Da</v>
       </c>
       <c r="J360" t="str">
-        <v>Djelimično</v>
+        <v>Da</v>
       </c>
       <c r="K360" t="str">
-        <v>M-003,M-006,F-092</v>
+        <v>M-002</v>
       </c>
       <c r="L360" t="str">
-        <v>Provjeravaju se scope, pravo plate/post, zaključana godina, aktivna analitička konta, duple zbirne komponente i balans. Duplo knjiženje je blokirano. Vrati u nacrt atomski vraća nalog u DRAFT i obračun u CALCULATED; Proknjiži je ponovo dostupan uz isti nalog/broj. Backend prava oba modula; godina/PDV i zavisni mjesečni obračuni; audit rollback; realni paralelni zahtjevi i render dugmadi. Direktne izmjene/brisanje payroll naloga su blokirane.</v>
+        <v>Brisanje je jedna backend transakcija sa agencijskim scope-om, audit zapisom i čišćenjem aktivnog konteksta. Obuhvata lokalne fiskalne/POS podatke; podaci poslati u zasebni Fiscal API ili Poresku upravu ostaju. Provjera db:check-company-purge pokriva tabele sa firma_id, uz obaveznu ručnu FK provjeru podređenih tabela pri svakoj promjeni šeme.</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="str">
-        <v>F-094</v>
+        <v>F-092</v>
       </c>
       <c r="B361" t="str">
         <v>Plate i zaposleni</v>
       </c>
       <c r="C361" t="str">
-        <v>OPP-ND prijava prireza</v>
+        <v>Podešavanje knjiženja po kategoriji</v>
       </c>
       <c r="D361" t="str">
-        <v>Mjesečna prijava razvrstava porez na lična primanja, samostalnu djelatnost, imovinu/imovinska prava i kapital, primjenjuje važeću stopu prireza opštine firme i generiše službeni A4 obrazac.</v>
+        <v>Firma za aktivnu poslovnu godinu bira vrstu naloga i posebna duguje/potražuje konta za neto, porez, prirez, svaki doprinos i ostale komponente redovnog rada, ugovora o djelu, zakupa i ostalih ugovora.</v>
       </c>
       <c r="E361" t="str">
         <v>Vrlo visok</v>
@@ -6740,27 +6740,27 @@
         <v>Da</v>
       </c>
       <c r="J361" t="str">
-        <v>Da</v>
+        <v>Djelimično</v>
       </c>
       <c r="K361" t="str">
-        <v>M-006,F-089</v>
+        <v>M-003,M-006,F-024</v>
       </c>
       <c r="L361" t="str">
-        <v>Redovan rad ide u lična primanja, ugovor o djelu i ostali ugovori u samostalnu djelatnost, a zakup u imovinu. Kapital ostaje prazan dok ne postoji odgovarajuća vrsta obračuna. Vizuelni render provjeren je prema zvaničnom PDF-u.</v>
+        <v>Početna redovna šema izvedena je iz 001LP.mdb/ZAR_Kontir i ZAR_TipZB i prilagođena važećem kontnom planu. Šemu koristi automatsko knjiženje obračuna.</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="str">
-        <v>F-095</v>
+        <v>F-093</v>
       </c>
       <c r="B362" t="str">
-        <v>Računi / KIF-KUF</v>
+        <v>Plate i zaposleni</v>
       </c>
       <c r="C362" t="str">
-        <v>Unos i knjiženje pazara</v>
+        <v>Proknjižavanje obračuna plata</v>
       </c>
       <c r="D362" t="str">
-        <v>KIF prihvata dnevni ili mjesečni zbirni pazar sa PDV razradom i načinima naplate; pazar ulazi u PDV i knjiži se kroz posebna konta naplate.</v>
+        <v>Akcija Proknjiži na obrađenom obračunu transakcijski kreira numerisan, izbalansiran i odmah POSTED PAYROLL nalog iz kategorijske D/P šeme i povezuje ga sa obračunom.</v>
       </c>
       <c r="E362" t="str">
         <v>Vrlo visok</v>
@@ -6781,24 +6781,24 @@
         <v>Djelimično</v>
       </c>
       <c r="K362" t="str">
-        <v>M-010,F-062,F-068</v>
+        <v>M-003,M-006,F-092</v>
       </c>
       <c r="L362" t="str">
-        <v>Podržani su gotovina, kartice, virman i ostalo; prihodi/PDV koriste KIF šemu, a konta naplate se podešavaju po firmi.</v>
+        <v>Provjeravaju se scope, pravo plate/post, zaključana godina, aktivna analitička konta, duple zbirne komponente i balans. Duplo knjiženje je blokirano. Vrati u nacrt atomski vraća nalog u DRAFT i obračun u CALCULATED; Proknjiži je ponovo dostupan uz isti nalog/broj. Backend prava oba modula; godina/PDV i zavisni mjesečni obračuni; audit rollback; realni paralelni zahtjevi i render dugmadi. Direktne izmjene/brisanje payroll naloga su blokirane.</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="str">
-        <v>F-096</v>
+        <v>F-094</v>
       </c>
       <c r="B363" t="str">
-        <v>POS / Kasa</v>
+        <v>Plate i zaposleni</v>
       </c>
       <c r="C363" t="str">
-        <v>Računovodstveni tok po načinu plaćanja</v>
+        <v>OPP-ND prijava prireza</v>
       </c>
       <c r="D363" t="str">
-        <v>Fiskalizovani POS virman ulazi pojedinačno u KIF i koristi nalog po šemi izlaznih računa; gotovina i kartica ulaze u zbirni dnevni ili mjesečni pazar.</v>
+        <v>Mjesečna prijava razvrstava porez na lična primanja, samostalnu djelatnost, imovinu/imovinska prava i kapital, primjenjuje važeću stopu prireza opštine firme i generiše službeni A4 obrazac.</v>
       </c>
       <c r="E363" t="str">
         <v>Vrlo visok</v>
@@ -6816,27 +6816,27 @@
         <v>Da</v>
       </c>
       <c r="J363" t="str">
-        <v>Djelimično</v>
+        <v>Da</v>
       </c>
       <c r="K363" t="str">
-        <v>M-010,F-062,F-095</v>
+        <v>M-006,F-089</v>
       </c>
       <c r="L363" t="str">
-        <v>Virman tok ostaje pojedinačan. Zbirna obrada gotovine i kartica kreira idempotentan PAZAR u otvorenom KIF-u, čuva članstvo računa i prati status do zajedničkog KIF naloga i njegovog knjiženja. Automatski POS KIF zapis zaštićen je od ručne izmjene i brisanja.</v>
+        <v>Redovan rad ide u lična primanja, ugovor o djelu i ostali ugovori u samostalnu djelatnost, a zakup u imovinu. Kapital ostaje prazan dok ne postoji odgovarajuća vrsta obračuna. Vizuelni render provjeren je prema zvaničnom PDF-u.</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="str">
-        <v>F-097</v>
+        <v>F-095</v>
       </c>
       <c r="B364" t="str">
-        <v>POS / Kasa</v>
+        <v>Računi / KIF-KUF</v>
       </c>
       <c r="C364" t="str">
-        <v>Potpuni storno POS računa</v>
+        <v>Unos i knjiženje pazara</v>
       </c>
       <c r="D364" t="str">
-        <v>Fiskalizovani POS račun može se potpuno stornirati povezanim negativnim korektivnim dokumentom bez brisanja originala.</v>
+        <v>KIF prihvata dnevni ili mjesečni zbirni pazar sa PDV razradom i načinima naplate; pazar ulazi u PDV i knjiži se kroz posebna konta naplate.</v>
       </c>
       <c r="E364" t="str">
         <v>Vrlo visok</v>
@@ -6857,24 +6857,24 @@
         <v>Djelimično</v>
       </c>
       <c r="K364" t="str">
-        <v>M-011,F-096</v>
+        <v>M-010,F-062,F-068</v>
       </c>
       <c r="L364" t="str">
-        <v>Agencijski POS i direktni portal koriste isti tenant-aware servis. Obavezni su razlog i potvrda; uključeni su Fiscal API storno, povrat robe, audit i retry. Agencijski tok zadržava računovodstvenu obradu, a direktni FISCAL_ONLY tok ne kreira KIF ni nalog. Djelimični povrat čeka API podršku.</v>
+        <v>Podržani su gotovina, kartice, virman i ostalo; prihodi/PDV koriste KIF šemu, a konta naplate se podešavaju po firmi.</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="str">
-        <v>F-098</v>
+        <v>F-096</v>
       </c>
       <c r="B365" t="str">
         <v>POS / Kasa</v>
       </c>
       <c r="C365" t="str">
-        <v>POS izvještaji i termalna štampa</v>
+        <v>Računovodstveni tok po načinu plaćanja</v>
       </c>
       <c r="D365" t="str">
-        <v>Promet po periodu i kasi sa neto stornima, plaćanjima, PDV-om i artiklima; fiskalni račun se štampa na 58/80 mm papiru.</v>
+        <v>Fiskalizovani POS virman ulazi pojedinačno u KIF i koristi nalog po šemi izlaznih računa; gotovina i kartica ulaze u zbirni dnevni ili mjesečni pazar.</v>
       </c>
       <c r="E365" t="str">
         <v>Vrlo visok</v>
@@ -6895,24 +6895,24 @@
         <v>Djelimično</v>
       </c>
       <c r="K365" t="str">
-        <v>M-011,F-097</v>
+        <v>M-010,F-062,F-095</v>
       </c>
       <c r="L365" t="str">
-        <v>Browser štampa fiskalnog računa čuva dvojezičnu srpsko-englesku A4 opciju i prikazuje QR, IKOF/JIKR, kupca i vezu storna. Izvještaj ima zasebnu štampu; direktni portal auditira otvaranje A4 i 58/80 mm štampe. Stvarni termalni printer i reprint audit agencijskog POS-a ostaju za ručni QA.</v>
+        <v>Virman tok ostaje pojedinačan. Zbirna obrada gotovine i kartica kreira idempotentan PAZAR u otvorenom KIF-u, čuva članstvo računa i prati status do zajedničkog KIF naloga i njegovog knjiženja. Automatski POS KIF zapis zaštićen je od ručne izmjene i brisanja.</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="str">
-        <v>F-099</v>
+        <v>F-097</v>
       </c>
       <c r="B366" t="str">
         <v>POS / Kasa</v>
       </c>
       <c r="C366" t="str">
-        <v>Smjenski presjek i predaja kase</v>
+        <v>Potpuni storno POS računa</v>
       </c>
       <c r="D366" t="str">
-        <v>Radnik otvara smjenu sa preuzetom gotovinom, a pri predaji zatvara smjenu i čuva presjek prometa do tog trenutka.</v>
+        <v>Fiskalizovani POS račun može se potpuno stornirati povezanim negativnim korektivnim dokumentom bez brisanja originala.</v>
       </c>
       <c r="E366" t="str">
         <v>Vrlo visok</v>
@@ -6933,24 +6933,24 @@
         <v>Djelimično</v>
       </c>
       <c r="K366" t="str">
-        <v>M-011,F-098</v>
+        <v>M-011,F-096</v>
       </c>
       <c r="L366" t="str">
-        <v>Jedna otvorena smjena po kasi; presjek čuva račune, plaćanja, ukupan promet i očekivanu gotovinu. Ne mijenja dnevni ili mjesečni KIF zbir.</v>
+        <v>Agencijski POS i direktni portal koriste isti tenant-aware servis. Obavezni su razlog i potvrda; uključeni su Fiscal API storno, povrat robe, audit i retry. Agencijski tok zadržava računovodstvenu obradu, a direktni FISCAL_ONLY tok ne kreira KIF ni nalog. Djelimični povrat čeka API podršku.</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="str">
-        <v>F-100</v>
+        <v>F-098</v>
       </c>
       <c r="B367" t="str">
-        <v>Portal direktnog fiskalnog klijenta</v>
+        <v>POS / Kasa</v>
       </c>
       <c r="C367" t="str">
-        <v>Siguran portal shell i automatski kontekst</v>
+        <v>POS izvještaji i termalna štampa</v>
       </c>
       <c r="D367" t="str">
-        <v>Direktni korisnik poslije prijave ulazi na /portal, dobija svoju jedinu firmu i važeću poslovnu godinu, ne vidi sistemski tenant i ne može otvoriti /agencija prostor.</v>
+        <v>Promet po periodu i kasi sa neto stornima, plaćanjima, PDV-om i artiklima; fiskalni račun se štampa na 58/80 mm papiru.</v>
       </c>
       <c r="E367" t="str">
         <v>Vrlo visok</v>
@@ -6968,27 +6968,27 @@
         <v>Da</v>
       </c>
       <c r="J367" t="str">
-        <v>Da</v>
+        <v>Djelimično</v>
       </c>
       <c r="K367" t="str">
-        <v>M-001,M-002,M-012</v>
+        <v>M-011,F-097</v>
       </c>
       <c r="L367" t="str">
-        <v>Centralni backend guard razlikuje direktnog korisnika preko sistemskog tenant-a, KorisnikFirma access_type-a i eksplicitnih prava; cookie nije dokaz ovlašćenja.</v>
+        <v>Browser štampa fiskalnog računa čuva dvojezičnu srpsko-englesku A4 opciju i prikazuje QR, IKOF/JIKR, kupca i vezu storna. Izvještaj ima zasebnu štampu; direktni portal auditira otvaranje A4 i 58/80 mm štampe. Stvarni termalni printer i reprint audit agencijskog POS-a ostaju za ručni QA.</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="str">
-        <v>F-101</v>
+        <v>F-099</v>
       </c>
       <c r="B368" t="str">
-        <v>Portal direktnog fiskalnog klijenta</v>
+        <v>POS / Kasa</v>
       </c>
       <c r="C368" t="str">
-        <v>Operativni dashboard</v>
+        <v>Smjenski presjek i predaja kase</v>
       </c>
       <c r="D368" t="str">
-        <v>Početna prikazuje današnji neto fiskalizovani promet, broj računa i storna, prosjek, načine plaćanja, posljednje račune i upozorenja sa correlation ID-em.</v>
+        <v>Radnik otvara smjenu sa preuzetom gotovinom, a pri predaji zatvara smjenu i čuva presjek prometa do tog trenutka.</v>
       </c>
       <c r="E368" t="str">
         <v>Vrlo visok</v>
@@ -7009,30 +7009,30 @@
         <v>Djelimično</v>
       </c>
       <c r="K368" t="str">
-        <v>F-100,F-097,F-098</v>
+        <v>M-011,F-098</v>
       </c>
       <c r="L368" t="str">
-        <v>Metrike koriste Europe/Podgorica, centnu aritmetiku i uključuju original plus negativni korektivni dokument radi ispravnog neto prometa.</v>
+        <v>Jedna otvorena smjena po kasi; presjek čuva račune, plaćanja, ukupan promet i očekivanu gotovinu. Ne mijenja dnevni ili mjesečni KIF zbir.</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="str">
-        <v>F-102</v>
+        <v>F-100</v>
       </c>
       <c r="B369" t="str">
         <v>Portal direktnog fiskalnog klijenta</v>
       </c>
       <c r="C369" t="str">
-        <v>POS i klasične bezgotovinske fakture</v>
+        <v>Siguran portal shell i automatski kontekst</v>
       </c>
       <c r="D369" t="str">
-        <v>Portal omogućava mobile-first POS i dokument-oriented OFFICE fakturu nad istim prodajnim dokumentom i postojećim Fiscal API tokom.</v>
+        <v>Direktni korisnik poslije prijave ulazi na /portal, dobija svoju jedinu firmu i važeću poslovnu godinu, ne vidi sistemski tenant i ne može otvoriti /agencija prostor.</v>
       </c>
       <c r="E369" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F369" t="str">
-        <v>Implementirano djelimično</v>
+        <v>Implementirano</v>
       </c>
       <c r="G369" t="str">
         <v>Da</v>
@@ -7044,27 +7044,27 @@
         <v>Da</v>
       </c>
       <c r="J369" t="str">
-        <v>Djelimično</v>
+        <v>Da</v>
       </c>
       <c r="K369" t="str">
-        <v>F-100,M-004,M-011</v>
+        <v>M-001,M-002,M-012</v>
       </c>
       <c r="L369" t="str">
-        <v>Oba toka koriste idempotency, eksplicitnu Production potvrdu, status recovery i štampu. POS puni storno koristi isti servis kao agencijski POS; direct FISCAL_ONLY uspjeh ne kreira KIF ni nalog. Ostaje ručni end-to-end QA.</v>
+        <v>Centralni backend guard razlikuje direktnog korisnika preko sistemskog tenant-a, KorisnikFirma access_type-a i eksplicitnih prava; cookie nije dokaz ovlašćenja.</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="str">
-        <v>F-103</v>
+        <v>F-101</v>
       </c>
       <c r="B370" t="str">
         <v>Portal direktnog fiskalnog klijenta</v>
       </c>
       <c r="C370" t="str">
-        <v>Fiskalni računi izvještaji šifarnici i podešavanja</v>
+        <v>Operativni dashboard</v>
       </c>
       <c r="D370" t="str">
-        <v>Jedinstveni pregled POS/OFFICE/storno dokumenata, prodajni izvještaji, artikli, cijene, kupci i samo dozvoljena operativna podešavanja.</v>
+        <v>Početna prikazuje današnji neto fiskalizovani promet, broj računa i storna, prosjek, načine plaćanja, posljednje račune i upozorenja sa correlation ID-em.</v>
       </c>
       <c r="E370" t="str">
         <v>Vrlo visok</v>
@@ -7085,30 +7085,30 @@
         <v>Djelimično</v>
       </c>
       <c r="K370" t="str">
-        <v>F-100,F-101,F-102</v>
+        <v>F-100,F-097,F-098</v>
       </c>
       <c r="L370" t="str">
-        <v>Operativna podešavanja obuhvataju kontakt, glavni račun, kasu, magacin, plaćanje, rok, štampu, smjene, lager i Test depozit. Fiskalna administracija ostaje platformskom adminu; produkcijski depozit čeka API rutu.</v>
+        <v>Metrike koriste Europe/Podgorica, centnu aritmetiku i uključuju original plus negativni korektivni dokument radi ispravnog neto prometa.</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="str">
-        <v>F-104</v>
+        <v>F-102</v>
       </c>
       <c r="B371" t="str">
-        <v>Plate i zaposleni</v>
+        <v>Portal direktnog fiskalnog klijenta</v>
       </c>
       <c r="C371" t="str">
-        <v>Pojedinačni period i sati radnika</v>
+        <v>POS i klasične bezgotovinske fakture</v>
       </c>
       <c r="D371" t="str">
-        <v>Obračunska stavka ima datum od/do unutar mjeseca i trajanja zaposlenja; sistem predlaže sate prema radnim danima i fondu, a računovođa može sa auditom ručno promijeniti ili vratiti automatske sate.</v>
+        <v>Portal omogućava mobile-first POS i dokument-oriented OFFICE fakturu nad istim prodajnim dokumentom i postojećim Fiscal API tokom.</v>
       </c>
       <c r="E371" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F371" t="str">
-        <v>Implementirano</v>
+        <v>Implementirano djelimično</v>
       </c>
       <c r="G371" t="str">
         <v>Da</v>
@@ -7120,30 +7120,30 @@
         <v>Da</v>
       </c>
       <c r="J371" t="str">
-        <v>Da</v>
+        <v>Djelimično</v>
       </c>
       <c r="K371" t="str">
-        <v>M-006</v>
+        <v>F-100,M-004,M-011</v>
       </c>
       <c r="L371" t="str">
-        <v>Priprema uključuje i radnike koji počnu ili završe radni odnos tokom mjeseca. Testovi pokrivaju početak 17-og, prestanak prije kraja, nekoliko dana rada i period van mjeseca; kalendar praznika i nestandardnih smjena ostaje dorada.</v>
+        <v>Oba toka koriste idempotency, eksplicitnu Production potvrdu, status recovery i štampu. POS puni storno koristi isti servis kao agencijski POS; direct FISCAL_ONLY uspjeh ne kreira KIF ni nalog. Ostaje ručni end-to-end QA.</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="str">
-        <v>F-105</v>
+        <v>F-103</v>
       </c>
       <c r="B372" t="str">
-        <v>Korisnici, agencije i prava</v>
+        <v>Portal direktnog fiskalnog klijenta</v>
       </c>
       <c r="C372" t="str">
-        <v>Sklopivi agencijski meni</v>
+        <v>Fiskalni računi izvještaji šifarnici i podešavanja</v>
       </c>
       <c r="D372" t="str">
-        <v>Glavni agencijski meni se na desktopu sklapa na ikonice i pamti izbor; na telefonu se otvara kao pristupačan bočni panel preko sadržaja.</v>
+        <v>Jedinstveni pregled POS/OFFICE/storno dokumenata, prodajni izvještaji, artikli, cijene, kupci i samo dozvoljena operativna podešavanja.</v>
       </c>
       <c r="E372" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F372" t="str">
         <v>Implementirano</v>
@@ -7155,33 +7155,33 @@
         <v>Da</v>
       </c>
       <c r="I372" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="J372" t="str">
-        <v>Da</v>
+        <v>Djelimično</v>
       </c>
       <c r="K372" t="str">
-        <v>M-001</v>
+        <v>F-100,F-101,F-102</v>
       </c>
       <c r="L372" t="str">
-        <v>Sadržaj koristi oslobođenu širinu; dostupni su ujednačene SVG ikonice, aktivna stavka, title opisi, aria oznake, Escape i backdrop zatvaranje te reduced-motion stilovi. TypeScript i lint su čisti; browser QA je potvrđen u otvorenom i sklopljenom stanju.</v>
+        <v>Operativna podešavanja obuhvataju kontakt, glavni račun, kasu, magacin, plaćanje, rok, štampu, smjene, lager i Test depozit. Fiskalna administracija ostaje platformskom adminu; produkcijski depozit čeka API rutu.</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="str">
-        <v>F-106</v>
+        <v>F-104</v>
       </c>
       <c r="B373" t="str">
-        <v>Izvještaji i dashboard</v>
+        <v>Plate i zaposleni</v>
       </c>
       <c r="C373" t="str">
-        <v>Operativne stavke početnog dashboarda</v>
+        <v>Pojedinačni period i sati radnika</v>
       </c>
       <c r="D373" t="str">
-        <v>Početna za aktivnu firmu/godinu prikazuje nacrte naloga, kalkulacije koje čekaju KUF i izlazne račune koji čekaju KIF, umjesto audit logova.</v>
+        <v>Obračunska stavka ima datum od/do unutar mjeseca i trajanja zaposlenja; sistem predlaže sate prema radnim danima i fondu, a računovođa može sa auditom ručno promijeniti ili vratiti automatske sate.</v>
       </c>
       <c r="E373" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F373" t="str">
         <v>Implementirano</v>
@@ -7199,27 +7199,27 @@
         <v>Da</v>
       </c>
       <c r="K373" t="str">
-        <v>M-003,M-004,M-009,M-010</v>
+        <v>M-006</v>
       </c>
       <c r="L373" t="str">
-        <v>Brojači i najnovije stavke koriste stvarne statuse DRAFT/WAITING_KUF/WAITING_KIF, tenant scope i prava pregleda; redovi vode direktno na izvorni dokument. Browser QA je potvrđen.</v>
+        <v>Priprema uključuje i radnike koji počnu ili završe radni odnos tokom mjeseca. Testovi pokrivaju početak 17-og, prestanak prije kraja, nekoliko dana rada i period van mjeseca; kalendar praznika i nestandardnih smjena ostaje dorada.</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="str">
-        <v>F-107</v>
+        <v>F-105</v>
       </c>
       <c r="B374" t="str">
-        <v>Robno i izvještaji</v>
+        <v>Korisnici, agencije i prava</v>
       </c>
       <c r="C374" t="str">
-        <v>Lager lista i kartica artikla</v>
+        <v>Sklopivi agencijski meni</v>
       </c>
       <c r="D374" t="str">
-        <v>Lager lista prikazuje stanje i vrijednosti po magacinu/artiklu, a kartica hronološke ulaze, izlaze i saldo za izabrani period.</v>
+        <v>Glavni agencijski meni se na desktopu sklapa na ikonice i pamti izbor; na telefonu se otvara kao pristupačan bočni panel preko sadržaja.</v>
       </c>
       <c r="E374" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F374" t="str">
         <v>Implementirano</v>
@@ -7231,30 +7231,30 @@
         <v>Da</v>
       </c>
       <c r="I374" t="str">
-        <v>Da</v>
+        <v>Ne</v>
       </c>
       <c r="J374" t="str">
         <v>Da</v>
       </c>
       <c r="K374" t="str">
-        <v>M-004,M-009</v>
+        <v>M-001</v>
       </c>
       <c r="L374" t="str">
-        <v>Iste serverske komponente koriste se u Robnom i centralnim Izvještajima. Filteri obuhvataju magacin, grupu, artikal, znak stanja i period; kartica računa početno stanje prije perioda i povezuje izvorne dokumente.</v>
+        <v>Sadržaj koristi oslobođenu širinu; dostupni su ujednačene SVG ikonice, aktivna stavka, title opisi, aria oznake, Escape i backdrop zatvaranje te reduced-motion stilovi. TypeScript i lint su čisti; browser QA je potvrđen u otvorenom i sklopljenom stanju.</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="str">
-        <v>F-108</v>
+        <v>F-106</v>
       </c>
       <c r="B375" t="str">
         <v>Izvještaji i dashboard</v>
       </c>
       <c r="C375" t="str">
-        <v>Centralne kartice konta i partnera, PDV i plate</v>
+        <v>Operativne stavke početnog dashboarda</v>
       </c>
       <c r="D375" t="str">
-        <v>Centralni meni izvještaja otvara postojeće funkcionalne kartice glavne knjige, mjesečni PDV pregled i pregled izvještaja plata bez dupliranja poslovne računice.</v>
+        <v>Početna za aktivnu firmu/godinu prikazuje nacrte naloga, kalkulacije koje čekaju KUF i izlazne račune koji čekaju KIF, umjesto audit logova.</v>
       </c>
       <c r="E375" t="str">
         <v>Visok</v>
@@ -7275,27 +7275,27 @@
         <v>Da</v>
       </c>
       <c r="K375" t="str">
-        <v>M-003,M-006,M-007,M-009</v>
+        <v>M-003,M-004,M-009,M-010</v>
       </c>
       <c r="L375" t="str">
-        <v>Kartica konta ima lijevi pretraživ spisak, izbor samo konta sa POSTED prometom ili svih aktivnih konta i desni detalj sa periodom/partnerom; na telefonu radi kao lista pa detalj. Isti master-detail prikaz koristi i ruta pod Nalozima. Partnerska kartica koristi analitička konta i partnera, PDV postojeće periode/prijave, a plate obračune, M-4, OPP-ND i IOPPD.</v>
+        <v>Brojači i najnovije stavke koriste stvarne statuse DRAFT/WAITING_KUF/WAITING_KIF, tenant scope i prava pregleda; redovi vode direktno na izvorni dokument. Browser QA je potvrđen.</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="str">
-        <v>F-109</v>
+        <v>F-107</v>
       </c>
       <c r="B376" t="str">
-        <v>Nalozi / Izvještaji</v>
+        <v>Robno i izvještaji</v>
       </c>
       <c r="C376" t="str">
-        <v>Ispravna štampa bruto bilansa</v>
+        <v>Lager lista i kartica artikla</v>
       </c>
       <c r="D376" t="str">
-        <v>Bruto bilans se štampa na A4 landscape sa osam stabilnih kolona, neprelomivim iznosima i ponovljenim zaglavljem tabele.</v>
+        <v>Lager lista prikazuje stanje i vrijednosti po magacinu/artiklu, a kartica hronološke ulaze, izlaze i saldo za izabrani period.</v>
       </c>
       <c r="E376" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F376" t="str">
         <v>Implementirano</v>
@@ -7307,30 +7307,30 @@
         <v>Da</v>
       </c>
       <c r="I376" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="J376" t="str">
         <v>Da</v>
       </c>
       <c r="K376" t="str">
-        <v>M-003,F-038</v>
+        <v>M-004,M-009</v>
       </c>
       <c r="L376" t="str">
-        <v>Zasebni stil i colgroup odvajaju bruto bilans od sedmokolonskog Bilansa stanja: konto 8%, naziv 26%, šest iznosa po 11%; redovi se ne cijepaju preko stranice.</v>
+        <v>Iste serverske komponente koriste se u Robnom i centralnim Izvještajima. Filteri obuhvataju magacin, grupu, artikal, znak stanja i period; kartica računa početno stanje prije perioda i povezuje izvorne dokumente.</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="str">
-        <v>F-110</v>
+        <v>F-108</v>
       </c>
       <c r="B377" t="str">
-        <v>Nalozi / Izvještaji</v>
+        <v>Izvještaji i dashboard</v>
       </c>
       <c r="C377" t="str">
-        <v>Štampa kartice konta</v>
+        <v>Centralne kartice konta i partnera, PDV i plate</v>
       </c>
       <c r="D377" t="str">
-        <v>Izabrana kartica konta štampa se sa aktivnim partnerom i periodom, početnim saldom, prometom, tekućim saldom i završnim zbirom.</v>
+        <v>Centralni meni izvještaja otvara postojeće funkcionalne kartice glavne knjige, mjesečni PDV pregled i pregled izvještaja plata bez dupliranja poslovne računice.</v>
       </c>
       <c r="E377" t="str">
         <v>Visok</v>
@@ -7345,33 +7345,33 @@
         <v>Da</v>
       </c>
       <c r="I377" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="J377" t="str">
         <v>Da</v>
       </c>
       <c r="K377" t="str">
-        <v>M-003,F-037,F-108</v>
+        <v>M-003,M-006,M-007,M-009</v>
       </c>
       <c r="L377" t="str">
-        <v>Čista A4 landscape ruta prikazuje samo POSTED stavke aktivne firme i godine, provjerava tenant/account/partner scope i ponavlja zaglavlje tabele preko stranica.</v>
+        <v>Kartica konta ima lijevi pretraživ spisak, izbor samo konta sa POSTED prometom ili svih aktivnih konta i desni detalj sa periodom/partnerom; na telefonu radi kao lista pa detalj. Isti master-detail prikaz koristi i ruta pod Nalozima. Partnerska kartica koristi analitička konta i partnera, PDV postojeće periode/prijave, a plate obračune, M-4, OPP-ND i IOPPD.</v>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="str">
-        <v>F-111</v>
+        <v>F-109</v>
       </c>
       <c r="B378" t="str">
-        <v>Završni račun</v>
+        <v>Nalozi / Izvještaji</v>
       </c>
       <c r="C378" t="str">
-        <v>Kontrole spremnosti završnog računa</v>
+        <v>Ispravna štampa bruto bilansa</v>
       </c>
       <c r="D378" t="str">
-        <v>Jedinstven ekran provjerava glavnu knjigu, pomoćne evidencije, šeme i zaključna knjiženja prije arhiviranja i zaključivanja godine.</v>
+        <v>Bruto bilans se štampa na A4 landscape sa osam stabilnih kolona, neprelomivim iznosima i ponovljenim zaglavljem tabele.</v>
       </c>
       <c r="E378" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F378" t="str">
         <v>Implementirano</v>
@@ -7389,27 +7389,27 @@
         <v>Da</v>
       </c>
       <c r="K378" t="str">
-        <v>M-003,M-005,M-006,M-007,M-008,M-010</v>
+        <v>M-003,F-038</v>
       </c>
       <c r="L378" t="str">
-        <v>Read-only tenant-aware kontrolni centar razdvaja greške/upozorenja/uspjehe i vodi direktno na razrješenje; provjerava POSTED balans, analitiku, nacrte, KIF/KUF, izvode, plate, PDV, šablone, 5990/6990, klase 5/6, korekcije, arhivu i matične podatke. Izvorna PDV konta moraju imati saldo 0,00, klasa 5 dugovni/nulti, a klasa 6 potražni/nulti saldo; sporna konta vode na karticu.</v>
+        <v>Zasebni stil i colgroup odvajaju bruto bilans od sedmokolonskog Bilansa stanja: konto 8%, naziv 26%, šest iznosa po 11%; redovi se ne cijepaju preko stranice.</v>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="str">
-        <v>F-112</v>
+        <v>F-110</v>
       </c>
       <c r="B379" t="str">
         <v>Nalozi / Izvještaji</v>
       </c>
       <c r="C379" t="str">
-        <v>Poslovne jedinice kroz dokumente i knjiženja</v>
+        <v>Štampa kartice konta</v>
       </c>
       <c r="D379" t="str">
-        <v>Organizaciona dimenzija prati magacin, dokument i stavku naloga te omogućava rezultat po jedinicama.</v>
+        <v>Izabrana kartica konta štampa se sa aktivnim partnerom i periodom, početnim saldom, prometom, tekućim saldom i završnim zbirom.</v>
       </c>
       <c r="E379" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F379" t="str">
         <v>Implementirano</v>
@@ -7421,33 +7421,33 @@
         <v>Da</v>
       </c>
       <c r="I379" t="str">
-        <v>Da</v>
+        <v>Ne</v>
       </c>
       <c r="J379" t="str">
-        <v>Djelimično</v>
+        <v>Da</v>
       </c>
       <c r="K379" t="str">
-        <v>F-026,F-029,F-041</v>
+        <v>M-003,F-037,F-108</v>
       </c>
       <c r="L379" t="str">
-        <v>Kalkulacije i izlazni/POS računi nasljeđuju jedinicu magacina; ručni KIF/KUF, pazar, izvod i plata imaju izbor. KIF/KUF knjiženje čuva jedinicu po stavci, izvještaj računa klasu 6 minus klasu 5, a završna kontrola prijavljuje obaveznu jedinicu koja nedostaje. Izbor se automatski skriva kada firma nema aktivnih jedinica.</v>
+        <v>Čista A4 landscape ruta prikazuje samo POSTED stavke aktivne firme i godine, provjerava tenant/account/partner scope i ponavlja zaglavlje tabele preko stranica.</v>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="str">
-        <v>F-113</v>
+        <v>F-111</v>
       </c>
       <c r="B380" t="str">
         <v>Završni račun</v>
       </c>
       <c r="C380" t="str">
-        <v>XML izvoz finansijskih iskaza</v>
+        <v>Kontrole spremnosti završnog računa</v>
       </c>
       <c r="D380" t="str">
-        <v>BS/BU/SA sa korekcijama i uporednim kolonama; ostale sekcije nulte prema potvrđenom obimu.</v>
+        <v>Jedinstven ekran provjerava glavnu knjigu, pomoćne evidencije, šeme i zaključna knjiženja prije arhiviranja i zaključivanja godine.</v>
       </c>
       <c r="E380" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F380" t="str">
         <v>Implementirano</v>
@@ -7465,27 +7465,27 @@
         <v>Da</v>
       </c>
       <c r="K380" t="str">
-        <v>M-008</v>
+        <v>M-003,M-005,M-006,M-007,M-008,M-010</v>
       </c>
       <c r="L380" t="str">
-        <v>Zaglavlje za pregled; view/export scope i audit; XSD test. Portal QA ostaje otvoren.</v>
+        <v>Read-only tenant-aware kontrolni centar razdvaja greške/upozorenja/uspjehe i vodi direktno na razrješenje; provjerava POSTED balans, analitiku, nacrte, KIF/KUF, izvode, plate, PDV, šablone, 5990/6990, klase 5/6, korekcije, arhivu i matične podatke. Izvorna PDV konta moraju imati saldo 0,00, klasa 5 dugovni/nulti, a klasa 6 potražni/nulti saldo; sporna konta vode na karticu.</v>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="str">
-        <v>F-114</v>
+        <v>F-112</v>
       </c>
       <c r="B381" t="str">
-        <v>Korisnici, agencije i prava</v>
+        <v>Nalozi / Izvještaji</v>
       </c>
       <c r="C381" t="str">
-        <v>Centralno slanje emaila i Reply-To agencije</v>
+        <v>Poslovne jedinice kroz dokumente i knjiženja</v>
       </c>
       <c r="D381" t="str">
-        <v>Sistem šalje sa admin@summasummarum.me, dok administrator agencije podešava adresu na koju prima odgovore.</v>
+        <v>Organizaciona dimenzija prati magacin, dokument i stavku naloga te omogućava rezultat po jedinicama.</v>
       </c>
       <c r="E381" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F381" t="str">
         <v>Implementirano</v>
@@ -7503,27 +7503,27 @@
         <v>Djelimično</v>
       </c>
       <c r="K381" t="str">
-        <v>M-001</v>
+        <v>F-026,F-029,F-041</v>
       </c>
       <c r="L381" t="str">
-        <v>Admin-only podešavanje po agenciji, backend validacija, audit i probno slanje. Pozivnice koje kreira admin agencije koriste sačuvani Reply-To; produkcijski SMTP nalog mora biti ovlašćen za centralnu From adresu.</v>
+        <v>Kalkulacije i izlazni/POS računi nasljeđuju jedinicu magacina; ručni KIF/KUF, pazar, izvod i plata imaju izbor. KIF/KUF knjiženje čuva jedinicu po stavci, izvještaj računa klasu 6 minus klasu 5, a završna kontrola prijavljuje obaveznu jedinicu koja nedostaje. Izbor se automatski skriva kada firma nema aktivnih jedinica.</v>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="str">
-        <v>F-115</v>
+        <v>F-113</v>
       </c>
       <c r="B382" t="str">
-        <v>Plate i zaposleni</v>
+        <v>Završni račun</v>
       </c>
       <c r="C382" t="str">
-        <v>Dokumenti obračuna plata</v>
+        <v>XML izvoz finansijskih iskaza</v>
       </c>
       <c r="D382" t="str">
-        <v>Obračun daje pojedinačne i zbirne platne liste, rekapitulaciju i kontrolisane naloge za plaćanje iz istih sačuvanih stavki.</v>
+        <v>BS/BU/SA sa korekcijama i uporednim kolonama; ostale sekcije nulte prema potvrđenom obimu.</v>
       </c>
       <c r="E382" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F382" t="str">
         <v>Implementirano</v>
@@ -7535,30 +7535,30 @@
         <v>Da</v>
       </c>
       <c r="I382" t="str">
-        <v>Da</v>
+        <v>Ne</v>
       </c>
       <c r="J382" t="str">
-        <v>Djelimično</v>
+        <v>Da</v>
       </c>
       <c r="K382" t="str">
-        <v>M-006,F-089</v>
+        <v>M-008</v>
       </c>
       <c r="L382" t="str">
-        <v>A4 HTML/CSS štampa je dostupna uz plate/view i plate/export; obračunati dokumenti nose NACRT. Virmani prate dostavljeni PDF raspored sa tri obrasca po A4 strani i podesivom gornjom/lijevom marginom. Kompaktna priprema bez horizontalnog skrola omogućava lokalnu korekciju svih polja prije štampe, bez izmjene obračuna u bazi. Neto ide po radniku; porez, PIO, nezaposlenost i Fond rada zbirno na 820-30000-74; prirez posebno po opštini, Komora na 520-939100-43 i sindikat na 510-105-16.</v>
+        <v>Zaglavlje za pregled; view/export scope i audit; XSD test. Portal QA ostaje otvoren.</v>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="str">
-        <v>F-116</v>
+        <v>F-114</v>
       </c>
       <c r="B383" t="str">
-        <v>Dashboard</v>
+        <v>Korisnici, agencije i prava</v>
       </c>
       <c r="C383" t="str">
-        <v>Opšti virmani</v>
+        <v>Centralno slanje emaila i Reply-To agencije</v>
       </c>
       <c r="D383" t="str">
-        <v>Ručni platni nalozi nevezani za obračun plata čuvaju se kao nacrti, odštampani zapisi ili šabloni i štampaju po tri na A4.</v>
+        <v>Sistem šalje sa admin@summasummarum.me, dok administrator agencije podešava adresu na koju prima odgovore.</v>
       </c>
       <c r="E383" t="str">
         <v>Visok</v>
@@ -7579,100 +7579,100 @@
         <v>Djelimično</v>
       </c>
       <c r="K383" t="str">
-        <v>M-001,M-002,M-009</v>
+        <v>M-001</v>
       </c>
       <c r="L383" t="str">
-        <v>Aktivna firma predlaže nalogodavca i glavni račun; sva polja su izmjenjiva. Zasebna virmani prava štite pregled/unos/izmjenu/brisanje/izvoz. Modul ne knjiži promet niti mijenja izvode.</v>
+        <v>Admin-only podešavanje po agenciji, backend validacija, audit i probno slanje. Pozivnice koje kreira admin agencije koriste sačuvani Reply-To; produkcijski SMTP nalog mora biti ovlašćen za centralnu From adresu.</v>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="str">
-        <v>M7-IMAP-01</v>
+        <v>F-115</v>
       </c>
       <c r="B384" t="str">
-        <v>Modul 7</v>
+        <v>Plate i zaposleni</v>
       </c>
       <c r="C384" t="str">
-        <v>IMAP test veze</v>
+        <v>Dokumenti obračuna plata</v>
       </c>
       <c r="D384" t="str">
-        <v>Read-only INBOX i broj poruka; bez preuzimanja i uvoza</v>
+        <v>Obračun daje pojedinačne i zbirne platne liste, rekapitulaciju i kontrolisane naloge za plaćanje iz istih sačuvanih stavki.</v>
       </c>
       <c r="E384" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F384" t="str">
-        <v>Završeno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G384" t="str">
-        <v>DA</v>
+        <v>Da</v>
       </c>
       <c r="H384" t="str">
-        <v>DA</v>
+        <v>Da</v>
       </c>
       <c r="I384" t="str">
-        <v>Nije potrebno</v>
+        <v>Da</v>
       </c>
       <c r="J384" t="str">
-        <v>10/10; TLS i prijava potvrđeni</v>
+        <v>Djelimično</v>
       </c>
       <c r="K384" t="str">
-        <v>Mail nalog u bazi</v>
+        <v>M-006,F-089</v>
       </c>
       <c r="L384" t="str">
-        <v>Admin agencije; sifrovana lozinka AES-256-GCM; MAIL_ENCRYPTION_KEY u env</v>
+        <v>A4 HTML/CSS štampa je dostupna uz plate/view i plate/export; obračunati dokumenti nose NACRT. Virmani prate dostavljeni PDF raspored sa tri obrasca po A4 strani i podesivom gornjom/lijevom marginom. Kompaktna priprema bez horizontalnog skrola omogućava lokalnu korekciju svih polja prije štampe, bez izmjene obračuna u bazi. Neto ide po radniku; porez, PIO, nezaposlenost i Fond rada zbirno na 820-30000-74; prirez posebno po opštini, Komora na 520-939100-43 i sindikat na 510-105-16.</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="str">
-        <v>M7-IMAP-02</v>
+        <v>F-116</v>
       </c>
       <c r="B385" t="str">
-        <v>Modul 7</v>
+        <v>Dashboard</v>
       </c>
       <c r="C385" t="str">
-        <v>Pregled mailova</v>
+        <v>Opšti virmani</v>
       </c>
       <c r="D385" t="str">
-        <v>INBOX lista i tekst poruke sa rucnim preuzimanjem priloga</v>
+        <v>Ručni platni nalozi nevezani za obračun plata čuvaju se kao nacrti, odštampani zapisi ili šabloni i štampaju po tri na A4.</v>
       </c>
       <c r="E385" t="str">
         <v>Visok</v>
       </c>
       <c r="F385" t="str">
-        <v>Završeno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G385" t="str">
-        <v>DA</v>
+        <v>Da</v>
       </c>
       <c r="H385" t="str">
-        <v>DA</v>
+        <v>Da</v>
       </c>
       <c r="I385" t="str">
-        <v>Nije potrebno</v>
+        <v>Da</v>
       </c>
       <c r="J385" t="str">
-        <v>16/16 i browser QA</v>
+        <v>Djelimično</v>
       </c>
       <c r="K385" t="str">
-        <v>IMAP veza</v>
+        <v>M-001,M-002,M-009</v>
       </c>
       <c r="L385" t="str">
-        <v>Read-only i tenant scope; bez uvoza izvoda</v>
+        <v>Aktivna firma predlaže nalogodavca i glavni račun; sva polja su izmjenjiva. Zasebna virmani prava štite pregled/unos/izmjenu/brisanje/izvoz. Modul ne knjiži promet niti mijenja izvode.</v>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="str">
-        <v>M7-IMAP-03</v>
+        <v>M7-IMAP-01</v>
       </c>
       <c r="B386" t="str">
         <v>Modul 7</v>
       </c>
       <c r="C386" t="str">
-        <v>Mail pravila po firmi</v>
+        <v>IMAP test veze</v>
       </c>
       <c r="D386" t="str">
-        <v>Folder i podfolderi uz filtrirani INBOX; opciona AND polja i OR pravila</v>
+        <v>Read-only INBOX i broj poruka; bez preuzimanja i uvoza</v>
       </c>
       <c r="E386" t="str">
         <v>Visok</v>
@@ -7687,30 +7687,30 @@
         <v>DA</v>
       </c>
       <c r="I386" t="str">
-        <v>DA</v>
+        <v>Nije potrebno</v>
       </c>
       <c r="J386" t="str">
-        <v>22/22; live i rollback purge</v>
+        <v>10/10; TLS i prijava potvrđeni</v>
       </c>
       <c r="K386" t="str">
-        <v>IMAP pregled</v>
+        <v>Mail nalog u bazi</v>
       </c>
       <c r="L386" t="str">
-        <v>Bez automatskog uvoza</v>
+        <v>Admin agencije; sifrovana lozinka AES-256-GCM; MAIL_ENCRYPTION_KEY u env</v>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="str">
-        <v>M7-IMAP-04</v>
+        <v>M7-IMAP-02</v>
       </c>
       <c r="B387" t="str">
         <v>Modul 7</v>
       </c>
       <c r="C387" t="str">
-        <v>Uvoz izvoda iz maila na klik</v>
+        <v>Pregled mailova</v>
       </c>
       <c r="D387" t="str">
-        <v>Isti parser i obrada kao ručni uvoz; račun i godina; hash i identitet; statusi priloga</v>
+        <v>INBOX lista i tekst poruke sa rucnim preuzimanjem priloga</v>
       </c>
       <c r="E387" t="str">
         <v>Visok</v>
@@ -7725,36 +7725,36 @@
         <v>DA</v>
       </c>
       <c r="I387" t="str">
-        <v>DA</v>
+        <v>Nije potrebno</v>
       </c>
       <c r="J387" t="str">
-        <v>27 testova i transakcijski rollback test</v>
+        <v>16/16 i browser QA</v>
       </c>
       <c r="K387" t="str">
-        <v>IMAP pregled i parseri</v>
+        <v>IMAP veza</v>
       </c>
       <c r="L387" t="str">
-        <v>Završeni mailovi se preskaču prije download-a; dnevna obrada dodata u M7-IMAP-05</v>
+        <v>Read-only i tenant scope; bez uvoza izvoda</v>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="str">
-        <v>M7-IMAP-05</v>
+        <v>M7-IMAP-03</v>
       </c>
       <c r="B388" t="str">
         <v>Modul 7</v>
       </c>
       <c r="C388" t="str">
-        <v>Dnevna automatska obrada mail izvoda</v>
+        <v>Mail pravila po firmi</v>
       </c>
       <c r="D388" t="str">
-        <v>10:00 Europe/Podgorica samo aktivne mail firme; uvoz i knjiženje READY mail izvoda</v>
+        <v>Folder i podfolderi uz filtrirani INBOX; opciona AND polja i OR pravila</v>
       </c>
       <c r="E388" t="str">
         <v>Visok</v>
       </c>
       <c r="F388" t="str">
-        <v>Implementirano; čeka deploy</v>
+        <v>Završeno</v>
       </c>
       <c r="G388" t="str">
         <v>DA</v>
@@ -7763,109 +7763,109 @@
         <v>DA</v>
       </c>
       <c r="I388" t="str">
-        <v>Postojeći audit</v>
+        <v>DA</v>
       </c>
       <c r="J388" t="str">
-        <v>DB rollback regresija</v>
+        <v>22/22; live i rollback purge</v>
       </c>
       <c r="K388" t="str">
-        <v>IMAP uvoz; pravila knjiženja</v>
+        <v>IMAP pregled</v>
       </c>
       <c r="L388" t="str">
-        <v>Runtime flag; advisory lock; dnevna evidencija; pregled rezultata</v>
+        <v>Bez automatskog uvoza</v>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="str">
-        <v>CLIENT-01</v>
+        <v>M7-IMAP-04</v>
       </c>
       <c r="B389" t="str">
-        <v>Klijentski portal</v>
+        <v>Modul 7</v>
       </c>
       <c r="C389" t="str">
-        <v>Read-only knjigovodstveni portal</v>
+        <v>Uvoz izvoda iz maila na klik</v>
       </c>
       <c r="D389" t="str">
-        <v>Kupci i dobavljači preko podešenih konta; kartice; robni dokumenti i šifarnici; lager i PDV.</v>
+        <v>Isti parser i obrada kao ručni uvoz; račun i godina; hash i identitet; statusi priloga</v>
       </c>
       <c r="E389" t="str">
         <v>Visok</v>
       </c>
       <c r="F389" t="str">
-        <v>Implementirano</v>
+        <v>Završeno</v>
       </c>
       <c r="G389" t="str">
-        <v>Da</v>
+        <v>DA</v>
       </c>
       <c r="H389" t="str">
-        <v>Da</v>
+        <v>DA</v>
       </c>
       <c r="I389" t="str">
-        <v>Nije potrebno</v>
+        <v>DA</v>
       </c>
       <c r="J389" t="str">
-        <v>DB rollback; TSC; lint; desktop/mobilni render</v>
+        <v>27 testova i transakcijski rollback test</v>
       </c>
       <c r="K389" t="str">
-        <v>F-006,F-018</v>
+        <v>IMAP pregled i parseri</v>
       </c>
       <c r="L389" t="str">
-        <v>Odvojene liste radnika i klijenata i matrice; dnevnik aktivnosti agencije sa filterima i paginacijom; bez unosa; početna ima top 10 grafikone dugovanja kupaca i dobavljača; interaktivni QA prijavljenog klijenta ostaje otvoren.</v>
+        <v>Završeni mailovi se preskaču prije download-a; dnevna obrada dodata u M7-IMAP-05</v>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="str">
-        <v>OFFICE-ST-01</v>
+        <v>M7-IMAP-05</v>
       </c>
       <c r="B390" t="str">
-        <v>Robno / Prodaja</v>
+        <v>Modul 7</v>
       </c>
       <c r="C390" t="str">
-        <v>Potpuni storno izlazne fakture</v>
+        <v>Dnevna automatska obrada mail izvoda</v>
       </c>
       <c r="D390" t="str">
-        <v>Fiskalni korektivni OFFICE dokument sa vezom na original; povrat robe, korektivni nalog, KIF i štampa.</v>
+        <v>10:00 Europe/Podgorica samo aktivne mail firme; uvoz i knjiženje READY mail izvoda</v>
       </c>
       <c r="E390" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F390" t="str">
-        <v>Implementirano</v>
+        <v>Implementirano; čeka deploy</v>
       </c>
       <c r="G390" t="str">
-        <v>Da</v>
+        <v>DA</v>
       </c>
       <c r="H390" t="str">
-        <v>Da</v>
+        <v>DA</v>
       </c>
       <c r="I390" t="str">
-        <v>Nije potrebno</v>
+        <v>Postojeći audit</v>
       </c>
       <c r="J390" t="str">
-        <v>DB rollback + simulirani Fiscal API</v>
+        <v>DB rollback regresija</v>
       </c>
       <c r="K390" t="str">
-        <v>F-097</v>
+        <v>IMAP uvoz; pravila knjiženja</v>
       </c>
       <c r="L390" t="str">
-        <v>Stabilan idempotency ključ; retry provjerava isti dokument; odvojena lokalna obrada; Live Test QA preostaje.</v>
+        <v>Runtime flag; advisory lock; dnevna evidencija; pregled rezultata</v>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="str">
-        <v>TEST-CORE-01</v>
+        <v>CLIENT-01</v>
       </c>
       <c r="B391" t="str">
-        <v>Računovodstveno jezgro</v>
+        <v>Klijentski portal</v>
       </c>
       <c r="C391" t="str">
-        <v>Regresioni testovi i CI</v>
+        <v>Read-only knjigovodstveni portal</v>
       </c>
       <c r="D391" t="str">
-        <v>Nalozi; KIF/KUF; PDV; izvodi; puni OFFICE lifecycle; prava i konkurentnost</v>
+        <v>Kupci i dobavljači preko podešenih konta; kartice; robni dokumenti i šifarnici; lager i PDV.</v>
       </c>
       <c r="E391" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F391" t="str">
         <v>Implementirano</v>
@@ -7880,30 +7880,30 @@
         <v>Nije potrebno</v>
       </c>
       <c r="J391" t="str">
-        <v>Unit + izolovana PostgreSQL baza + TSC + lint</v>
+        <v>DB rollback; TSC; lint; desktop/mobilni render</v>
       </c>
       <c r="K391" t="str">
-        <v>Postojeći moduli</v>
+        <v>F-006,F-018</v>
       </c>
       <c r="L391" t="str">
-        <v>GitHub Linux/PG i Windows/XSD; simulirani fiskalni servis; live QA i browser E2E preostaju.</v>
+        <v>Odvojene liste radnika i klijenata i matrice; dnevnik aktivnosti agencije sa filterima i paginacijom; bez unosa; početna ima top 10 grafikone dugovanja kupaca i dobavljača; interaktivni QA prijavljenog klijenta ostaje otvoren.</v>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="str">
-        <v>AGENCY-01</v>
+        <v>OFFICE-ST-01</v>
       </c>
       <c r="B392" t="str">
-        <v>Podešavanja</v>
+        <v>Robno / Prodaja</v>
       </c>
       <c r="C392" t="str">
-        <v>Profil agencije i podaci ugovora</v>
+        <v>Potpuni storno izlazne fakture</v>
       </c>
       <c r="D392" t="str">
-        <v>Identitet; zastupnik; kontakt; banke; sačuvane ugovorne strane</v>
+        <v>Fiskalni korektivni OFFICE dokument sa vezom na original; povrat robe, korektivni nalog, KIF i štampa.</v>
       </c>
       <c r="E392" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F392" t="str">
         <v>Implementirano</v>
@@ -7915,33 +7915,33 @@
         <v>Da</v>
       </c>
       <c r="I392" t="str">
-        <v>Da</v>
+        <v>Nije potrebno</v>
       </c>
       <c r="J392" t="str">
-        <v>DB regresija + TypeScript + lint</v>
+        <v>DB rollback + simulirani Fiscal API</v>
       </c>
       <c r="K392" t="str">
-        <v>Ugovori</v>
+        <v>F-097</v>
       </c>
       <c r="L392" t="str">
-        <v>Samo admin svoje agencije; snapshot i izričito osvježavanje; lokalna migracija; deploy preostaje.</v>
+        <v>Stabilan idempotency ključ; retry provjerava isti dokument; odvojena lokalna obrada; Live Test QA preostaje.</v>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="str">
-        <v>CONTRACT-01</v>
+        <v>TEST-CORE-01</v>
       </c>
       <c r="B393" t="str">
-        <v>Firme / Ugovori</v>
+        <v>Računovodstveno jezgro</v>
       </c>
       <c r="C393" t="str">
-        <v>Predložak računovodstvenog ugovora</v>
+        <v>Regresioni testovi i CI</v>
       </c>
       <c r="D393" t="str">
-        <v>13 članova iz Word-a; mapiranje strana i zastupnika; naknada; datumi; rok; sud</v>
+        <v>Nalozi; KIF/KUF; PDV; izvodi; puni OFFICE lifecycle; prava i konkurentnost</v>
       </c>
       <c r="E393" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F393" t="str">
         <v>Implementirano</v>
@@ -7953,30 +7953,30 @@
         <v>Da</v>
       </c>
       <c r="I393" t="str">
-        <v>Da</v>
+        <v>Nije potrebno</v>
       </c>
       <c r="J393" t="str">
-        <v>Unit + DB + A4 vizuelna provjera</v>
+        <v>Unit + izolovana PostgreSQL baza + TSC + lint</v>
       </c>
       <c r="K393" t="str">
-        <v>AGENCY-01</v>
+        <v>Postojeći moduli</v>
       </c>
       <c r="L393" t="str">
-        <v>Snapshot direktora; dva načina roka plaćanja; migracija lokalno; deploy preostaje.</v>
+        <v>GitHub Linux/PG i Windows/XSD; simulirani fiskalni servis; live QA i browser E2E preostaju.</v>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="str">
-        <v>WARN-BANK-01</v>
+        <v>AGENCY-01</v>
       </c>
       <c r="B394" t="str">
-        <v>Izvodi</v>
+        <v>Podešavanja</v>
       </c>
       <c r="C394" t="str">
-        <v>Upozorenja za preskočene izvode</v>
+        <v>Profil agencije i podaci ugovora</v>
       </c>
       <c r="D394" t="str">
-        <v>Pregled dostupnih firmi po računu i godini; rasponi i nepoznate oznake</v>
+        <v>Identitet; zastupnik; kontakt; banke; sačuvane ugovorne strane</v>
       </c>
       <c r="E394" t="str">
         <v>Visok</v>
@@ -7991,30 +7991,30 @@
         <v>Da</v>
       </c>
       <c r="I394" t="str">
-        <v>Nije potrebno</v>
+        <v>Da</v>
       </c>
       <c r="J394" t="str">
-        <v>Unit + DB rollback + TypeScript + lint</v>
+        <v>DB regresija + TypeScript + lint</v>
       </c>
       <c r="K394" t="str">
-        <v>Modul 7</v>
+        <v>Ugovori</v>
       </c>
       <c r="L394" t="str">
-        <v>Od 1 do najvećeg broja; svi uvezeni statusi; prava radnika; link sa kontekstom.</v>
+        <v>Samo admin svoje agencije; snapshot i izričito osvježavanje; lokalna migracija; deploy preostaje.</v>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="str">
-        <v>STATS-01</v>
+        <v>CONTRACT-01</v>
       </c>
       <c r="B395" t="str">
-        <v>Dashboard</v>
+        <v>Firme / Ugovori</v>
       </c>
       <c r="C395" t="str">
-        <v>Statistika rada agencije</v>
+        <v>Predložak računovodstvenog ugovora</v>
       </c>
       <c r="D395" t="str">
-        <v>Nalozi; KIF/KUF; izvodi; plate i ugovori; zaposleni; grafikoni po mjesecima</v>
+        <v>13 članova iz Word-a; mapiranje strana i zastupnika; naknada; datumi; rok; sud</v>
       </c>
       <c r="E395" t="str">
         <v>Visok</v>
@@ -8029,30 +8029,30 @@
         <v>Da</v>
       </c>
       <c r="I395" t="str">
-        <v>Nije potrebno</v>
+        <v>Da</v>
       </c>
       <c r="J395" t="str">
-        <v>DB rollback + TypeScript + lint + prikaz</v>
+        <v>Unit + DB + A4 vizuelna provjera</v>
       </c>
       <c r="K395" t="str">
-        <v>Postojeće evidencije</v>
+        <v>AGENCY-01</v>
       </c>
       <c r="L395" t="str">
-        <v>Periodični dokumenti; trenutno stanje ljudi; prava po modulu.</v>
+        <v>Snapshot direktora; dva načina roka plaćanja; migracija lokalno; deploy preostaje.</v>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="str">
-        <v>DEADLINES-01</v>
+        <v>WARN-BANK-01</v>
       </c>
       <c r="B396" t="str">
-        <v>Dashboard</v>
+        <v>Izvodi</v>
       </c>
       <c r="C396" t="str">
-        <v>Rokovi po firmama</v>
+        <v>Upozorenja za preskočene izvode</v>
       </c>
       <c r="D396" t="str">
-        <v>Tabovi PDV i plate prethodni mjesec; završni račun prethodna godina; kontrolna lista; raniji zaostaci</v>
+        <v>Pregled dostupnih firmi po računu i godini; rasponi i nepoznate oznake</v>
       </c>
       <c r="E396" t="str">
         <v>Visok</v>
@@ -8067,30 +8067,30 @@
         <v>Da</v>
       </c>
       <c r="I396" t="str">
-        <v>Da</v>
+        <v>Nije potrebno</v>
       </c>
       <c r="J396" t="str">
         <v>Unit + DB rollback + TypeScript + lint</v>
       </c>
       <c r="K396" t="str">
-        <v>Postojeće evidencije</v>
+        <v>Modul 7</v>
       </c>
       <c r="L396" t="str">
-        <v>Bez emailova; scope firmi; audit i verzije; nezavisna predaja i kontrolna lista.</v>
+        <v>Od 1 do najvećeg broja; svi uvezeni statusi; prava radnika; link sa kontekstom.</v>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="str">
-        <v>HR-JOBS-01</v>
+        <v>STATS-01</v>
       </c>
       <c r="B397" t="str">
-        <v>Plate</v>
+        <v>Dashboard</v>
       </c>
       <c r="C397" t="str">
-        <v>Radna mjesta i ugovori o radu</v>
+        <v>Statistika rada agencije</v>
       </c>
       <c r="D397" t="str">
-        <v>Globalni šifarnik i verzije agencije; jedna kartica radnika; rasporedi 8 do 1 sat; snapshot i štampa ugovora</v>
+        <v>Nalozi; KIF/KUF; izvodi; plate i ugovori; zaposleni; grafikoni po mjesecima</v>
       </c>
       <c r="E397" t="str">
         <v>Visok</v>
@@ -8105,30 +8105,30 @@
         <v>Da</v>
       </c>
       <c r="I397" t="str">
-        <v>Da</v>
+        <v>Nije potrebno</v>
       </c>
       <c r="J397" t="str">
-        <v>Unit + 13 DB skripti + TSC + lint + vizuelni pregled</v>
+        <v>DB rollback + TypeScript + lint + prikaz</v>
       </c>
       <c r="K397" t="str">
-        <v>Plate; Firme</v>
+        <v>Postojeće evidencije</v>
       </c>
       <c r="L397" t="str">
-        <v>Predložak iz starog sajta; pravna revizija odvojena; aneksi kasnije.</v>
+        <v>Periodični dokumenti; trenutno stanje ljudi; prava po modulu.</v>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="str">
-        <v>HR-TERM-01</v>
+        <v>DEADLINES-01</v>
       </c>
       <c r="B398" t="str">
-        <v>Plate</v>
+        <v>Dashboard</v>
       </c>
       <c r="C398" t="str">
-        <v>Prestanak radnog odnosa</v>
+        <v>Rokovi po firmama</v>
       </c>
       <c r="D398" t="str">
-        <v>Tri vrste otkaza; datumi; snapshot; štampa iz evidencije bivših radnika</v>
+        <v>Tabovi PDV i plate prethodni mjesec; završni račun prethodna godina; kontrolna lista; raniji zaostaci</v>
       </c>
       <c r="E398" t="str">
         <v>Visok</v>
@@ -8146,27 +8146,27 @@
         <v>Da</v>
       </c>
       <c r="J398" t="str">
-        <v>DB rollback + TSC + lint + vizuelni pregled</v>
+        <v>Unit + DB rollback + TypeScript + lint</v>
       </c>
       <c r="K398" t="str">
-        <v>Plate; Firme</v>
+        <v>Postojeće evidencije</v>
       </c>
       <c r="L398" t="str">
-        <v>Bez elektronske odjave; istorija ostaje nakon reaktivacije.</v>
+        <v>Bez emailova; scope firmi; audit i verzije; nezavisna predaja i kontrolna lista.</v>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="str">
-        <v>FIN-AGENCY-01</v>
+        <v>HR-JOBS-01</v>
       </c>
       <c r="B399" t="str">
-        <v>Završni račun</v>
+        <v>Plate</v>
       </c>
       <c r="C399" t="str">
-        <v>Zajednička šema agencije</v>
+        <v>Radna mjesta i ugovori o radu</v>
       </c>
       <c r="D399" t="str">
-        <v>Povezivanje BU/BS/SA bez izbora firme na postojećim stranicama</v>
+        <v>Globalni šifarnik i verzije agencije; jedna kartica radnika; rasporedi 8 do 1 sat; snapshot i štampa ugovora</v>
       </c>
       <c r="E399" t="str">
         <v>Visok</v>
@@ -8184,27 +8184,27 @@
         <v>Da</v>
       </c>
       <c r="J399" t="str">
-        <v>DB rollback i TypeScript</v>
+        <v>Unit + 13 DB skripti + TSC + lint + vizuelni pregled</v>
       </c>
       <c r="K399" t="str">
-        <v>M-008</v>
+        <v>Plate; Firme</v>
       </c>
       <c r="L399" t="str">
-        <v>Šema važi za sve firme agencije; admin prava; transakcioni audit; postojeća povezivanja prenesena.</v>
+        <v>Predložak iz starog sajta; pravna revizija odvojena; aneksi kasnije.</v>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="str">
-        <v>CALC-DELETE-01</v>
+        <v>HR-TERM-01</v>
       </c>
       <c r="B400" t="str">
-        <v>Robno</v>
+        <v>Plate</v>
       </c>
       <c r="C400" t="str">
-        <v>Brisanje završene kalkulacije</v>
+        <v>Prestanak radnog odnosa</v>
       </c>
       <c r="D400" t="str">
-        <v>Poništenje lagera i soft delete zasebnog naloga i KUF računa uz audit</v>
+        <v>Tri vrste otkaza; datumi; snapshot; štampa iz evidencije bivših radnika</v>
       </c>
       <c r="E400" t="str">
         <v>Visok</v>
@@ -8219,30 +8219,30 @@
         <v>Da</v>
       </c>
       <c r="I400" t="str">
-        <v>Bez migracije</v>
+        <v>Da</v>
       </c>
       <c r="J400" t="str">
-        <v>DB rollback regresija</v>
+        <v>DB rollback + TSC + lint + vizuelni pregled</v>
       </c>
       <c r="K400" t="str">
-        <v>Robno; KUF; Nalozi</v>
+        <v>Plate; Firme</v>
       </c>
       <c r="L400" t="str">
-        <v>Prava i zaključavanja; razlog i potvrda; blokada zavisnog prometa i plaćanja; idempotentnost.</v>
+        <v>Bez elektronske odjave; istorija ostaje nakon reaktivacije.</v>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="str">
-        <v>PAYROLL-TEST-01</v>
+        <v>FIN-AGENCY-01</v>
       </c>
       <c r="B401" t="str">
-        <v>Plate</v>
+        <v>Završni račun</v>
       </c>
       <c r="C401" t="str">
-        <v>Regresioni testovi obračuna i knjiženja</v>
+        <v>Zajednička šema agencije</v>
       </c>
       <c r="D401" t="str">
-        <v>Bruto/neto; sati; osnovice; dokumenti; prava; konkurentnost; audit rollback</v>
+        <v>Povezivanje BU/BS/SA bez izbora firme na postojećim stranicama</v>
       </c>
       <c r="E401" t="str">
         <v>Visok</v>
@@ -8257,33 +8257,33 @@
         <v>Da</v>
       </c>
       <c r="I401" t="str">
-        <v>Bez migracije</v>
+        <v>Da</v>
       </c>
       <c r="J401" t="str">
-        <v>Unit i izolovana DB regresija</v>
+        <v>DB rollback i TypeScript</v>
       </c>
       <c r="K401" t="str">
-        <v>Plate</v>
+        <v>M-008</v>
       </c>
       <c r="L401" t="str">
-        <v>Zbirni porez i neto dodatak testirani; stale obračun blokiran; stvarni portal nije testiran.</v>
+        <v>Šema važi za sve firme agencije; admin prava; transakcioni audit; postojeća povezivanja prenesena.</v>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="str">
-        <v>PDV-LOCK-01</v>
+        <v>CALC-DELETE-01</v>
       </c>
       <c r="B402" t="str">
-        <v>PDV</v>
+        <v>Robno</v>
       </c>
       <c r="C402" t="str">
-        <v>Zaključavanje i kontrolisano otključavanje</v>
+        <v>Brisanje završene kalkulacije</v>
       </c>
       <c r="D402" t="str">
-        <v>Zaštita KIF/KUF i PDV naloga; arhivske verzije; admin razlog i audit; nezavisna predaja u Rokovima</v>
+        <v>Poništenje lagera i soft delete zasebnog naloga i KUF računa uz audit</v>
       </c>
       <c r="E402" t="str">
-        <v>Vrlo visok</v>
+        <v>Visok</v>
       </c>
       <c r="F402" t="str">
         <v>Implementirano</v>
@@ -8295,30 +8295,30 @@
         <v>Da</v>
       </c>
       <c r="I402" t="str">
-        <v>Da</v>
+        <v>Bez migracije</v>
       </c>
       <c r="J402" t="str">
-        <v>DB lifecycle + concurrency; TSC; lint</v>
+        <v>DB rollback regresija</v>
       </c>
       <c r="K402" t="str">
-        <v>F-074</v>
+        <v>Robno; KUF; Nalozi</v>
       </c>
       <c r="L402" t="str">
-        <v>Tri migracije; purge usklađen. Plaćanja i nepovezani nalozi dozvoljeni. Ručni portal/browser QA ostaje. Kontrole prikazuju i razlike uz nulti KIF/KUF; tabela sa zelenim/crvenim statusom po kontu.</v>
+        <v>Prava i zaključavanja; razlog i potvrda; blokada zavisnog prometa i plaćanja; idempotentnost.</v>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="str">
-        <v>INVOICE-RATES-01</v>
+        <v>PAYROLL-TEST-01</v>
       </c>
       <c r="B403" t="str">
-        <v>Robno</v>
+        <v>Plate</v>
       </c>
       <c r="C403" t="str">
-        <v>Dinamička šema prihoda i izlaznog PDV-a</v>
+        <v>Regresioni testovi obračuna i knjiženja</v>
       </c>
       <c r="D403" t="str">
-        <v>Dodavanje redova sa stopom i kontom; OFFICE i POS virman</v>
+        <v>Bruto/neto; sati; osnovice; dokumenti; prava; konkurentnost; audit rollback</v>
       </c>
       <c r="E403" t="str">
         <v>Visok</v>
@@ -8333,33 +8333,33 @@
         <v>Da</v>
       </c>
       <c r="I403" t="str">
-        <v>Da</v>
+        <v>Bez migracije</v>
       </c>
       <c r="J403" t="str">
-        <v>Unit i DB lifecycle; TSC; lint</v>
+        <v>Unit i izolovana DB regresija</v>
       </c>
       <c r="K403" t="str">
-        <v>Izlazne fakture</v>
+        <v>Plate</v>
       </c>
       <c r="L403" t="str">
-        <v>Migracija uklanja stari unique indeks; stari nalozi se ne mijenjaju.</v>
+        <v>Zbirni porez i neto dodatak testirani; stale obračun blokiran; stvarni portal nije testiran.</v>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="str">
-        <v>CALC-RATES-01</v>
+        <v>PDV-LOCK-01</v>
       </c>
       <c r="B404" t="str">
-        <v>Robno</v>
+        <v>PDV</v>
       </c>
       <c r="C404" t="str">
-        <v>Dinamička šema kalkulacije</v>
+        <v>Zaključavanje i kontrolisano otključavanje</v>
       </c>
       <c r="D404" t="str">
-        <v>Dodavanje stavki i stopa; ulazni i ukalkulisani PDV po stopama</v>
+        <v>Zaštita KIF/KUF i PDV naloga; arhivske verzije; admin razlog i audit; nezavisna predaja u Rokovima</v>
       </c>
       <c r="E404" t="str">
-        <v>Visok</v>
+        <v>Vrlo visok</v>
       </c>
       <c r="F404" t="str">
         <v>Implementirano</v>
@@ -8371,30 +8371,30 @@
         <v>Da</v>
       </c>
       <c r="I404" t="str">
-        <v>Postojeća migracija</v>
+        <v>Da</v>
       </c>
       <c r="J404" t="str">
-        <v>Unit i DB rollback; TSC; lint</v>
+        <v>DB lifecycle + concurrency; TSC; lint</v>
       </c>
       <c r="K404" t="str">
-        <v>Kalkulacije</v>
+        <v>F-074</v>
       </c>
       <c r="L404" t="str">
-        <v>GENERAL fallback bez dupliranja; postojeći nalozi ostaju isti.</v>
+        <v>Tri migracije; purge usklađen. Plaćanja i nepovezani nalozi dozvoljeni. Ručni portal/browser QA ostaje. Kontrole prikazuju i razlike uz nulti KIF/KUF; tabela sa zelenim/crvenim statusom po kontu.</v>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="str">
-        <v>KUF-DELETE-01</v>
+        <v>INVOICE-RATES-01</v>
       </c>
       <c r="B405" t="str">
-        <v>KIF/KUF</v>
+        <v>Robno</v>
       </c>
       <c r="C405" t="str">
-        <v>Direktno brisanje računa i knjiženja</v>
+        <v>Dinamička šema prihoda i izlaznog PDV-a</v>
       </c>
       <c r="D405" t="str">
-        <v>Kantica i modal; razlog i potvrda; uklanjanje samo povezanih stavki naloga</v>
+        <v>Dodavanje redova sa stopom i kontom; OFFICE i POS virman</v>
       </c>
       <c r="E405" t="str">
         <v>Visok</v>
@@ -8412,27 +8412,27 @@
         <v>Da</v>
       </c>
       <c r="J405" t="str">
-        <v>Izolovana DB regresija; TSC; lint</v>
+        <v>Unit i DB lifecycle; TSC; lint</v>
       </c>
       <c r="K405" t="str">
-        <v>KUF; Nalozi; PDV</v>
+        <v>Izlazne fakture</v>
       </c>
       <c r="L405" t="str">
-        <v>Veza kuf_entry_id; stare naloge ponovo knjižiti; zaključavanja i audit; purge usklađen.</v>
+        <v>Migracija uklanja stari unique indeks; stari nalozi se ne mijenjaju.</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="str">
-        <v>MAIL-NOISE-01</v>
+        <v>CALC-RATES-01</v>
       </c>
       <c r="B406" t="str">
-        <v>Izvodi</v>
+        <v>Robno</v>
       </c>
       <c r="C406" t="str">
-        <v>Preskakanje logotipa bez evidencije</v>
+        <v>Dinamička šema kalkulacije</v>
       </c>
       <c r="D406" t="str">
-        <v>Mailovi bez podržanih priloga ne pune obradu ni pojedinačni audit</v>
+        <v>Dodavanje stavki i stopa; ulazni i ukalkulisani PDV po stopama</v>
       </c>
       <c r="E406" t="str">
         <v>Visok</v>
@@ -8441,36 +8441,36 @@
         <v>Implementirano</v>
       </c>
       <c r="G406" t="str">
-        <v>Nije potrebno</v>
+        <v>Da</v>
       </c>
       <c r="H406" t="str">
         <v>Da</v>
       </c>
       <c r="I406" t="str">
-        <v>Bez migracije</v>
+        <v>Postojeća migracija</v>
       </c>
       <c r="J406" t="str">
-        <v>Izolovana DB regresija</v>
+        <v>Unit i DB rollback; TSC; lint</v>
       </c>
       <c r="K406" t="str">
-        <v>Mail import</v>
+        <v>Kalkulacije</v>
       </c>
       <c r="L406" t="str">
-        <v>Postojeći zapisi nijesu brisani.</v>
+        <v>GENERAL fallback bez dupliranja; postojeći nalozi ostaju isti.</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="str">
-        <v>NAL-DNEVNIK</v>
+        <v>KUF-DELETE-01</v>
       </c>
       <c r="B407" t="str">
-        <v>Nalozi za knjiženje</v>
+        <v>KIF/KUF</v>
       </c>
       <c r="C407" t="str">
-        <v>Dnevnik knjiženja</v>
+        <v>Direktno brisanje računa i knjiženja</v>
       </c>
       <c r="D407" t="str">
-        <v>Sve proknjižene stavke hronološki po datumu naloga sa kontom, partnerom, dokumentom i iznosima.</v>
+        <v>Kantica i modal; razlog i potvrda; uklanjanje samo povezanih stavki naloga</v>
       </c>
       <c r="E407" t="str">
         <v>Visok</v>
@@ -8485,68 +8485,68 @@
         <v>Da</v>
       </c>
       <c r="I407" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="J407" t="str">
-        <v>Regresije; TSC; ESLint; browser</v>
+        <v>Izolovana DB regresija; TSC; lint</v>
       </c>
       <c r="K407" t="str">
-        <v>M-003</v>
+        <v>KUF; Nalozi; PDV</v>
       </c>
       <c r="L407" t="str">
-        <v>Kombinovani filteri svih kolona i perioda; 100 stavki po stranici; ukupni zbir filtriranog perioda u centima; A4 pejzažna štampa svih stavki; POSTED i tenant scope; view/export prava.</v>
+        <v>Veza kuf_entry_id; stare naloge ponovo knjižiti; zaključavanja i audit; purge usklađen.</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="str">
-        <v>FISCAL-ADVANCE</v>
+        <v>MAIL-NOISE-01</v>
       </c>
       <c r="B408" t="str">
-        <v>Fiskalizacija</v>
+        <v>Izvodi</v>
       </c>
       <c r="C408" t="str">
-        <v>Avansni računi i umanjenje</v>
+        <v>Preskakanje logotipa bez evidencije</v>
       </c>
       <c r="D408" t="str">
-        <v>Avans, konačni račun sa vezom i negativno umanjenje u Robnom i direktnom portalu.</v>
+        <v>Mailovi bez podržanih priloga ne pune obradu ni pojedinačni audit</v>
       </c>
       <c r="E408" t="str">
         <v>Visok</v>
       </c>
       <c r="F408" t="str">
-        <v>Implementirano djelimicno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G408" t="str">
-        <v>Da</v>
+        <v>Nije potrebno</v>
       </c>
       <c r="H408" t="str">
         <v>Da</v>
       </c>
       <c r="I408" t="str">
-        <v>Da</v>
+        <v>Bez migracije</v>
       </c>
       <c r="J408" t="str">
-        <v>TSC; lint; mock; DB rollback; browser</v>
+        <v>Izolovana DB regresija</v>
       </c>
       <c r="K408" t="str">
-        <v>F-037</v>
+        <v>Mail import</v>
       </c>
       <c r="L408" t="str">
-        <v>Fiskalni tok implementiran; odvojeni meni i pregled Avansni racuni u Robnom; unos preko dugmeta na pregledu; decimalni format kao obicni racuni; bez lagera za avans; sema avansnih konta po stopama i template povezana sa DRAFT nalozima i KIF SOURCE_DOCUMENT prenosom; umanjenje koristi snimak izvornih konta; odvojeni poreski mjeseci i nastavak bez novog slanja; storno-obnova sajta ostaje naredni; potreban deploy nove Fiscal API verzije.</v>
+        <v>Postojeći zapisi nijesu brisani.</v>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="str">
-        <v>PAYROLL-COPY</v>
+        <v>NAL-DNEVNIK</v>
       </c>
       <c r="B409" t="str">
-        <v>Plate i zaposleni</v>
+        <v>Nalozi za knjiženje</v>
       </c>
       <c r="C409" t="str">
-        <v>Grupno kopiranje obračuna u drugi mjesec</v>
+        <v>Dnevnik knjiženja</v>
       </c>
       <c r="D409" t="str">
-        <v>Izvorni i ciljni mjesec; izbor firmi agencije; kopije odmah CALCULATED nezavisno od aktivne firme.</v>
+        <v>Sve proknjižene stavke hronološki po datumu naloga sa kontom, partnerom, dokumentom i iznosima.</v>
       </c>
       <c r="E409" t="str">
         <v>Visok</v>
@@ -8561,59 +8561,135 @@
         <v>Da</v>
       </c>
       <c r="I409" t="str">
-        <v>Nije potrebno</v>
+        <v>Ne</v>
       </c>
       <c r="J409" t="str">
-        <v>Unit; DB rollback; konkurentnost; lifecycle; browser</v>
+        <v>Regresije; TSC; ESLint; browser</v>
       </c>
       <c r="K409" t="str">
-        <v>M-006</v>
+        <v>M-003</v>
       </c>
       <c r="L409" t="str">
-        <v>Preuzimaju se ulazi i fond sati; pomjeranje datuma i kraja mjeseca; važeće poreske stope; više izvora; scope/prava/verzije/periodi; bez duplikata; audit i rollback po firmi; knjiženje ostaje posebna akcija.</v>
+        <v>Kombinovani filteri svih kolona i perioda; 100 stavki po stranici; ukupni zbir filtriranog perioda u centima; A4 pejzažna štampa svih stavki; POSTED i tenant scope; view/export prava.</v>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="str">
-        <v>M7-IMAP-06</v>
+        <v>FISCAL-ADVANCE</v>
       </c>
       <c r="B410" t="str">
-        <v>Modul 7</v>
+        <v>Fiskalizacija</v>
       </c>
       <c r="C410" t="str">
-        <v>Mail nalozi agencije u bazi</v>
+        <v>Avansni računi i umanjenje</v>
       </c>
       <c r="D410" t="str">
-        <v>Vise naloga po agenciji i jedan izbor po firmi uz sifrovanu lozinku i prenos stare konfiguracije</v>
+        <v>Avans, konačni račun sa vezom i negativno umanjenje u Robnom i direktnom portalu.</v>
       </c>
       <c r="E410" t="str">
         <v>Visok</v>
       </c>
       <c r="F410" t="str">
+        <v>Implementirano djelimicno</v>
+      </c>
+      <c r="G410" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H410" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I410" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J410" t="str">
+        <v>TSC; lint; mock; DB rollback; browser</v>
+      </c>
+      <c r="K410" t="str">
+        <v>F-037</v>
+      </c>
+      <c r="L410" t="str">
+        <v>Fiskalni tok implementiran; odvojeni meni i pregled Avansni racuni u Robnom; unos preko dugmeta na pregledu; decimalni format kao obicni racuni; bez lagera za avans; sema avansnih konta po stopama i template povezana sa DRAFT nalozima i KIF SOURCE_DOCUMENT prenosom; umanjenje koristi snimak izvornih konta; odvojeni poreski mjeseci i nastavak bez novog slanja; storno-obnova sajta ostaje naredni; potreban deploy nove Fiscal API verzije.</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="str">
+        <v>PAYROLL-COPY</v>
+      </c>
+      <c r="B411" t="str">
+        <v>Plate i zaposleni</v>
+      </c>
+      <c r="C411" t="str">
+        <v>Grupno kopiranje obračuna u drugi mjesec</v>
+      </c>
+      <c r="D411" t="str">
+        <v>Izvorni i ciljni mjesec; izbor firmi agencije; kopije odmah CALCULATED nezavisno od aktivne firme.</v>
+      </c>
+      <c r="E411" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F411" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G411" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H411" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I411" t="str">
+        <v>Nije potrebno</v>
+      </c>
+      <c r="J411" t="str">
+        <v>Unit; DB rollback; konkurentnost; lifecycle; browser</v>
+      </c>
+      <c r="K411" t="str">
+        <v>M-006</v>
+      </c>
+      <c r="L411" t="str">
+        <v>Preuzimaju se ulazi i fond sati; pomjeranje datuma i kraja mjeseca; važeće poreske stope; više izvora; scope/prava/verzije/periodi; bez duplikata; audit i rollback po firmi; knjiženje ostaje posebna akcija.</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="str">
+        <v>M7-IMAP-06</v>
+      </c>
+      <c r="B412" t="str">
+        <v>Modul 7</v>
+      </c>
+      <c r="C412" t="str">
+        <v>Mail nalozi agencije u bazi</v>
+      </c>
+      <c r="D412" t="str">
+        <v>Vise naloga po agenciji i jedan izbor po firmi uz sifrovanu lozinku i prenos stare konfiguracije</v>
+      </c>
+      <c r="E412" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F412" t="str">
         <v>Implementirano lokalno; ceka deploy</v>
       </c>
-      <c r="G410" t="str">
+      <c r="G412" t="str">
         <v>DA</v>
       </c>
-      <c r="H410" t="str">
+      <c r="H412" t="str">
         <v>DA</v>
       </c>
-      <c r="I410" t="str">
+      <c r="I412" t="str">
         <v>DA</v>
       </c>
-      <c r="J410" t="str">
+      <c r="J412" t="str">
         <v>TSC; lint; unit; DB rollback; live read-only</v>
       </c>
-      <c r="K410" t="str">
+      <c r="K412" t="str">
         <v>IMAP pregled i uvoz</v>
       </c>
-      <c r="L410" t="str">
+      <c r="L412" t="str">
         <v>Kompozitni tenant FK; bez tajni u UI i auditu; verzije; namespace istorije; opt-in automatike; idempotentan CLI; purge zadrzava agencijski nalog. Lokalno prenesene 3 firme i 39 obrada bez promjene pravila. Server nije mijenjan.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA410"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA412"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>